<commit_message>
data: Actualización automática de reportes (2026-09-15 09:45)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>8 de septiembre de 2026</t>
+          <t>11 de septiembre de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -576,10 +576,10 @@
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>14976.76</v>
+        <v>19029.58</v>
       </c>
       <c r="I6" t="n">
-        <v>14976.76</v>
+        <v>19029.58</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -588,16 +588,16 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>94372.73</v>
+        <v>90474.05</v>
       </c>
       <c r="M6" t="n">
-        <v>94372.73</v>
+        <v>90474.05</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>117440</t>
+          <t>87538</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -607,22 +607,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MONSERRAT VELASCO SANTOS</t>
+          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>6853.85</v>
       </c>
       <c r="H7" t="n">
-        <v>10023.33</v>
+        <v>12121.29</v>
       </c>
       <c r="I7" t="n">
-        <v>10023.33</v>
+        <v>18975.14</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -631,16 +631,16 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>65066.43</v>
+        <v>231506.85</v>
       </c>
       <c r="M7" t="n">
-        <v>65066.43</v>
+        <v>231506.85</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>87538</t>
+          <t>104718</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -650,7 +650,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
+          <t>ROGELIO TORRES ORTIZ</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -662,28 +662,28 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>9142.639999999999</v>
+        <v>18318.58</v>
       </c>
       <c r="I8" t="n">
-        <v>9142.639999999999</v>
+        <v>18318.58</v>
       </c>
       <c r="J8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>9832.18</v>
+        <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>234093.61</v>
+        <v>16324.8</v>
       </c>
       <c r="M8" t="n">
-        <v>243925.79</v>
+        <v>16324.8</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>88234</t>
+          <t>117440</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
+          <t>MONSERRAT VELASCO SANTOS</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
@@ -705,10 +705,10 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>8492.07</v>
+        <v>12218.55</v>
       </c>
       <c r="I9" t="n">
-        <v>8492.07</v>
+        <v>12218.55</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -717,16 +717,16 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>3845.25</v>
+        <v>62871.21</v>
       </c>
       <c r="M9" t="n">
-        <v>3845.25</v>
+        <v>62871.21</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -736,7 +736,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -748,10 +748,10 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>5431.4</v>
+        <v>11245.61</v>
       </c>
       <c r="I10" t="n">
-        <v>5431.4</v>
+        <v>11245.61</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -760,16 +760,16 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>12899.71</v>
+        <v>0</v>
       </c>
       <c r="M10" t="n">
-        <v>12899.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>104718</t>
+          <t>88234</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ROGELIO TORRES ORTIZ</t>
+          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -791,10 +791,10 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>5152.9</v>
+        <v>8492.07</v>
       </c>
       <c r="I11" t="n">
-        <v>5152.9</v>
+        <v>8492.07</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -803,10 +803,10 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>29490.48</v>
+        <v>3845.25</v>
       </c>
       <c r="M11" t="n">
-        <v>29490.48</v>
+        <v>3845.25</v>
       </c>
     </row>
     <row r="12">
@@ -834,10 +834,10 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>5090.96</v>
+        <v>6968.21</v>
       </c>
       <c r="I12" t="n">
-        <v>5090.96</v>
+        <v>6968.21</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -846,16 +846,16 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>48657.15</v>
+        <v>47121.66</v>
       </c>
       <c r="M12" t="n">
-        <v>48657.15</v>
+        <v>47121.66</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>94156</t>
+          <t>104750</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -865,7 +865,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MARIA TERESA ASENCIO LOZANO</t>
+          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -877,10 +877,10 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>4709.73</v>
+        <v>5442.15</v>
       </c>
       <c r="I13" t="n">
-        <v>4709.73</v>
+        <v>5442.15</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -889,16 +889,16 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>2309.36</v>
+        <v>35695.8</v>
       </c>
       <c r="M13" t="n">
-        <v>2309.36</v>
+        <v>35695.8</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -920,10 +920,10 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>4021.19</v>
+        <v>5431.4</v>
       </c>
       <c r="I14" t="n">
-        <v>4021.19</v>
+        <v>5431.4</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -932,26 +932,26 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>31449.72</v>
+        <v>12899.71</v>
       </c>
       <c r="M14" t="n">
-        <v>31449.72</v>
+        <v>12899.71</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>94156</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>MARIA TERESA ASENCIO LOZANO</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -963,10 +963,10 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>3524.19</v>
+        <v>4709.73</v>
       </c>
       <c r="I15" t="n">
-        <v>3524.19</v>
+        <v>4709.73</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -975,16 +975,16 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>68825.82000000001</v>
+        <v>2309.36</v>
       </c>
       <c r="M15" t="n">
-        <v>68825.82000000001</v>
+        <v>2309.36</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>109998</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1006,38 +1006,38 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>2966.58</v>
+        <v>4021.19</v>
       </c>
       <c r="I16" t="n">
-        <v>2966.58</v>
+        <v>4021.19</v>
       </c>
       <c r="J16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>1483.13</v>
       </c>
       <c r="L16" t="n">
-        <v>0</v>
+        <v>31449.72</v>
       </c>
       <c r="M16" t="n">
-        <v>0</v>
+        <v>32932.85</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>104750</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1049,10 +1049,10 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>2426.76</v>
+        <v>3524.19</v>
       </c>
       <c r="I17" t="n">
-        <v>2426.76</v>
+        <v>3524.19</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1061,16 +1061,16 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>38711.19</v>
+        <v>68825.82000000001</v>
       </c>
       <c r="M17" t="n">
-        <v>38711.19</v>
+        <v>68825.82000000001</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>109998</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1080,7 +1080,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1092,10 +1092,10 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>2408.61</v>
+        <v>2966.58</v>
       </c>
       <c r="I18" t="n">
-        <v>2408.61</v>
+        <v>2966.58</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1104,41 +1104,41 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>5453.73</v>
+        <v>0</v>
       </c>
       <c r="M18" t="n">
-        <v>5453.73</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>118246</t>
+          <t>120051</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>JOSE ANTEMIO OLIVA SANTOS</t>
+          <t>GUILLERMO JOSE RAMIREZ RAMIREZ</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G19" t="n">
-        <v>0</v>
+        <v>2488.17</v>
       </c>
       <c r="H19" t="n">
-        <v>1967.73</v>
+        <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>1967.73</v>
+        <v>2488.17</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1147,16 +1147,16 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>26288.67</v>
+        <v>27369.85</v>
       </c>
       <c r="M19" t="n">
-        <v>26288.67</v>
+        <v>27369.85</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>118246</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>JOSE ANTEMIO OLIVA SANTOS</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1178,10 +1178,10 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>1800.77</v>
+        <v>1967.73</v>
       </c>
       <c r="I20" t="n">
-        <v>1800.77</v>
+        <v>1967.73</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1190,16 +1190,16 @@
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>10804.65</v>
+        <v>26288.67</v>
       </c>
       <c r="M20" t="n">
-        <v>10804.65</v>
+        <v>26288.67</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1221,10 +1221,10 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>1761.04</v>
+        <v>1800.77</v>
       </c>
       <c r="I21" t="n">
-        <v>1761.04</v>
+        <v>1800.77</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -1233,16 +1233,16 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>7337.05</v>
+        <v>10804.65</v>
       </c>
       <c r="M21" t="n">
-        <v>7337.05</v>
+        <v>10804.65</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>65046</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -1264,10 +1264,10 @@
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>1747.29</v>
+        <v>1761.04</v>
       </c>
       <c r="I22" t="n">
-        <v>1747.29</v>
+        <v>1761.04</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1276,16 +1276,16 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>3494.59</v>
+        <v>38072.49</v>
       </c>
       <c r="M22" t="n">
-        <v>3494.59</v>
+        <v>38072.49</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>105696</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>GABRIELA CASTAÐEDA SALAZAR</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -1307,10 +1307,10 @@
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>1737.43</v>
+        <v>1761.04</v>
       </c>
       <c r="I23" t="n">
-        <v>1737.43</v>
+        <v>1761.04</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -1319,16 +1319,16 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>91447.39999999999</v>
+        <v>7337.05</v>
       </c>
       <c r="M23" t="n">
-        <v>91447.39999999999</v>
+        <v>7337.05</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>65046</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1350,10 +1350,10 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>1516.55</v>
+        <v>1747.29</v>
       </c>
       <c r="I24" t="n">
-        <v>1516.55</v>
+        <v>1747.29</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
@@ -1362,26 +1362,26 @@
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>0</v>
+        <v>3494.59</v>
       </c>
       <c r="M24" t="n">
-        <v>0</v>
+        <v>3494.59</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>120051</t>
+          <t>105696</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>GUILLERMO JOSE RAMIREZ RAMIREZ</t>
+          <t>GABRIELA CASTAÐEDA SALAZAR</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1393,38 +1393,38 @@
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>0</v>
+        <v>1737.43</v>
       </c>
       <c r="I25" t="n">
-        <v>0</v>
+        <v>1737.43</v>
       </c>
       <c r="J25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K25" t="n">
-        <v>2488.17</v>
+        <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>27369.85</v>
+        <v>91447.39999999999</v>
       </c>
       <c r="M25" t="n">
-        <v>29858.02</v>
+        <v>91447.39999999999</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>119447</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>LUIS ANTONIO SALAZAR ESPINOSA</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1436,10 +1436,10 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>0</v>
+        <v>1516.55</v>
       </c>
       <c r="I26" t="n">
-        <v>0</v>
+        <v>1516.55</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1448,26 +1448,26 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>52810.13</v>
+        <v>0</v>
       </c>
       <c r="M26" t="n">
-        <v>52810.13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>119223</t>
+          <t>119447</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>OSCAR RAMIREZ RUIZ</t>
+          <t>LUIS ANTONIO SALAZAR ESPINOSA</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1485,22 +1485,22 @@
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K27" t="n">
-        <v>0</v>
+        <v>1742.89</v>
       </c>
       <c r="L27" t="n">
-        <v>26414.27</v>
+        <v>71981.92</v>
       </c>
       <c r="M27" t="n">
-        <v>26414.27</v>
+        <v>73724.81</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>118915</t>
+          <t>119223</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1510,7 +1510,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
+          <t>OSCAR RAMIREZ RUIZ</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1534,26 +1534,26 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>49113.6</v>
+        <v>26414.27</v>
       </c>
       <c r="M28" t="n">
-        <v>49113.6</v>
+        <v>26414.27</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>118069</t>
+          <t>118915</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>MARIO IVAN ROMERO GONZALEZ</t>
+          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1577,26 +1577,26 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>42404.25</v>
+        <v>49113.6</v>
       </c>
       <c r="M29" t="n">
-        <v>42404.25</v>
+        <v>49113.6</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>116795</t>
+          <t>118069</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>GERARDO DANIEL BARAJAS TORRES</t>
+          <t>MARIO IVAN ROMERO GONZALEZ</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1620,26 +1620,26 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>4796.14</v>
+        <v>42404.25</v>
       </c>
       <c r="M30" t="n">
-        <v>4796.14</v>
+        <v>42404.25</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>116795</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>GERARDO DANIEL BARAJAS TORRES</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1663,26 +1663,26 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>17269.74</v>
+        <v>4796.14</v>
       </c>
       <c r="M31" t="n">
-        <v>17269.74</v>
+        <v>4796.14</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>115404</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -1706,16 +1706,16 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>3487.19</v>
+        <v>17269.74</v>
       </c>
       <c r="M32" t="n">
-        <v>3487.19</v>
+        <v>17269.74</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1749,16 +1749,16 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>1693.99</v>
+        <v>3487.19</v>
       </c>
       <c r="M33" t="n">
-        <v>1693.99</v>
+        <v>3487.19</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1768,7 +1768,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1792,26 +1792,26 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>17425.73</v>
+        <v>1693.99</v>
       </c>
       <c r="M34" t="n">
-        <v>17425.73</v>
+        <v>1693.99</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>114100</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1835,26 +1835,26 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>6410.16</v>
+        <v>17425.73</v>
       </c>
       <c r="M35" t="n">
-        <v>6410.16</v>
+        <v>17425.73</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>113450</t>
+          <t>114100</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
+          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1878,16 +1878,16 @@
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>18650.03</v>
+        <v>6410.16</v>
       </c>
       <c r="M36" t="n">
-        <v>18650.03</v>
+        <v>6410.16</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>111056</t>
+          <t>113450</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>JORGE ANTONIO LUNA LARA</t>
+          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1921,16 +1921,16 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>67074.12</v>
+        <v>18650.03</v>
       </c>
       <c r="M37" t="n">
-        <v>67074.12</v>
+        <v>18650.03</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>110575</t>
+          <t>111056</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>JOSE RENE DE ALBA MORALES</t>
+          <t>JORGE ANTONIO LUNA LARA</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1964,16 +1964,16 @@
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>14427.08</v>
+        <v>67074.12</v>
       </c>
       <c r="M38" t="n">
-        <v>14427.08</v>
+        <v>67074.12</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>110575</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>JOSE RENE DE ALBA MORALES</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -2007,16 +2007,16 @@
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>3041.47</v>
+        <v>14427.08</v>
       </c>
       <c r="M39" t="n">
-        <v>3041.47</v>
+        <v>14427.08</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>108405</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2050,10 +2050,10 @@
         <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>39833.53</v>
+        <v>3041.47</v>
       </c>
       <c r="M40" t="n">
-        <v>39833.53</v>
+        <v>3041.47</v>
       </c>
     </row>
     <row r="41">

</xml_diff>

<commit_message>
data: Actualización de reporte Pagado / Pendiente (corte 15 de septiembre 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>11 de septiembre de 2026</t>
+          <t>15 de septiembre de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -468,7 +468,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>115047</t>
+          <t>110453</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -478,7 +478,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>VELIA PATRICIA BERNAL RAMOS</t>
+          <t>ANAIS LUA MORENO</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -487,31 +487,31 @@
         <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>39037.05</v>
+        <v>29655.2</v>
       </c>
       <c r="H4" t="n">
-        <v>6821.96</v>
+        <v>17330.39</v>
       </c>
       <c r="I4" t="n">
-        <v>45859.01</v>
+        <v>46985.59</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>35695.85</v>
       </c>
       <c r="L4" t="n">
-        <v>19745.09</v>
+        <v>84031.55</v>
       </c>
       <c r="M4" t="n">
-        <v>19745.09</v>
+        <v>119727.4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>110453</t>
+          <t>115047</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -521,7 +521,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ANAIS LUA MORENO</t>
+          <t>VELIA PATRICIA BERNAL RAMOS</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -530,13 +530,13 @@
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>29655.2</v>
+        <v>39037.05</v>
       </c>
       <c r="H5" t="n">
-        <v>11503.4</v>
+        <v>6821.96</v>
       </c>
       <c r="I5" t="n">
-        <v>41158.6</v>
+        <v>45859.01</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -545,41 +545,41 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>89858.53999999999</v>
+        <v>19745.09</v>
       </c>
       <c r="M5" t="n">
-        <v>89858.53999999999</v>
+        <v>19745.09</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>116883</t>
+          <t>104750</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>SOFIA CAMPILLO VASCONCELOS</t>
+          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>37215.83</v>
       </c>
       <c r="H6" t="n">
-        <v>19029.58</v>
+        <v>5442.15</v>
       </c>
       <c r="I6" t="n">
-        <v>19029.58</v>
+        <v>42657.98</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -588,41 +588,41 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>90474.05</v>
+        <v>35695.8</v>
       </c>
       <c r="M6" t="n">
-        <v>90474.05</v>
+        <v>35695.8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>87538</t>
+          <t>116883</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
+          <t>SOFIA CAMPILLO VASCONCELOS</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>6853.85</v>
+        <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>12121.29</v>
+        <v>19029.58</v>
       </c>
       <c r="I7" t="n">
-        <v>18975.14</v>
+        <v>19029.58</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -631,16 +631,16 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>231506.85</v>
+        <v>90474.05</v>
       </c>
       <c r="M7" t="n">
-        <v>231506.85</v>
+        <v>90474.05</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>104718</t>
+          <t>87538</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -650,22 +650,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ROGELIO TORRES ORTIZ</t>
+          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>6853.85</v>
       </c>
       <c r="H8" t="n">
-        <v>18318.58</v>
+        <v>12121.29</v>
       </c>
       <c r="I8" t="n">
-        <v>18318.58</v>
+        <v>18975.14</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -674,16 +674,16 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>16324.8</v>
+        <v>231506.85</v>
       </c>
       <c r="M8" t="n">
-        <v>16324.8</v>
+        <v>231506.85</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>117440</t>
+          <t>104718</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MONSERRAT VELASCO SANTOS</t>
+          <t>ROGELIO TORRES ORTIZ</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
@@ -705,10 +705,10 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>12218.55</v>
+        <v>18318.58</v>
       </c>
       <c r="I9" t="n">
-        <v>12218.55</v>
+        <v>18318.58</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -717,16 +717,16 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>62871.21</v>
+        <v>16324.8</v>
       </c>
       <c r="M9" t="n">
-        <v>62871.21</v>
+        <v>16324.8</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>117440</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -736,7 +736,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>MONSERRAT VELASCO SANTOS</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -748,10 +748,10 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>11245.61</v>
+        <v>12218.55</v>
       </c>
       <c r="I10" t="n">
-        <v>11245.61</v>
+        <v>12218.55</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -760,16 +760,16 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>0</v>
+        <v>62871.21</v>
       </c>
       <c r="M10" t="n">
-        <v>0</v>
+        <v>62871.21</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>88234</t>
+          <t>119223</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -779,22 +779,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
+          <t>OSCAR RAMIREZ RUIZ</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>12054.68</v>
       </c>
       <c r="H11" t="n">
-        <v>8492.07</v>
+        <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>8492.07</v>
+        <v>12054.68</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -803,16 +803,16 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>3845.25</v>
+        <v>38468.95</v>
       </c>
       <c r="M11" t="n">
-        <v>3845.25</v>
+        <v>38468.95</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>47116</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -822,7 +822,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -834,10 +834,10 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>6968.21</v>
+        <v>11245.61</v>
       </c>
       <c r="I12" t="n">
-        <v>6968.21</v>
+        <v>11245.61</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -846,16 +846,16 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>47121.66</v>
+        <v>0</v>
       </c>
       <c r="M12" t="n">
-        <v>47121.66</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>104750</t>
+          <t>88234</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -865,7 +865,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
+          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -877,10 +877,10 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>5442.15</v>
+        <v>8492.07</v>
       </c>
       <c r="I13" t="n">
-        <v>5442.15</v>
+        <v>8492.07</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -889,16 +889,16 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>35695.8</v>
+        <v>3845.25</v>
       </c>
       <c r="M13" t="n">
-        <v>35695.8</v>
+        <v>3845.25</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>47116</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -920,10 +920,10 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>5431.4</v>
+        <v>6968.21</v>
       </c>
       <c r="I14" t="n">
-        <v>5431.4</v>
+        <v>6968.21</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -932,16 +932,16 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>12899.71</v>
+        <v>47121.66</v>
       </c>
       <c r="M14" t="n">
-        <v>12899.71</v>
+        <v>47121.66</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>94156</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -951,22 +951,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MARIA TERESA ASENCIO LOZANO</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>1203.25</v>
       </c>
       <c r="H15" t="n">
-        <v>4709.73</v>
+        <v>4925.15</v>
       </c>
       <c r="I15" t="n">
-        <v>4709.73</v>
+        <v>6128.4</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -975,16 +975,16 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>2309.36</v>
+        <v>31449.72</v>
       </c>
       <c r="M15" t="n">
-        <v>2309.36</v>
+        <v>31449.72</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1006,38 +1006,38 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>4021.19</v>
+        <v>6091.05</v>
       </c>
       <c r="I16" t="n">
-        <v>4021.19</v>
+        <v>6091.05</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>1483.13</v>
+        <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>31449.72</v>
+        <v>14237.3</v>
       </c>
       <c r="M16" t="n">
-        <v>32932.85</v>
+        <v>14237.3</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1049,10 +1049,10 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>3524.19</v>
+        <v>5431.4</v>
       </c>
       <c r="I17" t="n">
-        <v>3524.19</v>
+        <v>5431.4</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1061,16 +1061,16 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>68825.82000000001</v>
+        <v>12899.71</v>
       </c>
       <c r="M17" t="n">
-        <v>68825.82000000001</v>
+        <v>12899.71</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>109998</t>
+          <t>80122</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1080,7 +1080,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
+          <t>DESIREE DE LA PEÐA OROZCO</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1092,53 +1092,53 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>2966.58</v>
+        <v>4743.3</v>
       </c>
       <c r="I18" t="n">
-        <v>2966.58</v>
+        <v>4743.3</v>
       </c>
       <c r="J18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>72893.8</v>
       </c>
       <c r="L18" t="n">
-        <v>0</v>
+        <v>75998.97</v>
       </c>
       <c r="M18" t="n">
-        <v>0</v>
+        <v>148892.77</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>120051</t>
+          <t>94156</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>GUILLERMO JOSE RAMIREZ RAMIREZ</t>
+          <t>MARIA TERESA ASENCIO LOZANO</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>2488.17</v>
+        <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>0</v>
+        <v>4709.73</v>
       </c>
       <c r="I19" t="n">
-        <v>2488.17</v>
+        <v>4709.73</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1147,26 +1147,26 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>27369.85</v>
+        <v>2309.36</v>
       </c>
       <c r="M19" t="n">
-        <v>27369.85</v>
+        <v>2309.36</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>118246</t>
+          <t>114100</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>JOSE ANTEMIO OLIVA SANTOS</t>
+          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1178,10 +1178,10 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>1967.73</v>
+        <v>3961.9</v>
       </c>
       <c r="I20" t="n">
-        <v>1967.73</v>
+        <v>3961.9</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1190,16 +1190,16 @@
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>26288.67</v>
+        <v>6410.16</v>
       </c>
       <c r="M20" t="n">
-        <v>26288.67</v>
+        <v>6410.16</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>108405</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1221,10 +1221,10 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>1800.77</v>
+        <v>3041.47</v>
       </c>
       <c r="I21" t="n">
-        <v>1800.77</v>
+        <v>3041.47</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -1233,16 +1233,16 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>10804.65</v>
+        <v>0</v>
       </c>
       <c r="M21" t="n">
-        <v>10804.65</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>109998</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -1264,10 +1264,10 @@
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>1761.04</v>
+        <v>2966.58</v>
       </c>
       <c r="I22" t="n">
-        <v>1761.04</v>
+        <v>2966.58</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1276,41 +1276,41 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>38072.49</v>
+        <v>0</v>
       </c>
       <c r="M22" t="n">
-        <v>38072.49</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>120051</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>GUILLERMO JOSE RAMIREZ RAMIREZ</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G23" t="n">
-        <v>0</v>
+        <v>2488.17</v>
       </c>
       <c r="H23" t="n">
-        <v>1761.04</v>
+        <v>0</v>
       </c>
       <c r="I23" t="n">
-        <v>1761.04</v>
+        <v>2488.17</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -1319,16 +1319,16 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>7337.05</v>
+        <v>27369.85</v>
       </c>
       <c r="M23" t="n">
-        <v>7337.05</v>
+        <v>27369.85</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>65046</t>
+          <t>118246</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+          <t>JOSE ANTEMIO OLIVA SANTOS</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1350,10 +1350,10 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>1747.29</v>
+        <v>1967.73</v>
       </c>
       <c r="I24" t="n">
-        <v>1747.29</v>
+        <v>1967.73</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
@@ -1362,16 +1362,16 @@
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>3494.59</v>
+        <v>23551.39</v>
       </c>
       <c r="M24" t="n">
-        <v>3494.59</v>
+        <v>23551.39</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>105696</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1381,7 +1381,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>GABRIELA CASTAÐEDA SALAZAR</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1393,10 +1393,10 @@
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>1737.43</v>
+        <v>1800.77</v>
       </c>
       <c r="I25" t="n">
-        <v>1737.43</v>
+        <v>1800.77</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -1405,16 +1405,16 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>91447.39999999999</v>
+        <v>10804.65</v>
       </c>
       <c r="M25" t="n">
-        <v>91447.39999999999</v>
+        <v>10804.65</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1436,10 +1436,10 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>1516.55</v>
+        <v>1761.04</v>
       </c>
       <c r="I26" t="n">
-        <v>1516.55</v>
+        <v>1761.04</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1448,26 +1448,26 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>0</v>
+        <v>7337.05</v>
       </c>
       <c r="M26" t="n">
-        <v>0</v>
+        <v>7337.05</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>119447</t>
+          <t>65046</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>LUIS ANTONIO SALAZAR ESPINOSA</t>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1479,53 +1479,53 @@
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>0</v>
+        <v>1747.29</v>
       </c>
       <c r="I27" t="n">
-        <v>0</v>
+        <v>1747.29</v>
       </c>
       <c r="J27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K27" t="n">
-        <v>1742.89</v>
+        <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>71981.92</v>
+        <v>3494.59</v>
       </c>
       <c r="M27" t="n">
-        <v>73724.81</v>
+        <v>3494.59</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>119223</t>
+          <t>119447</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>OSCAR RAMIREZ RUIZ</t>
+          <t>LUIS ANTONIO SALAZAR ESPINOSA</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G28" t="n">
-        <v>0</v>
+        <v>1742.89</v>
       </c>
       <c r="H28" t="n">
         <v>0</v>
       </c>
       <c r="I28" t="n">
-        <v>0</v>
+        <v>1742.89</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -1534,16 +1534,16 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>26414.27</v>
+        <v>71981.92</v>
       </c>
       <c r="M28" t="n">
-        <v>26414.27</v>
+        <v>71981.92</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>118915</t>
+          <t>105696</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
+          <t>GABRIELA CASTAÐEDA SALAZAR</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1565,10 +1565,10 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>0</v>
+        <v>1737.43</v>
       </c>
       <c r="I29" t="n">
-        <v>0</v>
+        <v>1737.43</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -1577,10 +1577,10 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>49113.6</v>
+        <v>91447.39999999999</v>
       </c>
       <c r="M29" t="n">
-        <v>49113.6</v>
+        <v>91447.39999999999</v>
       </c>
     </row>
     <row r="30">
@@ -1608,10 +1608,10 @@
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>0</v>
+        <v>1662.54</v>
       </c>
       <c r="I30" t="n">
-        <v>0</v>
+        <v>1662.54</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1620,16 +1620,16 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>42404.25</v>
+        <v>40741.71</v>
       </c>
       <c r="M30" t="n">
-        <v>42404.25</v>
+        <v>40741.71</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>116795</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>GERARDO DANIEL BARAJAS TORRES</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1651,10 +1651,10 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>0</v>
+        <v>1516.55</v>
       </c>
       <c r="I31" t="n">
-        <v>0</v>
+        <v>1516.55</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1663,16 +1663,16 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>4796.14</v>
+        <v>0</v>
       </c>
       <c r="M31" t="n">
-        <v>4796.14</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -1691,13 +1691,13 @@
         <v>0</v>
       </c>
       <c r="G32" t="n">
-        <v>0</v>
+        <v>-2313.19</v>
       </c>
       <c r="H32" t="n">
-        <v>0</v>
+        <v>3524.19</v>
       </c>
       <c r="I32" t="n">
-        <v>0</v>
+        <v>1211</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1706,16 +1706,16 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>17269.74</v>
+        <v>43380.7</v>
       </c>
       <c r="M32" t="n">
-        <v>17269.74</v>
+        <v>43380.7</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>115404</t>
+          <t>118915</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
+          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1749,16 +1749,16 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>3487.19</v>
+        <v>49113.6</v>
       </c>
       <c r="M33" t="n">
-        <v>3487.19</v>
+        <v>49113.6</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>116795</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1768,7 +1768,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>GERARDO DANIEL BARAJAS TORRES</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1792,26 +1792,26 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>1693.99</v>
+        <v>4796.14</v>
       </c>
       <c r="M34" t="n">
-        <v>1693.99</v>
+        <v>4796.14</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1835,26 +1835,26 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>17425.73</v>
+        <v>17269.74</v>
       </c>
       <c r="M35" t="n">
-        <v>17425.73</v>
+        <v>17269.74</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>114100</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1878,16 +1878,16 @@
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>6410.16</v>
+        <v>3487.19</v>
       </c>
       <c r="M36" t="n">
-        <v>6410.16</v>
+        <v>3487.19</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>113450</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1921,16 +1921,16 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>18650.03</v>
+        <v>1693.99</v>
       </c>
       <c r="M37" t="n">
-        <v>18650.03</v>
+        <v>1693.99</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>111056</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>JORGE ANTONIO LUNA LARA</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1964,16 +1964,16 @@
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>67074.12</v>
+        <v>17425.73</v>
       </c>
       <c r="M38" t="n">
-        <v>67074.12</v>
+        <v>17425.73</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>110575</t>
+          <t>113450</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>JOSE RENE DE ALBA MORALES</t>
+          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -2007,16 +2007,16 @@
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>14427.08</v>
+        <v>18650.03</v>
       </c>
       <c r="M39" t="n">
-        <v>14427.08</v>
+        <v>18650.03</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>111056</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>JORGE ANTONIO LUNA LARA</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2050,16 +2050,16 @@
         <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>3041.47</v>
+        <v>67074.12</v>
       </c>
       <c r="M40" t="n">
-        <v>3041.47</v>
+        <v>67074.12</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>106018</t>
+          <t>110575</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>MIREYA LIZETTE TORRES GARCIA</t>
+          <t>JOSE RENE DE ALBA MORALES</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2093,16 +2093,16 @@
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>23106.58</v>
+        <v>14427.08</v>
       </c>
       <c r="M41" t="n">
-        <v>23106.58</v>
+        <v>14427.08</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>104343</t>
+          <t>106018</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
+          <t>MIREYA LIZETTE TORRES GARCIA</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2136,16 +2136,16 @@
         <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>12811.03</v>
+        <v>23106.58</v>
       </c>
       <c r="M42" t="n">
-        <v>12811.03</v>
+        <v>23106.58</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>103982</t>
+          <t>104343</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA RIOS BERNAL</t>
+          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -2179,16 +2179,16 @@
         <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>6060.86</v>
+        <v>12811.03</v>
       </c>
       <c r="M43" t="n">
-        <v>6060.86</v>
+        <v>12811.03</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>101640</t>
+          <t>103982</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2198,7 +2198,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>SAMUEL NUÐO RIVERA</t>
+          <t>MARIA FERNANDA RIOS BERNAL</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -2222,16 +2222,16 @@
         <v>0</v>
       </c>
       <c r="L44" t="n">
-        <v>3214.14</v>
+        <v>6060.86</v>
       </c>
       <c r="M44" t="n">
-        <v>3214.14</v>
+        <v>6060.86</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>95148</t>
+          <t>101640</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2241,7 +2241,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
+          <t>SAMUEL NUÐO RIVERA</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -2265,16 +2265,16 @@
         <v>0</v>
       </c>
       <c r="L45" t="n">
-        <v>56725.37</v>
+        <v>3214.14</v>
       </c>
       <c r="M45" t="n">
-        <v>56725.37</v>
+        <v>3214.14</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>90355</t>
+          <t>95148</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2284,7 +2284,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>DARINKA UREÐA CASILLAS</t>
+          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -2308,16 +2308,16 @@
         <v>0</v>
       </c>
       <c r="L46" t="n">
-        <v>86129.07000000001</v>
+        <v>56725.37</v>
       </c>
       <c r="M46" t="n">
-        <v>86129.07000000001</v>
+        <v>56725.37</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>80122</t>
+          <t>90355</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2327,7 +2327,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>DESIREE DE LA PEÐA OROZCO</t>
+          <t>DARINKA UREÐA CASILLAS</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -2345,16 +2345,16 @@
         <v>0</v>
       </c>
       <c r="J47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K47" t="n">
-        <v>72893.8</v>
+        <v>0</v>
       </c>
       <c r="L47" t="n">
-        <v>80312.75</v>
+        <v>86129.07000000001</v>
       </c>
       <c r="M47" t="n">
-        <v>153206.55</v>
+        <v>86129.07000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-09-18 14:05)
Incluye snapshot corregido tras el fix de fecha de corte (QsQ GMM y
Asesores sin Emisión).
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>15 de septiembre de 2026</t>
+          <t>17 de septiembre de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -490,10 +490,10 @@
         <v>29655.2</v>
       </c>
       <c r="H4" t="n">
-        <v>17330.39</v>
+        <v>19128.87</v>
       </c>
       <c r="I4" t="n">
-        <v>46985.59</v>
+        <v>48784.07</v>
       </c>
       <c r="J4" t="n">
         <v>1</v>
@@ -502,10 +502,10 @@
         <v>35695.85</v>
       </c>
       <c r="L4" t="n">
-        <v>84031.55</v>
+        <v>82233.07000000001</v>
       </c>
       <c r="M4" t="n">
-        <v>119727.4</v>
+        <v>117928.92</v>
       </c>
     </row>
     <row r="5">
@@ -619,10 +619,10 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>19029.58</v>
+        <v>20796.52</v>
       </c>
       <c r="I7" t="n">
-        <v>19029.58</v>
+        <v>20796.52</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -631,10 +631,10 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>90474.05</v>
+        <v>88707.11</v>
       </c>
       <c r="M7" t="n">
-        <v>90474.05</v>
+        <v>88707.11</v>
       </c>
     </row>
     <row r="8">
@@ -726,7 +726,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>117440</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -736,7 +736,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MONSERRAT VELASCO SANTOS</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -748,10 +748,10 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>12218.55</v>
+        <v>12261.72</v>
       </c>
       <c r="I10" t="n">
-        <v>12218.55</v>
+        <v>12261.72</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -760,16 +760,16 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>62871.21</v>
+        <v>0</v>
       </c>
       <c r="M10" t="n">
-        <v>62871.21</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>119223</t>
+          <t>117440</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -779,22 +779,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>OSCAR RAMIREZ RUIZ</t>
+          <t>MONSERRAT VELASCO SANTOS</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>12054.68</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>12218.55</v>
       </c>
       <c r="I11" t="n">
-        <v>12054.68</v>
+        <v>12218.55</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -803,16 +803,16 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>38468.95</v>
+        <v>62871.21</v>
       </c>
       <c r="M11" t="n">
-        <v>38468.95</v>
+        <v>62871.21</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>119223</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -822,22 +822,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>OSCAR RAMIREZ RUIZ</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>12054.68</v>
       </c>
       <c r="H12" t="n">
-        <v>11245.61</v>
+        <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>11245.61</v>
+        <v>12054.68</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -846,10 +846,10 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>0</v>
+        <v>38468.95</v>
       </c>
       <c r="M12" t="n">
-        <v>0</v>
+        <v>38468.95</v>
       </c>
     </row>
     <row r="13">
@@ -898,7 +898,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>47116</t>
+          <t>80122</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
+          <t>DESIREE DE LA PEÐA OROZCO</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -920,28 +920,28 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>6968.21</v>
+        <v>8390.049999999999</v>
       </c>
       <c r="I14" t="n">
-        <v>6968.21</v>
+        <v>8390.049999999999</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>72893.8</v>
       </c>
       <c r="L14" t="n">
-        <v>47121.66</v>
+        <v>75998.97</v>
       </c>
       <c r="M14" t="n">
-        <v>47121.66</v>
+        <v>148892.77</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -951,22 +951,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>1203.25</v>
+        <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>4925.15</v>
+        <v>7624.07</v>
       </c>
       <c r="I15" t="n">
-        <v>6128.4</v>
+        <v>7624.07</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -975,16 +975,16 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>31449.72</v>
+        <v>12705.8</v>
       </c>
       <c r="M15" t="n">
-        <v>31449.72</v>
+        <v>12705.8</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>47116</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1006,10 +1006,10 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>6091.05</v>
+        <v>6968.21</v>
       </c>
       <c r="I16" t="n">
-        <v>6091.05</v>
+        <v>6968.21</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1018,16 +1018,16 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>14237.3</v>
+        <v>47121.66</v>
       </c>
       <c r="M16" t="n">
-        <v>14237.3</v>
+        <v>47121.66</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1037,40 +1037,40 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G17" t="n">
-        <v>0</v>
+        <v>1203.25</v>
       </c>
       <c r="H17" t="n">
-        <v>5431.4</v>
+        <v>4925.15</v>
       </c>
       <c r="I17" t="n">
-        <v>5431.4</v>
+        <v>6128.4</v>
       </c>
       <c r="J17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K17" t="n">
-        <v>0</v>
+        <v>29652.91</v>
       </c>
       <c r="L17" t="n">
-        <v>12899.71</v>
+        <v>31449.72</v>
       </c>
       <c r="M17" t="n">
-        <v>12899.71</v>
+        <v>61102.63</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>80122</t>
+          <t>103982</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1080,7 +1080,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>DESIREE DE LA PEÐA OROZCO</t>
+          <t>MARIA FERNANDA RIOS BERNAL</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1092,28 +1092,28 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>4743.3</v>
+        <v>6060.91</v>
       </c>
       <c r="I18" t="n">
-        <v>4743.3</v>
+        <v>6060.91</v>
       </c>
       <c r="J18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>72893.8</v>
+        <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>75998.97</v>
+        <v>0</v>
       </c>
       <c r="M18" t="n">
-        <v>148892.77</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>94156</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MARIA TERESA ASENCIO LOZANO</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>4709.73</v>
+        <v>5431.4</v>
       </c>
       <c r="I19" t="n">
-        <v>4709.73</v>
+        <v>5431.4</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1147,26 +1147,26 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>2309.36</v>
+        <v>12899.71</v>
       </c>
       <c r="M19" t="n">
-        <v>2309.36</v>
+        <v>12899.71</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>114100</t>
+          <t>94156</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
+          <t>MARIA TERESA ASENCIO LOZANO</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1178,10 +1178,10 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>3961.9</v>
+        <v>4709.73</v>
       </c>
       <c r="I20" t="n">
-        <v>3961.9</v>
+        <v>4709.73</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1190,26 +1190,26 @@
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>6410.16</v>
+        <v>2309.36</v>
       </c>
       <c r="M20" t="n">
-        <v>6410.16</v>
+        <v>2309.36</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>114100</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1221,10 +1221,10 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>3041.47</v>
+        <v>3961.9</v>
       </c>
       <c r="I21" t="n">
-        <v>3041.47</v>
+        <v>3961.9</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -1233,16 +1233,16 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>0</v>
+        <v>6410.16</v>
       </c>
       <c r="M21" t="n">
-        <v>0</v>
+        <v>6410.16</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>109998</t>
+          <t>95148</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
+          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -1264,10 +1264,10 @@
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>2966.58</v>
+        <v>3898.73</v>
       </c>
       <c r="I22" t="n">
-        <v>2966.58</v>
+        <v>3898.73</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1276,41 +1276,41 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>0</v>
+        <v>52826.69</v>
       </c>
       <c r="M22" t="n">
-        <v>0</v>
+        <v>52826.69</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>120051</t>
+          <t>108405</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>GUILLERMO JOSE RAMIREZ RAMIREZ</t>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>2488.17</v>
+        <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>0</v>
+        <v>3041.47</v>
       </c>
       <c r="I23" t="n">
-        <v>2488.17</v>
+        <v>3041.47</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -1319,16 +1319,16 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>27369.85</v>
+        <v>0</v>
       </c>
       <c r="M23" t="n">
-        <v>27369.85</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>118246</t>
+          <t>109998</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>JOSE ANTEMIO OLIVA SANTOS</t>
+          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1350,10 +1350,10 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>1967.73</v>
+        <v>2966.58</v>
       </c>
       <c r="I24" t="n">
-        <v>1967.73</v>
+        <v>2966.58</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
@@ -1362,41 +1362,41 @@
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>23551.39</v>
+        <v>0</v>
       </c>
       <c r="M24" t="n">
-        <v>23551.39</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>120051</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>GUILLERMO JOSE RAMIREZ RAMIREZ</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G25" t="n">
-        <v>0</v>
+        <v>2488.17</v>
       </c>
       <c r="H25" t="n">
-        <v>1800.77</v>
+        <v>0</v>
       </c>
       <c r="I25" t="n">
-        <v>1800.77</v>
+        <v>2488.17</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -1405,16 +1405,16 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>10804.65</v>
+        <v>27369.85</v>
       </c>
       <c r="M25" t="n">
-        <v>10804.65</v>
+        <v>27369.85</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>90355</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>DARINKA UREÐA CASILLAS</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1436,10 +1436,10 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>1761.04</v>
+        <v>2362.88</v>
       </c>
       <c r="I26" t="n">
-        <v>1761.04</v>
+        <v>2362.88</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1448,16 +1448,16 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>7337.05</v>
+        <v>83766.14999999999</v>
       </c>
       <c r="M26" t="n">
-        <v>7337.05</v>
+        <v>83766.14999999999</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>65046</t>
+          <t>118246</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+          <t>JOSE ANTEMIO OLIVA SANTOS</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1479,10 +1479,10 @@
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>1747.29</v>
+        <v>1967.73</v>
       </c>
       <c r="I27" t="n">
-        <v>1747.29</v>
+        <v>1967.73</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
@@ -1491,41 +1491,41 @@
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>3494.59</v>
+        <v>23551.39</v>
       </c>
       <c r="M27" t="n">
-        <v>3494.59</v>
+        <v>23551.39</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>119447</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>LUIS ANTONIO SALAZAR ESPINOSA</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>1742.89</v>
+        <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>0</v>
+        <v>1800.77</v>
       </c>
       <c r="I28" t="n">
-        <v>1742.89</v>
+        <v>1800.77</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -1534,16 +1534,16 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>71981.92</v>
+        <v>10804.65</v>
       </c>
       <c r="M28" t="n">
-        <v>71981.92</v>
+        <v>10804.65</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>105696</t>
+          <t>106018</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>GABRIELA CASTAÐEDA SALAZAR</t>
+          <t>MIREYA LIZETTE TORRES GARCIA</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1565,10 +1565,10 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>1737.43</v>
+        <v>1773.2</v>
       </c>
       <c r="I29" t="n">
-        <v>1737.43</v>
+        <v>1773.2</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -1577,26 +1577,26 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>91447.39999999999</v>
+        <v>21333.38</v>
       </c>
       <c r="M29" t="n">
-        <v>91447.39999999999</v>
+        <v>21333.38</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>118069</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>MARIO IVAN ROMERO GONZALEZ</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1608,10 +1608,10 @@
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>1662.54</v>
+        <v>1761.04</v>
       </c>
       <c r="I30" t="n">
-        <v>1662.54</v>
+        <v>1761.04</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1620,16 +1620,16 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>40741.71</v>
+        <v>7337.05</v>
       </c>
       <c r="M30" t="n">
-        <v>40741.71</v>
+        <v>7337.05</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>65046</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1651,10 +1651,10 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>1516.55</v>
+        <v>1747.29</v>
       </c>
       <c r="I31" t="n">
-        <v>1516.55</v>
+        <v>1747.29</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1663,16 +1663,16 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>0</v>
+        <v>3494.59</v>
       </c>
       <c r="M31" t="n">
-        <v>0</v>
+        <v>3494.59</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>119447</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1682,22 +1682,22 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>LUIS ANTONIO SALAZAR ESPINOSA</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G32" t="n">
-        <v>-2313.19</v>
+        <v>1742.89</v>
       </c>
       <c r="H32" t="n">
-        <v>3524.19</v>
+        <v>0</v>
       </c>
       <c r="I32" t="n">
-        <v>1211</v>
+        <v>1742.89</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1706,16 +1706,16 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>43380.7</v>
+        <v>71981.92</v>
       </c>
       <c r="M32" t="n">
-        <v>43380.7</v>
+        <v>71981.92</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>118915</t>
+          <t>105696</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
+          <t>GABRIELA CASTAÐEDA SALAZAR</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1737,10 +1737,10 @@
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>0</v>
+        <v>1737.43</v>
       </c>
       <c r="I33" t="n">
-        <v>0</v>
+        <v>1737.43</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -1749,26 +1749,26 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>49113.6</v>
+        <v>91447.39999999999</v>
       </c>
       <c r="M33" t="n">
-        <v>49113.6</v>
+        <v>91447.39999999999</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>116795</t>
+          <t>118069</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>GERARDO DANIEL BARAJAS TORRES</t>
+          <t>MARIO IVAN ROMERO GONZALEZ</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1780,10 +1780,10 @@
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>0</v>
+        <v>1662.54</v>
       </c>
       <c r="I34" t="n">
-        <v>0</v>
+        <v>1662.54</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
@@ -1792,26 +1792,26 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>4796.14</v>
+        <v>40741.71</v>
       </c>
       <c r="M34" t="n">
-        <v>4796.14</v>
+        <v>40741.71</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1823,10 +1823,10 @@
         <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>0</v>
+        <v>1516.55</v>
       </c>
       <c r="I35" t="n">
-        <v>0</v>
+        <v>1516.55</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -1835,26 +1835,26 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>17269.74</v>
+        <v>0</v>
       </c>
       <c r="M35" t="n">
-        <v>17269.74</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>115404</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1863,13 +1863,13 @@
         <v>0</v>
       </c>
       <c r="G36" t="n">
-        <v>0</v>
+        <v>-2313.19</v>
       </c>
       <c r="H36" t="n">
-        <v>0</v>
+        <v>3524.19</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>1211</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
@@ -1878,16 +1878,16 @@
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>3487.19</v>
+        <v>43380.7</v>
       </c>
       <c r="M36" t="n">
-        <v>3487.19</v>
+        <v>43380.7</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>118915</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1921,16 +1921,16 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>1693.99</v>
+        <v>49113.6</v>
       </c>
       <c r="M37" t="n">
-        <v>1693.99</v>
+        <v>49113.6</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>116795</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>GERARDO DANIEL BARAJAS TORRES</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1964,26 +1964,26 @@
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>17425.73</v>
+        <v>4796.14</v>
       </c>
       <c r="M38" t="n">
-        <v>17425.73</v>
+        <v>4796.14</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>113450</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -2007,16 +2007,16 @@
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>18650.03</v>
+        <v>17269.74</v>
       </c>
       <c r="M39" t="n">
-        <v>18650.03</v>
+        <v>17269.74</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>111056</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>JORGE ANTONIO LUNA LARA</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2050,16 +2050,16 @@
         <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>67074.12</v>
+        <v>3487.19</v>
       </c>
       <c r="M40" t="n">
-        <v>67074.12</v>
+        <v>3487.19</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>110575</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>JOSE RENE DE ALBA MORALES</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2093,16 +2093,16 @@
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>14427.08</v>
+        <v>1693.99</v>
       </c>
       <c r="M41" t="n">
-        <v>14427.08</v>
+        <v>1693.99</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>106018</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>MIREYA LIZETTE TORRES GARCIA</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2136,16 +2136,16 @@
         <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>23106.58</v>
+        <v>17425.73</v>
       </c>
       <c r="M42" t="n">
-        <v>23106.58</v>
+        <v>17425.73</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>104343</t>
+          <t>113450</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
+          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -2179,16 +2179,16 @@
         <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>12811.03</v>
+        <v>18650.03</v>
       </c>
       <c r="M43" t="n">
-        <v>12811.03</v>
+        <v>18650.03</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>103982</t>
+          <t>111056</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2198,7 +2198,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA RIOS BERNAL</t>
+          <t>JORGE ANTONIO LUNA LARA</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -2222,16 +2222,16 @@
         <v>0</v>
       </c>
       <c r="L44" t="n">
-        <v>6060.86</v>
+        <v>67074.12</v>
       </c>
       <c r="M44" t="n">
-        <v>6060.86</v>
+        <v>67074.12</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>101640</t>
+          <t>110575</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2241,7 +2241,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>SAMUEL NUÐO RIVERA</t>
+          <t>JOSE RENE DE ALBA MORALES</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -2265,16 +2265,16 @@
         <v>0</v>
       </c>
       <c r="L45" t="n">
-        <v>3214.14</v>
+        <v>14427.08</v>
       </c>
       <c r="M45" t="n">
-        <v>3214.14</v>
+        <v>14427.08</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>95148</t>
+          <t>104343</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2284,7 +2284,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
+          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -2308,16 +2308,16 @@
         <v>0</v>
       </c>
       <c r="L46" t="n">
-        <v>56725.37</v>
+        <v>12811.03</v>
       </c>
       <c r="M46" t="n">
-        <v>56725.37</v>
+        <v>12811.03</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>90355</t>
+          <t>101640</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2327,7 +2327,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>DARINKA UREÐA CASILLAS</t>
+          <t>SAMUEL NUÐO RIVERA</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -2351,10 +2351,10 @@
         <v>0</v>
       </c>
       <c r="L47" t="n">
-        <v>86129.07000000001</v>
+        <v>3214.14</v>
       </c>
       <c r="M47" t="n">
-        <v>86129.07000000001</v>
+        <v>3214.14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-09-23)
Incluye campañas (Camino a la Cumbre, MDRT, Graduación, Educar es Creer,
El Poder de Elegirte, Convención Asesores) y reportes admin (Proactivos,
Asesores sin Emisión, Comparativo Vida, Pagado/Pendiente) con snapshot
corregido y notificaciones ya enviadas para ambos grupos.
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>17 de septiembre de 2026</t>
+          <t>22 de septiembre de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -468,50 +468,50 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>110453</t>
+          <t>104750</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ANAIS LUA MORENO</t>
+          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G4" t="n">
-        <v>29655.2</v>
+        <v>134134.05</v>
       </c>
       <c r="H4" t="n">
-        <v>19128.87</v>
+        <v>5442.15</v>
       </c>
       <c r="I4" t="n">
-        <v>48784.07</v>
+        <v>139576.2</v>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>35695.85</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>82233.07000000001</v>
+        <v>35695.8</v>
       </c>
       <c r="M4" t="n">
-        <v>117928.92</v>
+        <v>35695.8</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>115047</t>
+          <t>110453</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -521,22 +521,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>VELIA PATRICIA BERNAL RAMOS</t>
+          <t>ANAIS LUA MORENO</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G5" t="n">
-        <v>39037.05</v>
+        <v>31348.75</v>
       </c>
       <c r="H5" t="n">
-        <v>6821.96</v>
+        <v>53131.17</v>
       </c>
       <c r="I5" t="n">
-        <v>45859.01</v>
+        <v>84479.92</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -545,16 +545,16 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>19745.09</v>
+        <v>82233.07000000001</v>
       </c>
       <c r="M5" t="n">
-        <v>19745.09</v>
+        <v>82233.07000000001</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>104750</t>
+          <t>87538</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -564,7 +564,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
+          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -573,13 +573,13 @@
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>37215.83</v>
+        <v>6853.85</v>
       </c>
       <c r="H6" t="n">
-        <v>5442.15</v>
+        <v>76663.98</v>
       </c>
       <c r="I6" t="n">
-        <v>42657.98</v>
+        <v>83517.83</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -588,16 +588,16 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>35695.8</v>
+        <v>166964.16</v>
       </c>
       <c r="M6" t="n">
-        <v>35695.8</v>
+        <v>166964.16</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>116883</t>
+          <t>115047</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -607,22 +607,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>SOFIA CAMPILLO VASCONCELOS</t>
+          <t>VELIA PATRICIA BERNAL RAMOS</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>39037.05</v>
       </c>
       <c r="H7" t="n">
-        <v>20796.52</v>
+        <v>6821.96</v>
       </c>
       <c r="I7" t="n">
-        <v>20796.52</v>
+        <v>45859.01</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -631,16 +631,16 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>88707.11</v>
+        <v>19745.09</v>
       </c>
       <c r="M7" t="n">
-        <v>88707.11</v>
+        <v>19745.09</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>87538</t>
+          <t>80122</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -650,34 +650,34 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
+          <t>DESIREE DE LA PEÐA OROZCO</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" t="n">
+        <v>7045.66</v>
+      </c>
+      <c r="H8" t="n">
+        <v>24936.66</v>
+      </c>
+      <c r="I8" t="n">
+        <v>31982.32</v>
+      </c>
+      <c r="J8" t="n">
         <v>1</v>
       </c>
-      <c r="G8" t="n">
-        <v>6853.85</v>
-      </c>
-      <c r="H8" t="n">
-        <v>12121.29</v>
-      </c>
-      <c r="I8" t="n">
-        <v>18975.14</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0</v>
-      </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>72893.8</v>
       </c>
       <c r="L8" t="n">
-        <v>231506.85</v>
+        <v>137881.24</v>
       </c>
       <c r="M8" t="n">
-        <v>231506.85</v>
+        <v>210775.04</v>
       </c>
     </row>
     <row r="9">
@@ -705,38 +705,38 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>18318.58</v>
+        <v>21193.35</v>
       </c>
       <c r="I9" t="n">
-        <v>18318.58</v>
+        <v>21193.35</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>17672.07</v>
       </c>
       <c r="L9" t="n">
-        <v>16324.8</v>
+        <v>13450.01</v>
       </c>
       <c r="M9" t="n">
-        <v>16324.8</v>
+        <v>31122.08</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>116883</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>SOFIA CAMPILLO VASCONCELOS</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -748,10 +748,10 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>12261.72</v>
+        <v>20796.52</v>
       </c>
       <c r="I10" t="n">
-        <v>12261.72</v>
+        <v>20796.52</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -760,16 +760,16 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>0</v>
+        <v>88707.11</v>
       </c>
       <c r="M10" t="n">
-        <v>0</v>
+        <v>88707.11</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>117440</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MONSERRAT VELASCO SANTOS</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -791,10 +791,10 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>12218.55</v>
+        <v>20509.75</v>
       </c>
       <c r="I11" t="n">
-        <v>12218.55</v>
+        <v>20509.75</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -803,16 +803,16 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>62871.21</v>
+        <v>7492.65</v>
       </c>
       <c r="M11" t="n">
-        <v>62871.21</v>
+        <v>7492.65</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>119223</t>
+          <t>117440</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -822,22 +822,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>OSCAR RAMIREZ RUIZ</t>
+          <t>MONSERRAT VELASCO SANTOS</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>12054.68</v>
+        <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>15217.64</v>
       </c>
       <c r="I12" t="n">
-        <v>12054.68</v>
+        <v>15217.64</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -846,16 +846,16 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>38468.95</v>
+        <v>59872.08</v>
       </c>
       <c r="M12" t="n">
-        <v>38468.95</v>
+        <v>59872.08</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>88234</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -865,7 +865,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -877,10 +877,10 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>8492.07</v>
+        <v>14591.69</v>
       </c>
       <c r="I13" t="n">
-        <v>8492.07</v>
+        <v>14591.69</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -889,16 +889,16 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>3845.25</v>
+        <v>5738.18</v>
       </c>
       <c r="M13" t="n">
-        <v>3845.25</v>
+        <v>5738.18</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>80122</t>
+          <t>119223</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -908,40 +908,40 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>DESIREE DE LA PEÐA OROZCO</t>
+          <t>OSCAR RAMIREZ RUIZ</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G14" t="n">
-        <v>0</v>
+        <v>12054.68</v>
       </c>
       <c r="H14" t="n">
-        <v>8390.049999999999</v>
+        <v>2401.3</v>
       </c>
       <c r="I14" t="n">
-        <v>8390.049999999999</v>
+        <v>14455.98</v>
       </c>
       <c r="J14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>72893.8</v>
+        <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>75998.97</v>
+        <v>36067.65</v>
       </c>
       <c r="M14" t="n">
-        <v>148892.77</v>
+        <v>36067.65</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -963,10 +963,10 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>7624.07</v>
+        <v>12261.72</v>
       </c>
       <c r="I15" t="n">
-        <v>7624.07</v>
+        <v>12261.72</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -975,16 +975,16 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>12705.8</v>
+        <v>0</v>
       </c>
       <c r="M15" t="n">
-        <v>12705.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>47116</t>
+          <t>105696</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
+          <t>GABRIELA CASTAÐEDA SALAZAR</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1006,28 +1006,28 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>6968.21</v>
+        <v>10691.34</v>
       </c>
       <c r="I16" t="n">
-        <v>6968.21</v>
+        <v>10691.34</v>
       </c>
       <c r="J16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>59086.36</v>
       </c>
       <c r="L16" t="n">
-        <v>47121.66</v>
+        <v>82953.16</v>
       </c>
       <c r="M16" t="n">
-        <v>47121.66</v>
+        <v>142039.52</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>108405</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1037,40 +1037,40 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>1203.25</v>
+        <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>4925.15</v>
+        <v>9124.58</v>
       </c>
       <c r="I17" t="n">
-        <v>6128.4</v>
+        <v>9124.58</v>
       </c>
       <c r="J17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>29652.91</v>
+        <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>31449.72</v>
+        <v>0</v>
       </c>
       <c r="M17" t="n">
-        <v>61102.63</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>103982</t>
+          <t>88234</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1080,7 +1080,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA RIOS BERNAL</t>
+          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1092,10 +1092,10 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>6060.91</v>
+        <v>8492.07</v>
       </c>
       <c r="I18" t="n">
-        <v>6060.91</v>
+        <v>8492.07</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1104,16 +1104,16 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>0</v>
+        <v>3845.25</v>
       </c>
       <c r="M18" t="n">
-        <v>0</v>
+        <v>3845.25</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>106018</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>MIREYA LIZETTE TORRES GARCIA</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>5431.4</v>
+        <v>7955.43</v>
       </c>
       <c r="I19" t="n">
-        <v>5431.4</v>
+        <v>7955.43</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1147,16 +1147,16 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>12899.71</v>
+        <v>15958.78</v>
       </c>
       <c r="M19" t="n">
-        <v>12899.71</v>
+        <v>15958.78</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>94156</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1166,50 +1166,50 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>MARIA TERESA ASENCIO LOZANO</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G20" t="n">
-        <v>0</v>
+        <v>1203.25</v>
       </c>
       <c r="H20" t="n">
-        <v>4709.73</v>
+        <v>6686.19</v>
       </c>
       <c r="I20" t="n">
-        <v>4709.73</v>
+        <v>7889.44</v>
       </c>
       <c r="J20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K20" t="n">
-        <v>0</v>
+        <v>29652.91</v>
       </c>
       <c r="L20" t="n">
-        <v>2309.36</v>
+        <v>33210.76</v>
       </c>
       <c r="M20" t="n">
-        <v>2309.36</v>
+        <v>62863.67</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>114100</t>
+          <t>94156</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
+          <t>MARIA TERESA ASENCIO LOZANO</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1221,10 +1221,10 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>3961.9</v>
+        <v>7019.13</v>
       </c>
       <c r="I21" t="n">
-        <v>3961.9</v>
+        <v>7019.13</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -1233,16 +1233,16 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>6410.16</v>
+        <v>0</v>
       </c>
       <c r="M21" t="n">
-        <v>6410.16</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>95148</t>
+          <t>47116</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
+          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -1264,10 +1264,10 @@
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>3898.73</v>
+        <v>6968.21</v>
       </c>
       <c r="I22" t="n">
-        <v>3898.73</v>
+        <v>6968.21</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1276,41 +1276,41 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>52826.69</v>
+        <v>45397.15</v>
       </c>
       <c r="M22" t="n">
-        <v>52826.69</v>
+        <v>45397.15</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>119447</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>LUIS ANTONIO SALAZAR ESPINOSA</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G23" t="n">
-        <v>0</v>
+        <v>1742.89</v>
       </c>
       <c r="H23" t="n">
-        <v>3041.47</v>
+        <v>4800.92</v>
       </c>
       <c r="I23" t="n">
-        <v>3041.47</v>
+        <v>6543.81</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -1319,26 +1319,26 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>0</v>
+        <v>67181</v>
       </c>
       <c r="M23" t="n">
-        <v>0</v>
+        <v>67181</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>109998</t>
+          <t>114100</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
+          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1350,10 +1350,10 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>2966.58</v>
+        <v>6098.62</v>
       </c>
       <c r="I24" t="n">
-        <v>2966.58</v>
+        <v>6098.62</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
@@ -1362,41 +1362,41 @@
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>0</v>
+        <v>4273.44</v>
       </c>
       <c r="M24" t="n">
-        <v>0</v>
+        <v>4273.44</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>120051</t>
+          <t>111056</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>GUILLERMO JOSE RAMIREZ RAMIREZ</t>
+          <t>JORGE ANTONIO LUNA LARA</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>2488.17</v>
+        <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>0</v>
+        <v>6097.65</v>
       </c>
       <c r="I25" t="n">
-        <v>2488.17</v>
+        <v>6097.65</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -1405,16 +1405,16 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>27369.85</v>
+        <v>60976.47</v>
       </c>
       <c r="M25" t="n">
-        <v>27369.85</v>
+        <v>60976.47</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>90355</t>
+          <t>103982</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>DARINKA UREÐA CASILLAS</t>
+          <t>MARIA FERNANDA RIOS BERNAL</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1436,10 +1436,10 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>2362.88</v>
+        <v>6060.91</v>
       </c>
       <c r="I26" t="n">
-        <v>2362.88</v>
+        <v>6060.91</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1448,16 +1448,16 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>83766.14999999999</v>
+        <v>0</v>
       </c>
       <c r="M26" t="n">
-        <v>83766.14999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>118246</t>
+          <t>95148</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>JOSE ANTEMIO OLIVA SANTOS</t>
+          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1479,10 +1479,10 @@
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>1967.73</v>
+        <v>5686.91</v>
       </c>
       <c r="I27" t="n">
-        <v>1967.73</v>
+        <v>5686.91</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
@@ -1491,16 +1491,16 @@
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>23551.39</v>
+        <v>51038.52</v>
       </c>
       <c r="M27" t="n">
-        <v>23551.39</v>
+        <v>51038.52</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>109998</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1510,7 +1510,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1522,10 +1522,10 @@
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>1800.77</v>
+        <v>2966.58</v>
       </c>
       <c r="I28" t="n">
-        <v>1800.77</v>
+        <v>2966.58</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -1534,16 +1534,16 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>10804.65</v>
+        <v>0</v>
       </c>
       <c r="M28" t="n">
-        <v>10804.65</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>106018</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>MIREYA LIZETTE TORRES GARCIA</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1565,10 +1565,10 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>1773.2</v>
+        <v>2513.54</v>
       </c>
       <c r="I29" t="n">
-        <v>1773.2</v>
+        <v>2513.54</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -1577,41 +1577,41 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>21333.38</v>
+        <v>3062.5</v>
       </c>
       <c r="M29" t="n">
-        <v>21333.38</v>
+        <v>3062.5</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>120051</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>GUILLERMO JOSE RAMIREZ RAMIREZ</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G30" t="n">
-        <v>0</v>
+        <v>2488.17</v>
       </c>
       <c r="H30" t="n">
-        <v>1761.04</v>
+        <v>0</v>
       </c>
       <c r="I30" t="n">
-        <v>1761.04</v>
+        <v>2488.17</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1620,16 +1620,16 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>7337.05</v>
+        <v>27369.85</v>
       </c>
       <c r="M30" t="n">
-        <v>7337.05</v>
+        <v>27369.85</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>65046</t>
+          <t>90355</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+          <t>DARINKA UREÐA CASILLAS</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1651,10 +1651,10 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>1747.29</v>
+        <v>2362.88</v>
       </c>
       <c r="I31" t="n">
-        <v>1747.29</v>
+        <v>2362.88</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1663,41 +1663,41 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>3494.59</v>
+        <v>83766.14999999999</v>
       </c>
       <c r="M31" t="n">
-        <v>3494.59</v>
+        <v>83766.14999999999</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>119447</t>
+          <t>113450</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>LUIS ANTONIO SALAZAR ESPINOSA</t>
+          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G32" t="n">
-        <v>1742.89</v>
+        <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>0</v>
+        <v>2072.23</v>
       </c>
       <c r="I32" t="n">
-        <v>1742.89</v>
+        <v>2072.23</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1706,16 +1706,16 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>71981.92</v>
+        <v>16577.8</v>
       </c>
       <c r="M32" t="n">
-        <v>71981.92</v>
+        <v>16577.8</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>105696</t>
+          <t>118246</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>GABRIELA CASTAÐEDA SALAZAR</t>
+          <t>JOSE ANTEMIO OLIVA SANTOS</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1737,10 +1737,10 @@
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>1737.43</v>
+        <v>1967.73</v>
       </c>
       <c r="I33" t="n">
-        <v>1737.43</v>
+        <v>1967.73</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -1749,26 +1749,26 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>91447.39999999999</v>
+        <v>23551.39</v>
       </c>
       <c r="M33" t="n">
-        <v>91447.39999999999</v>
+        <v>23551.39</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>118069</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>MARIO IVAN ROMERO GONZALEZ</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1780,10 +1780,10 @@
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>1662.54</v>
+        <v>1800.77</v>
       </c>
       <c r="I34" t="n">
-        <v>1662.54</v>
+        <v>1800.77</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
@@ -1792,26 +1792,26 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>40741.71</v>
+        <v>10804.65</v>
       </c>
       <c r="M34" t="n">
-        <v>40741.71</v>
+        <v>10804.65</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1823,10 +1823,10 @@
         <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>1516.55</v>
+        <v>1781.04</v>
       </c>
       <c r="I35" t="n">
-        <v>1516.55</v>
+        <v>1781.04</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -1835,26 +1835,26 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>0</v>
+        <v>15488.7</v>
       </c>
       <c r="M35" t="n">
-        <v>0</v>
+        <v>15488.7</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>65046</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1863,13 +1863,13 @@
         <v>0</v>
       </c>
       <c r="G36" t="n">
-        <v>-2313.19</v>
+        <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>3524.19</v>
+        <v>1747.29</v>
       </c>
       <c r="I36" t="n">
-        <v>1211</v>
+        <v>1747.29</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
@@ -1878,26 +1878,26 @@
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>43380.7</v>
+        <v>3494.59</v>
       </c>
       <c r="M36" t="n">
-        <v>43380.7</v>
+        <v>3494.59</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>118915</t>
+          <t>118069</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
+          <t>MARIO IVAN ROMERO GONZALEZ</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1909,10 +1909,10 @@
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>0</v>
+        <v>1662.54</v>
       </c>
       <c r="I37" t="n">
-        <v>0</v>
+        <v>1662.54</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -1921,10 +1921,10 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>49113.6</v>
+        <v>40741.71</v>
       </c>
       <c r="M37" t="n">
-        <v>49113.6</v>
+        <v>40741.71</v>
       </c>
     </row>
     <row r="38">
@@ -1952,10 +1952,10 @@
         <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>0</v>
+        <v>1598.75</v>
       </c>
       <c r="I38" t="n">
-        <v>0</v>
+        <v>1598.75</v>
       </c>
       <c r="J38" t="n">
         <v>0</v>
@@ -1964,26 +1964,26 @@
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>4796.14</v>
+        <v>0</v>
       </c>
       <c r="M38" t="n">
-        <v>4796.14</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1995,10 +1995,10 @@
         <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>0</v>
+        <v>1516.55</v>
       </c>
       <c r="I39" t="n">
-        <v>0</v>
+        <v>1516.55</v>
       </c>
       <c r="J39" t="n">
         <v>0</v>
@@ -2007,26 +2007,26 @@
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>17269.74</v>
+        <v>0</v>
       </c>
       <c r="M39" t="n">
-        <v>17269.74</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>115404</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2035,13 +2035,13 @@
         <v>0</v>
       </c>
       <c r="G40" t="n">
-        <v>0</v>
+        <v>-2313.19</v>
       </c>
       <c r="H40" t="n">
-        <v>0</v>
+        <v>3524.19</v>
       </c>
       <c r="I40" t="n">
-        <v>0</v>
+        <v>1211</v>
       </c>
       <c r="J40" t="n">
         <v>0</v>
@@ -2050,16 +2050,16 @@
         <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>3487.19</v>
+        <v>43380.7</v>
       </c>
       <c r="M40" t="n">
-        <v>3487.19</v>
+        <v>43380.7</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>118915</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2093,16 +2093,16 @@
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>1693.99</v>
+        <v>49113.6</v>
       </c>
       <c r="M41" t="n">
-        <v>1693.99</v>
+        <v>49113.6</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2136,16 +2136,16 @@
         <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>17425.73</v>
+        <v>3487.19</v>
       </c>
       <c r="M42" t="n">
-        <v>17425.73</v>
+        <v>3487.19</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>113450</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -2179,16 +2179,16 @@
         <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>18650.03</v>
+        <v>1693.99</v>
       </c>
       <c r="M43" t="n">
-        <v>18650.03</v>
+        <v>1693.99</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>111056</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2198,7 +2198,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>JORGE ANTONIO LUNA LARA</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -2222,10 +2222,10 @@
         <v>0</v>
       </c>
       <c r="L44" t="n">
-        <v>67074.12</v>
+        <v>17425.73</v>
       </c>
       <c r="M44" t="n">
-        <v>67074.12</v>
+        <v>17425.73</v>
       </c>
     </row>
     <row r="45">

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-09-29 10:51)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>22 de septiembre de 2026</t>
+          <t>25 de septiembre de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -490,10 +490,10 @@
         <v>134134.05</v>
       </c>
       <c r="H4" t="n">
-        <v>5442.15</v>
+        <v>7177.82</v>
       </c>
       <c r="I4" t="n">
-        <v>139576.2</v>
+        <v>141311.87</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -502,84 +502,84 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>35695.8</v>
+        <v>30697.04</v>
       </c>
       <c r="M4" t="n">
-        <v>35695.8</v>
+        <v>30697.04</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>110453</t>
+          <t>87538</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ANAIS LUA MORENO</t>
+          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>31348.75</v>
+        <v>6853.85</v>
       </c>
       <c r="H5" t="n">
-        <v>53131.17</v>
+        <v>92281.44</v>
       </c>
       <c r="I5" t="n">
-        <v>84479.92</v>
+        <v>99135.28999999999</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>59479.39</v>
       </c>
       <c r="L5" t="n">
-        <v>82233.07000000001</v>
+        <v>151566.93</v>
       </c>
       <c r="M5" t="n">
-        <v>82233.07000000001</v>
+        <v>211046.32</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>87538</t>
+          <t>110453</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
+          <t>ANAIS LUA MORENO</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G6" t="n">
-        <v>6853.85</v>
+        <v>31348.75</v>
       </c>
       <c r="H6" t="n">
-        <v>76663.98</v>
+        <v>55094.76</v>
       </c>
       <c r="I6" t="n">
-        <v>83517.83</v>
+        <v>86443.50999999999</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -588,10 +588,10 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>166964.16</v>
+        <v>80269.48</v>
       </c>
       <c r="M6" t="n">
-        <v>166964.16</v>
+        <v>80269.48</v>
       </c>
     </row>
     <row r="7">
@@ -619,10 +619,10 @@
         <v>39037.05</v>
       </c>
       <c r="H7" t="n">
-        <v>6821.96</v>
+        <v>8614.280000000001</v>
       </c>
       <c r="I7" t="n">
-        <v>45859.01</v>
+        <v>47651.33</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -631,16 +631,16 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>19745.09</v>
+        <v>17952.77</v>
       </c>
       <c r="M7" t="n">
-        <v>19745.09</v>
+        <v>17952.77</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>80122</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -650,7 +650,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>DESIREE DE LA PEÐA OROZCO</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -659,31 +659,31 @@
         <v>2</v>
       </c>
       <c r="G8" t="n">
-        <v>7045.66</v>
+        <v>30856.16</v>
       </c>
       <c r="H8" t="n">
-        <v>24936.66</v>
+        <v>6686.19</v>
       </c>
       <c r="I8" t="n">
-        <v>31982.32</v>
+        <v>37542.35</v>
       </c>
       <c r="J8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>72893.8</v>
+        <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>137881.24</v>
+        <v>33210.76</v>
       </c>
       <c r="M8" t="n">
-        <v>210775.04</v>
+        <v>33210.76</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>104718</t>
+          <t>80122</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -693,50 +693,50 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ROGELIO TORRES ORTIZ</t>
+          <t>DESIREE DE LA PEÐA OROZCO</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>7045.66</v>
       </c>
       <c r="H9" t="n">
-        <v>21193.35</v>
+        <v>24936.66</v>
       </c>
       <c r="I9" t="n">
-        <v>21193.35</v>
+        <v>31982.32</v>
       </c>
       <c r="J9" t="n">
         <v>1</v>
       </c>
       <c r="K9" t="n">
-        <v>17672.07</v>
+        <v>72893.8</v>
       </c>
       <c r="L9" t="n">
-        <v>13450.01</v>
+        <v>137881.24</v>
       </c>
       <c r="M9" t="n">
-        <v>31122.08</v>
+        <v>210775.04</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>116883</t>
+          <t>104718</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>SOFIA CAMPILLO VASCONCELOS</t>
+          <t>ROGELIO TORRES ORTIZ</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -748,38 +748,38 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>20796.52</v>
+        <v>23664.87</v>
       </c>
       <c r="I10" t="n">
-        <v>20796.52</v>
+        <v>23664.87</v>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>17672.07</v>
       </c>
       <c r="L10" t="n">
-        <v>88707.11</v>
+        <v>10978.48</v>
       </c>
       <c r="M10" t="n">
-        <v>88707.11</v>
+        <v>28650.55</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>116883</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>SOFIA CAMPILLO VASCONCELOS</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -791,10 +791,10 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>20509.75</v>
+        <v>20796.52</v>
       </c>
       <c r="I11" t="n">
-        <v>20509.75</v>
+        <v>20796.52</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -803,16 +803,16 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>7492.65</v>
+        <v>88707.11</v>
       </c>
       <c r="M11" t="n">
-        <v>7492.65</v>
+        <v>88707.11</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>117440</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -822,7 +822,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MONSERRAT VELASCO SANTOS</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -834,10 +834,10 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>15217.64</v>
+        <v>20509.75</v>
       </c>
       <c r="I12" t="n">
-        <v>15217.64</v>
+        <v>20509.75</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -846,10 +846,10 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>59872.08</v>
+        <v>7492.65</v>
       </c>
       <c r="M12" t="n">
-        <v>59872.08</v>
+        <v>7492.65</v>
       </c>
     </row>
     <row r="13">
@@ -877,10 +877,10 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>14591.69</v>
+        <v>16856.07</v>
       </c>
       <c r="I13" t="n">
-        <v>14591.69</v>
+        <v>16856.07</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -889,16 +889,16 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>5738.18</v>
+        <v>3473.8</v>
       </c>
       <c r="M13" t="n">
-        <v>5738.18</v>
+        <v>3473.8</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>119223</t>
+          <t>118915</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -908,22 +908,22 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>OSCAR RAMIREZ RUIZ</t>
+          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>12054.68</v>
+        <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>2401.3</v>
+        <v>16371.2</v>
       </c>
       <c r="I14" t="n">
-        <v>14455.98</v>
+        <v>16371.2</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -932,16 +932,16 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>36067.65</v>
+        <v>32742.4</v>
       </c>
       <c r="M14" t="n">
-        <v>36067.65</v>
+        <v>32742.4</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>117440</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>MONSERRAT VELASCO SANTOS</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -963,28 +963,28 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>12261.72</v>
+        <v>15217.64</v>
       </c>
       <c r="I15" t="n">
-        <v>12261.72</v>
+        <v>15217.64</v>
       </c>
       <c r="J15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>2384.03</v>
       </c>
       <c r="L15" t="n">
-        <v>0</v>
+        <v>86096.39</v>
       </c>
       <c r="M15" t="n">
-        <v>0</v>
+        <v>88480.42</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>105696</t>
+          <t>119223</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -994,40 +994,40 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>GABRIELA CASTAÐEDA SALAZAR</t>
+          <t>OSCAR RAMIREZ RUIZ</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G16" t="n">
-        <v>0</v>
+        <v>12054.68</v>
       </c>
       <c r="H16" t="n">
-        <v>10691.34</v>
+        <v>2401.3</v>
       </c>
       <c r="I16" t="n">
-        <v>10691.34</v>
+        <v>14455.98</v>
       </c>
       <c r="J16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>59086.36</v>
+        <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>82953.16</v>
+        <v>36067.65</v>
       </c>
       <c r="M16" t="n">
-        <v>142039.52</v>
+        <v>36067.65</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>90355</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>DARINKA UREÐA CASILLAS</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1049,10 +1049,10 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>9124.58</v>
+        <v>12509.74</v>
       </c>
       <c r="I17" t="n">
-        <v>9124.58</v>
+        <v>12509.74</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1061,16 +1061,16 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>0</v>
+        <v>76989.35000000001</v>
       </c>
       <c r="M17" t="n">
-        <v>0</v>
+        <v>76989.35000000001</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>88234</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1080,7 +1080,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1092,10 +1092,10 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>8492.07</v>
+        <v>12261.72</v>
       </c>
       <c r="I18" t="n">
-        <v>8492.07</v>
+        <v>12261.72</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1104,16 +1104,16 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>3845.25</v>
+        <v>0</v>
       </c>
       <c r="M18" t="n">
-        <v>3845.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>106018</t>
+          <t>105696</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MIREYA LIZETTE TORRES GARCIA</t>
+          <t>GABRIELA CASTAÐEDA SALAZAR</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -1135,28 +1135,28 @@
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>7955.43</v>
+        <v>10691.34</v>
       </c>
       <c r="I19" t="n">
-        <v>7955.43</v>
+        <v>10691.34</v>
       </c>
       <c r="J19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K19" t="n">
-        <v>0</v>
+        <v>59086.36</v>
       </c>
       <c r="L19" t="n">
-        <v>15958.78</v>
+        <v>82953.16</v>
       </c>
       <c r="M19" t="n">
-        <v>15958.78</v>
+        <v>142039.52</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>108405</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1166,40 +1166,40 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>1203.25</v>
+        <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>6686.19</v>
+        <v>9124.58</v>
       </c>
       <c r="I20" t="n">
-        <v>7889.44</v>
+        <v>9124.58</v>
       </c>
       <c r="J20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K20" t="n">
-        <v>29652.91</v>
+        <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>33210.76</v>
+        <v>0</v>
       </c>
       <c r="M20" t="n">
-        <v>62863.67</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>94156</t>
+          <t>88234</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>MARIA TERESA ASENCIO LOZANO</t>
+          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1221,10 +1221,10 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>7019.13</v>
+        <v>8492.07</v>
       </c>
       <c r="I21" t="n">
-        <v>7019.13</v>
+        <v>8492.07</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -1233,16 +1233,16 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>0</v>
+        <v>3845.25</v>
       </c>
       <c r="M21" t="n">
-        <v>0</v>
+        <v>3845.25</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>47116</t>
+          <t>106018</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
+          <t>MIREYA LIZETTE TORRES GARCIA</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -1264,10 +1264,10 @@
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>6968.21</v>
+        <v>7955.43</v>
       </c>
       <c r="I22" t="n">
-        <v>6968.21</v>
+        <v>7955.43</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1276,41 +1276,41 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>45397.15</v>
+        <v>15958.78</v>
       </c>
       <c r="M22" t="n">
-        <v>45397.15</v>
+        <v>15958.78</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>119447</t>
+          <t>94156</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>LUIS ANTONIO SALAZAR ESPINOSA</t>
+          <t>MARIA TERESA ASENCIO LOZANO</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>1742.89</v>
+        <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>4800.92</v>
+        <v>7019.13</v>
       </c>
       <c r="I23" t="n">
-        <v>6543.81</v>
+        <v>7019.13</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -1319,26 +1319,26 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>67181</v>
+        <v>0</v>
       </c>
       <c r="M23" t="n">
-        <v>67181</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>114100</t>
+          <t>47116</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
+          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1350,10 +1350,10 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>6098.62</v>
+        <v>6968.21</v>
       </c>
       <c r="I24" t="n">
-        <v>6098.62</v>
+        <v>6968.21</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
@@ -1362,41 +1362,41 @@
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>4273.44</v>
+        <v>45397.15</v>
       </c>
       <c r="M24" t="n">
-        <v>4273.44</v>
+        <v>45397.15</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>111056</t>
+          <t>119447</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>JORGE ANTONIO LUNA LARA</t>
+          <t>LUIS ANTONIO SALAZAR ESPINOSA</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G25" t="n">
-        <v>0</v>
+        <v>1742.89</v>
       </c>
       <c r="H25" t="n">
-        <v>6097.65</v>
+        <v>4800.92</v>
       </c>
       <c r="I25" t="n">
-        <v>6097.65</v>
+        <v>6543.81</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -1405,26 +1405,26 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>60976.47</v>
+        <v>67181</v>
       </c>
       <c r="M25" t="n">
-        <v>60976.47</v>
+        <v>67181</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>103982</t>
+          <t>114100</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA RIOS BERNAL</t>
+          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1436,10 +1436,10 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>6060.91</v>
+        <v>6098.62</v>
       </c>
       <c r="I26" t="n">
-        <v>6060.91</v>
+        <v>6098.62</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1448,16 +1448,16 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>0</v>
+        <v>4273.44</v>
       </c>
       <c r="M26" t="n">
-        <v>0</v>
+        <v>4273.44</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>95148</t>
+          <t>111056</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
+          <t>JORGE ANTONIO LUNA LARA</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1479,10 +1479,10 @@
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>5686.91</v>
+        <v>6097.65</v>
       </c>
       <c r="I27" t="n">
-        <v>5686.91</v>
+        <v>6097.65</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
@@ -1491,16 +1491,16 @@
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>51038.52</v>
+        <v>60976.47</v>
       </c>
       <c r="M27" t="n">
-        <v>51038.52</v>
+        <v>60976.47</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>109998</t>
+          <t>103982</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1510,7 +1510,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
+          <t>MARIA FERNANDA RIOS BERNAL</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1522,10 +1522,10 @@
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>2966.58</v>
+        <v>6060.91</v>
       </c>
       <c r="I28" t="n">
-        <v>2966.58</v>
+        <v>6060.91</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -1543,7 +1543,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>95148</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1565,10 +1565,10 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>2513.54</v>
+        <v>5686.91</v>
       </c>
       <c r="I29" t="n">
-        <v>2513.54</v>
+        <v>5686.91</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -1577,41 +1577,41 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>3062.5</v>
+        <v>51038.52</v>
       </c>
       <c r="M29" t="n">
-        <v>3062.5</v>
+        <v>51038.52</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>120051</t>
+          <t>109998</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>GUILLERMO JOSE RAMIREZ RAMIREZ</t>
+          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G30" t="n">
-        <v>2488.17</v>
+        <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>0</v>
+        <v>2966.58</v>
       </c>
       <c r="I30" t="n">
-        <v>2488.17</v>
+        <v>2966.58</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1620,16 +1620,16 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>27369.85</v>
+        <v>0</v>
       </c>
       <c r="M30" t="n">
-        <v>27369.85</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>90355</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>DARINKA UREÐA CASILLAS</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1651,10 +1651,10 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>2362.88</v>
+        <v>2513.54</v>
       </c>
       <c r="I31" t="n">
-        <v>2362.88</v>
+        <v>2513.54</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1663,41 +1663,41 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>83766.14999999999</v>
+        <v>3062.5</v>
       </c>
       <c r="M31" t="n">
-        <v>83766.14999999999</v>
+        <v>3062.5</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>113450</t>
+          <t>120051</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
+          <t>GUILLERMO JOSE RAMIREZ RAMIREZ</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G32" t="n">
-        <v>0</v>
+        <v>2488.17</v>
       </c>
       <c r="H32" t="n">
-        <v>2072.23</v>
+        <v>0</v>
       </c>
       <c r="I32" t="n">
-        <v>2072.23</v>
+        <v>2488.17</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1706,16 +1706,16 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>16577.8</v>
+        <v>27369.85</v>
       </c>
       <c r="M32" t="n">
-        <v>16577.8</v>
+        <v>27369.85</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>118246</t>
+          <t>113450</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>JOSE ANTEMIO OLIVA SANTOS</t>
+          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1737,10 +1737,10 @@
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>1967.73</v>
+        <v>2072.23</v>
       </c>
       <c r="I33" t="n">
-        <v>1967.73</v>
+        <v>2072.23</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -1749,16 +1749,16 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>23551.39</v>
+        <v>16577.8</v>
       </c>
       <c r="M33" t="n">
-        <v>23551.39</v>
+        <v>16577.8</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>118246</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1768,7 +1768,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>JOSE ANTEMIO OLIVA SANTOS</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1780,10 +1780,10 @@
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>1800.77</v>
+        <v>1967.73</v>
       </c>
       <c r="I34" t="n">
-        <v>1800.77</v>
+        <v>1967.73</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
@@ -1792,26 +1792,26 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>10804.65</v>
+        <v>0</v>
       </c>
       <c r="M34" t="n">
-        <v>10804.65</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1823,10 +1823,10 @@
         <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>1781.04</v>
+        <v>1800.77</v>
       </c>
       <c r="I35" t="n">
-        <v>1781.04</v>
+        <v>1800.77</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -1835,26 +1835,26 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>15488.7</v>
+        <v>10804.65</v>
       </c>
       <c r="M35" t="n">
-        <v>15488.7</v>
+        <v>10804.65</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>65046</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1866,10 +1866,10 @@
         <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>1747.29</v>
+        <v>1781.04</v>
       </c>
       <c r="I36" t="n">
-        <v>1747.29</v>
+        <v>1781.04</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
@@ -1878,26 +1878,26 @@
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>3494.59</v>
+        <v>15488.7</v>
       </c>
       <c r="M36" t="n">
-        <v>3494.59</v>
+        <v>15488.7</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>118069</t>
+          <t>65046</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>MARIO IVAN ROMERO GONZALEZ</t>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1909,10 +1909,10 @@
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>1662.54</v>
+        <v>1747.29</v>
       </c>
       <c r="I37" t="n">
-        <v>1662.54</v>
+        <v>1747.29</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -1921,26 +1921,26 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>40741.71</v>
+        <v>3494.59</v>
       </c>
       <c r="M37" t="n">
-        <v>40741.71</v>
+        <v>3494.59</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>116795</t>
+          <t>118069</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>GERARDO DANIEL BARAJAS TORRES</t>
+          <t>MARIO IVAN ROMERO GONZALEZ</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1952,10 +1952,10 @@
         <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>1598.75</v>
+        <v>1662.54</v>
       </c>
       <c r="I38" t="n">
-        <v>1598.75</v>
+        <v>1662.54</v>
       </c>
       <c r="J38" t="n">
         <v>0</v>
@@ -1964,16 +1964,16 @@
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>0</v>
+        <v>40741.71</v>
       </c>
       <c r="M38" t="n">
-        <v>0</v>
+        <v>40741.71</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>116795</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>GERARDO DANIEL BARAJAS TORRES</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1995,10 +1995,10 @@
         <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>1516.55</v>
+        <v>1598.75</v>
       </c>
       <c r="I39" t="n">
-        <v>1516.55</v>
+        <v>1598.75</v>
       </c>
       <c r="J39" t="n">
         <v>0</v>
@@ -2016,17 +2016,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2035,13 +2035,13 @@
         <v>0</v>
       </c>
       <c r="G40" t="n">
-        <v>-2313.19</v>
+        <v>0</v>
       </c>
       <c r="H40" t="n">
-        <v>3524.19</v>
+        <v>1516.55</v>
       </c>
       <c r="I40" t="n">
-        <v>1211</v>
+        <v>1516.55</v>
       </c>
       <c r="J40" t="n">
         <v>0</v>
@@ -2050,26 +2050,26 @@
         <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>43380.7</v>
+        <v>0</v>
       </c>
       <c r="M40" t="n">
-        <v>43380.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>118915</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2078,13 +2078,13 @@
         <v>0</v>
       </c>
       <c r="G41" t="n">
-        <v>0</v>
+        <v>-2313.19</v>
       </c>
       <c r="H41" t="n">
-        <v>0</v>
+        <v>3524.19</v>
       </c>
       <c r="I41" t="n">
-        <v>0</v>
+        <v>1211</v>
       </c>
       <c r="J41" t="n">
         <v>0</v>
@@ -2093,10 +2093,10 @@
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>49113.6</v>
+        <v>43380.7</v>
       </c>
       <c r="M41" t="n">
-        <v>49113.6</v>
+        <v>43380.7</v>
       </c>
     </row>
     <row r="42">

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-09-30 13:08)
Primera corrida con el fix de pageSize=100 — Legión Centurión vuelve a
detectarse y actualizarse (28 de septiembre) después de semanas atorada
por el límite de la carpeta "Campañas" del portal.
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -413,13 +413,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M47"/>
+  <dimension ref="A1:M46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>25 de septiembre de 2026</t>
+          <t>29 de septiembre de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -468,7 +468,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>104750</t>
+          <t>87538</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -478,22 +478,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
+          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G4" t="n">
-        <v>134134.05</v>
+        <v>66333.24000000001</v>
       </c>
       <c r="H4" t="n">
-        <v>7177.82</v>
+        <v>99213.17</v>
       </c>
       <c r="I4" t="n">
-        <v>141311.87</v>
+        <v>165546.41</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -502,16 +502,16 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>30697.04</v>
+        <v>144635.2</v>
       </c>
       <c r="M4" t="n">
-        <v>30697.04</v>
+        <v>144635.2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>87538</t>
+          <t>104750</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -521,34 +521,34 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
+          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G5" t="n">
-        <v>6853.85</v>
+        <v>134134.05</v>
       </c>
       <c r="H5" t="n">
-        <v>92281.44</v>
+        <v>7177.82</v>
       </c>
       <c r="I5" t="n">
-        <v>99135.28999999999</v>
+        <v>141311.87</v>
       </c>
       <c r="J5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>59479.39</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>151566.93</v>
+        <v>30697.04</v>
       </c>
       <c r="M5" t="n">
-        <v>211046.32</v>
+        <v>30697.04</v>
       </c>
     </row>
     <row r="6">
@@ -576,10 +576,10 @@
         <v>31348.75</v>
       </c>
       <c r="H6" t="n">
-        <v>55094.76</v>
+        <v>57335.88</v>
       </c>
       <c r="I6" t="n">
-        <v>86443.50999999999</v>
+        <v>88684.63</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -588,10 +588,10 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>80269.48</v>
+        <v>78028.36</v>
       </c>
       <c r="M6" t="n">
-        <v>80269.48</v>
+        <v>78028.36</v>
       </c>
     </row>
     <row r="7">
@@ -640,7 +640,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>104718</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -650,22 +650,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>ROGELIO TORRES ORTIZ</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>30856.16</v>
+        <v>1606.94</v>
       </c>
       <c r="H8" t="n">
-        <v>6686.19</v>
+        <v>38540.14</v>
       </c>
       <c r="I8" t="n">
-        <v>37542.35</v>
+        <v>40147.08</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -674,16 +674,16 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>33210.76</v>
+        <v>10978.48</v>
       </c>
       <c r="M8" t="n">
-        <v>33210.76</v>
+        <v>10978.48</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>80122</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>DESIREE DE LA PEÐA OROZCO</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
@@ -702,117 +702,117 @@
         <v>2</v>
       </c>
       <c r="G9" t="n">
-        <v>7045.66</v>
+        <v>30856.16</v>
       </c>
       <c r="H9" t="n">
-        <v>24936.66</v>
+        <v>8648.110000000001</v>
       </c>
       <c r="I9" t="n">
-        <v>31982.32</v>
+        <v>39504.27</v>
       </c>
       <c r="J9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>72893.8</v>
+        <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>137881.24</v>
+        <v>31248.84</v>
       </c>
       <c r="M9" t="n">
-        <v>210775.04</v>
+        <v>31248.84</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>104718</t>
+          <t>119447</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ROGELIO TORRES ORTIZ</t>
+          <t>LUIS ANTONIO SALAZAR ESPINOSA</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>29059.35</v>
       </c>
       <c r="H10" t="n">
-        <v>23664.87</v>
+        <v>4800.92</v>
       </c>
       <c r="I10" t="n">
-        <v>23664.87</v>
+        <v>33860.27</v>
       </c>
       <c r="J10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>17672.07</v>
+        <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>10978.48</v>
+        <v>67181</v>
       </c>
       <c r="M10" t="n">
-        <v>28650.55</v>
+        <v>67181</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>116883</t>
+          <t>80122</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>SOFIA CAMPILLO VASCONCELOS</t>
+          <t>DESIREE DE LA PEÐA OROZCO</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>7045.66</v>
       </c>
       <c r="H11" t="n">
-        <v>20796.52</v>
+        <v>24936.66</v>
       </c>
       <c r="I11" t="n">
-        <v>20796.52</v>
+        <v>31982.32</v>
       </c>
       <c r="J11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>99962.16</v>
       </c>
       <c r="L11" t="n">
-        <v>88707.11</v>
+        <v>137881.24</v>
       </c>
       <c r="M11" t="n">
-        <v>88707.11</v>
+        <v>237843.4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>117440</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -822,22 +822,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>MONSERRAT VELASCO SANTOS</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>2384.03</v>
       </c>
       <c r="H12" t="n">
-        <v>20509.75</v>
+        <v>23106.28</v>
       </c>
       <c r="I12" t="n">
-        <v>20509.75</v>
+        <v>25490.31</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -846,26 +846,26 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>7492.65</v>
+        <v>80679.25999999999</v>
       </c>
       <c r="M12" t="n">
-        <v>7492.65</v>
+        <v>80679.25999999999</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>116883</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>SOFIA CAMPILLO VASCONCELOS</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -877,10 +877,10 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>16856.07</v>
+        <v>24632.7</v>
       </c>
       <c r="I13" t="n">
-        <v>16856.07</v>
+        <v>24632.7</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -889,16 +889,16 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>3473.8</v>
+        <v>84870.92999999999</v>
       </c>
       <c r="M13" t="n">
-        <v>3473.8</v>
+        <v>84870.92999999999</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>118915</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -920,10 +920,10 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>16371.2</v>
+        <v>20509.75</v>
       </c>
       <c r="I14" t="n">
-        <v>16371.2</v>
+        <v>20509.75</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -932,16 +932,16 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>32742.4</v>
+        <v>7492.65</v>
       </c>
       <c r="M14" t="n">
-        <v>32742.4</v>
+        <v>7492.65</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>117440</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MONSERRAT VELASCO SANTOS</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -963,28 +963,28 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>15217.64</v>
+        <v>16856.07</v>
       </c>
       <c r="I15" t="n">
-        <v>15217.64</v>
+        <v>16856.07</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>2384.03</v>
+        <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>86096.39</v>
+        <v>0</v>
       </c>
       <c r="M15" t="n">
-        <v>88480.42</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>119223</t>
+          <t>118915</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -994,22 +994,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>OSCAR RAMIREZ RUIZ</t>
+          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>12054.68</v>
+        <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>2401.3</v>
+        <v>16371.2</v>
       </c>
       <c r="I16" t="n">
-        <v>14455.98</v>
+        <v>16371.2</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1018,16 +1018,16 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>36067.65</v>
+        <v>32742.4</v>
       </c>
       <c r="M16" t="n">
-        <v>36067.65</v>
+        <v>32742.4</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>90355</t>
+          <t>119223</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1037,22 +1037,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>DARINKA UREÐA CASILLAS</t>
+          <t>OSCAR RAMIREZ RUIZ</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G17" t="n">
-        <v>0</v>
+        <v>12054.68</v>
       </c>
       <c r="H17" t="n">
-        <v>12509.74</v>
+        <v>2401.3</v>
       </c>
       <c r="I17" t="n">
-        <v>12509.74</v>
+        <v>14455.98</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1061,16 +1061,16 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>76989.35000000001</v>
+        <v>36067.65</v>
       </c>
       <c r="M17" t="n">
-        <v>76989.35000000001</v>
+        <v>36067.65</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>110575</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1080,7 +1080,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>JOSE RENE DE ALBA MORALES</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1092,10 +1092,10 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>12261.72</v>
+        <v>14427.08</v>
       </c>
       <c r="I18" t="n">
-        <v>12261.72</v>
+        <v>14427.08</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1135,28 +1135,28 @@
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>10691.34</v>
+        <v>12748.41</v>
       </c>
       <c r="I19" t="n">
-        <v>10691.34</v>
+        <v>12748.41</v>
       </c>
       <c r="J19" t="n">
         <v>2</v>
       </c>
       <c r="K19" t="n">
-        <v>59086.36</v>
+        <v>5179.68</v>
       </c>
       <c r="L19" t="n">
-        <v>82953.16</v>
+        <v>137872.6</v>
       </c>
       <c r="M19" t="n">
-        <v>142039.52</v>
+        <v>143052.28</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>90355</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>DARINKA UREÐA CASILLAS</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1178,10 +1178,10 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>9124.58</v>
+        <v>12509.74</v>
       </c>
       <c r="I20" t="n">
-        <v>9124.58</v>
+        <v>12509.74</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1190,16 +1190,16 @@
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>0</v>
+        <v>76989.35000000001</v>
       </c>
       <c r="M20" t="n">
-        <v>0</v>
+        <v>76989.35000000001</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>88234</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1221,10 +1221,10 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>8492.07</v>
+        <v>12261.72</v>
       </c>
       <c r="I21" t="n">
-        <v>8492.07</v>
+        <v>12261.72</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -1233,16 +1233,16 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>3845.25</v>
+        <v>0</v>
       </c>
       <c r="M21" t="n">
-        <v>3845.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>106018</t>
+          <t>108405</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>MIREYA LIZETTE TORRES GARCIA</t>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -1264,10 +1264,10 @@
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>7955.43</v>
+        <v>9124.58</v>
       </c>
       <c r="I22" t="n">
-        <v>7955.43</v>
+        <v>9124.58</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1276,16 +1276,16 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>15958.78</v>
+        <v>0</v>
       </c>
       <c r="M22" t="n">
-        <v>15958.78</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>94156</t>
+          <t>88234</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>MARIA TERESA ASENCIO LOZANO</t>
+          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -1307,10 +1307,10 @@
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>7019.13</v>
+        <v>8492.07</v>
       </c>
       <c r="I23" t="n">
-        <v>7019.13</v>
+        <v>8492.07</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -1319,16 +1319,16 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>0</v>
+        <v>3845.25</v>
       </c>
       <c r="M23" t="n">
-        <v>0</v>
+        <v>3845.25</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>47116</t>
+          <t>106018</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
+          <t>MIREYA LIZETTE TORRES GARCIA</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1350,10 +1350,10 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>6968.21</v>
+        <v>7955.43</v>
       </c>
       <c r="I24" t="n">
-        <v>6968.21</v>
+        <v>7955.43</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
@@ -1362,41 +1362,41 @@
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>45397.15</v>
+        <v>15958.78</v>
       </c>
       <c r="M24" t="n">
-        <v>45397.15</v>
+        <v>15958.78</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>119447</t>
+          <t>94156</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>LUIS ANTONIO SALAZAR ESPINOSA</t>
+          <t>MARIA TERESA ASENCIO LOZANO</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>1742.89</v>
+        <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>4800.92</v>
+        <v>7019.13</v>
       </c>
       <c r="I25" t="n">
-        <v>6543.81</v>
+        <v>7019.13</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -1405,26 +1405,26 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>67181</v>
+        <v>0</v>
       </c>
       <c r="M25" t="n">
-        <v>67181</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>114100</t>
+          <t>47116</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
+          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1436,10 +1436,10 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>6098.62</v>
+        <v>6968.21</v>
       </c>
       <c r="I26" t="n">
-        <v>6098.62</v>
+        <v>6968.21</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1448,26 +1448,26 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>4273.44</v>
+        <v>45397.15</v>
       </c>
       <c r="M26" t="n">
-        <v>4273.44</v>
+        <v>45397.15</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>111056</t>
+          <t>114100</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>JORGE ANTONIO LUNA LARA</t>
+          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1479,10 +1479,10 @@
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>6097.65</v>
+        <v>6098.62</v>
       </c>
       <c r="I27" t="n">
-        <v>6097.65</v>
+        <v>6098.62</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
@@ -1491,16 +1491,16 @@
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>60976.47</v>
+        <v>4273.44</v>
       </c>
       <c r="M27" t="n">
-        <v>60976.47</v>
+        <v>4273.44</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>103982</t>
+          <t>111056</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1510,7 +1510,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA RIOS BERNAL</t>
+          <t>JORGE ANTONIO LUNA LARA</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1522,10 +1522,10 @@
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>6060.91</v>
+        <v>6097.65</v>
       </c>
       <c r="I28" t="n">
-        <v>6060.91</v>
+        <v>6097.65</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -1534,16 +1534,16 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>0</v>
+        <v>60976.47</v>
       </c>
       <c r="M28" t="n">
-        <v>0</v>
+        <v>60976.47</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>95148</t>
+          <t>103982</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
+          <t>MARIA FERNANDA RIOS BERNAL</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1565,10 +1565,10 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>5686.91</v>
+        <v>6060.91</v>
       </c>
       <c r="I29" t="n">
-        <v>5686.91</v>
+        <v>6060.91</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -1577,16 +1577,16 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>51038.52</v>
+        <v>0</v>
       </c>
       <c r="M29" t="n">
-        <v>51038.52</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>109998</t>
+          <t>95148</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
+          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1608,10 +1608,10 @@
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>2966.58</v>
+        <v>5686.91</v>
       </c>
       <c r="I30" t="n">
-        <v>2966.58</v>
+        <v>5686.91</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1620,16 +1620,16 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>0</v>
+        <v>51038.52</v>
       </c>
       <c r="M30" t="n">
-        <v>0</v>
+        <v>51038.52</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>118246</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1639,22 +1639,22 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>JOSE ANTEMIO OLIVA SANTOS</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G31" t="n">
-        <v>0</v>
+        <v>1869.76</v>
       </c>
       <c r="H31" t="n">
-        <v>2513.54</v>
+        <v>1967.73</v>
       </c>
       <c r="I31" t="n">
-        <v>2513.54</v>
+        <v>3837.49</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1663,16 +1663,16 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>3062.5</v>
+        <v>20567.37</v>
       </c>
       <c r="M31" t="n">
-        <v>3062.5</v>
+        <v>20567.37</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>120051</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1682,22 +1682,22 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>GUILLERMO JOSE RAMIREZ RAMIREZ</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G32" t="n">
-        <v>2488.17</v>
+        <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>0</v>
+        <v>3616.88</v>
       </c>
       <c r="I32" t="n">
-        <v>2488.17</v>
+        <v>3616.88</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1706,26 +1706,26 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>27369.85</v>
+        <v>13652.86</v>
       </c>
       <c r="M32" t="n">
-        <v>27369.85</v>
+        <v>13652.86</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>113450</t>
+          <t>118069</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
+          <t>MARIO IVAN ROMERO GONZALEZ</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1737,10 +1737,10 @@
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>2072.23</v>
+        <v>3446.05</v>
       </c>
       <c r="I33" t="n">
-        <v>2072.23</v>
+        <v>3446.05</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -1749,26 +1749,26 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>16577.8</v>
+        <v>38958.2</v>
       </c>
       <c r="M33" t="n">
-        <v>16577.8</v>
+        <v>38958.2</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>118246</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>JOSE ANTEMIO OLIVA SANTOS</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1777,13 +1777,13 @@
         <v>0</v>
       </c>
       <c r="G34" t="n">
-        <v>0</v>
+        <v>-2313.19</v>
       </c>
       <c r="H34" t="n">
-        <v>1967.73</v>
+        <v>5550.6</v>
       </c>
       <c r="I34" t="n">
-        <v>1967.73</v>
+        <v>3237.41</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
@@ -1792,16 +1792,16 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>0</v>
+        <v>41354.29</v>
       </c>
       <c r="M34" t="n">
-        <v>0</v>
+        <v>41354.29</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>109998</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1811,7 +1811,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>EVELYN CAROLINA VENEGAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1823,10 +1823,10 @@
         <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>1800.77</v>
+        <v>2966.58</v>
       </c>
       <c r="I35" t="n">
-        <v>1800.77</v>
+        <v>2966.58</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -1835,26 +1835,26 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>10804.65</v>
+        <v>0</v>
       </c>
       <c r="M35" t="n">
-        <v>10804.65</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1866,10 +1866,10 @@
         <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>1781.04</v>
+        <v>2513.54</v>
       </c>
       <c r="I36" t="n">
-        <v>1781.04</v>
+        <v>2513.54</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
@@ -1878,41 +1878,41 @@
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>15488.7</v>
+        <v>3062.5</v>
       </c>
       <c r="M36" t="n">
-        <v>15488.7</v>
+        <v>3062.5</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>65046</t>
+          <t>120051</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+          <t>GUILLERMO JOSE RAMIREZ RAMIREZ</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G37" t="n">
-        <v>0</v>
+        <v>2488.17</v>
       </c>
       <c r="H37" t="n">
-        <v>1747.29</v>
+        <v>0</v>
       </c>
       <c r="I37" t="n">
-        <v>1747.29</v>
+        <v>2488.17</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -1921,26 +1921,26 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>3494.59</v>
+        <v>27369.85</v>
       </c>
       <c r="M37" t="n">
-        <v>3494.59</v>
+        <v>27369.85</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>118069</t>
+          <t>113450</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>MARIO IVAN ROMERO GONZALEZ</t>
+          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1952,10 +1952,10 @@
         <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>1662.54</v>
+        <v>2072.23</v>
       </c>
       <c r="I38" t="n">
-        <v>1662.54</v>
+        <v>2072.23</v>
       </c>
       <c r="J38" t="n">
         <v>0</v>
@@ -1964,16 +1964,16 @@
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>40741.71</v>
+        <v>16577.8</v>
       </c>
       <c r="M38" t="n">
-        <v>40741.71</v>
+        <v>16577.8</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>116795</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>GERARDO DANIEL BARAJAS TORRES</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1995,10 +1995,10 @@
         <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>1598.75</v>
+        <v>1800.77</v>
       </c>
       <c r="I39" t="n">
-        <v>1598.75</v>
+        <v>1800.77</v>
       </c>
       <c r="J39" t="n">
         <v>0</v>
@@ -2007,16 +2007,16 @@
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>0</v>
+        <v>10804.65</v>
       </c>
       <c r="M39" t="n">
-        <v>0</v>
+        <v>10804.65</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>65046</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2038,10 +2038,10 @@
         <v>0</v>
       </c>
       <c r="H40" t="n">
-        <v>1516.55</v>
+        <v>1747.29</v>
       </c>
       <c r="I40" t="n">
-        <v>1516.55</v>
+        <v>1747.29</v>
       </c>
       <c r="J40" t="n">
         <v>0</v>
@@ -2050,26 +2050,26 @@
         <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>0</v>
+        <v>3494.59</v>
       </c>
       <c r="M40" t="n">
-        <v>0</v>
+        <v>3494.59</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>116795</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>GERARDO DANIEL BARAJAS TORRES</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2078,13 +2078,13 @@
         <v>0</v>
       </c>
       <c r="G41" t="n">
-        <v>-2313.19</v>
+        <v>0</v>
       </c>
       <c r="H41" t="n">
-        <v>3524.19</v>
+        <v>1598.75</v>
       </c>
       <c r="I41" t="n">
-        <v>1211</v>
+        <v>1598.75</v>
       </c>
       <c r="J41" t="n">
         <v>0</v>
@@ -2093,16 +2093,16 @@
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>43380.7</v>
+        <v>0</v>
       </c>
       <c r="M41" t="n">
-        <v>43380.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>115404</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2124,10 +2124,10 @@
         <v>0</v>
       </c>
       <c r="H42" t="n">
-        <v>0</v>
+        <v>1516.55</v>
       </c>
       <c r="I42" t="n">
-        <v>0</v>
+        <v>1516.55</v>
       </c>
       <c r="J42" t="n">
         <v>0</v>
@@ -2136,16 +2136,16 @@
         <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>3487.19</v>
+        <v>0</v>
       </c>
       <c r="M42" t="n">
-        <v>3487.19</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -2179,16 +2179,16 @@
         <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>1693.99</v>
+        <v>3487.19</v>
       </c>
       <c r="M43" t="n">
-        <v>1693.99</v>
+        <v>3487.19</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2198,7 +2198,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -2222,16 +2222,16 @@
         <v>0</v>
       </c>
       <c r="L44" t="n">
-        <v>17425.73</v>
+        <v>1693.99</v>
       </c>
       <c r="M44" t="n">
-        <v>17425.73</v>
+        <v>1693.99</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>110575</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2241,7 +2241,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>JOSE RENE DE ALBA MORALES</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -2265,10 +2265,10 @@
         <v>0</v>
       </c>
       <c r="L45" t="n">
-        <v>14427.08</v>
+        <v>17425.73</v>
       </c>
       <c r="M45" t="n">
-        <v>14427.08</v>
+        <v>17425.73</v>
       </c>
     </row>
     <row r="46">
@@ -2312,49 +2312,6 @@
       </c>
       <c r="M46" t="n">
         <v>12811.03</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>101640</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>2043</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>SAMUEL NUÐO RIVERA</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
-      <c r="F47" t="n">
-        <v>0</v>
-      </c>
-      <c r="G47" t="n">
-        <v>0</v>
-      </c>
-      <c r="H47" t="n">
-        <v>0</v>
-      </c>
-      <c r="I47" t="n">
-        <v>0</v>
-      </c>
-      <c r="J47" t="n">
-        <v>0</v>
-      </c>
-      <c r="K47" t="n">
-        <v>0</v>
-      </c>
-      <c r="L47" t="n">
-        <v>3214.14</v>
-      </c>
-      <c r="M47" t="n">
-        <v>3214.14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-10-01 12:16)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M46"/>
+  <dimension ref="A1:N46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,6 +434,7 @@
       <c r="K1" t="inlineStr"/>
       <c r="L1" t="inlineStr"/>
       <c r="M1" t="inlineStr"/>
+      <c r="N1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr"/>
@@ -449,6 +450,7 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr"/>
@@ -464,6 +466,7 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -507,6 +510,11 @@
       <c r="M4" t="n">
         <v>144635.2</v>
       </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>2019-09-23</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -550,6 +558,11 @@
       <c r="M5" t="n">
         <v>30697.04</v>
       </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>2023-11-06</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -593,6 +606,11 @@
       <c r="M6" t="n">
         <v>78028.36</v>
       </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>2024-11-04</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -636,6 +654,11 @@
       <c r="M7" t="n">
         <v>17952.77</v>
       </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>2025-10-14</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -679,6 +702,11 @@
       <c r="M8" t="n">
         <v>10978.48</v>
       </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>2023-12-04</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -722,6 +750,11 @@
       <c r="M9" t="n">
         <v>31248.84</v>
       </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>2024-06-24</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -765,6 +798,11 @@
       <c r="M10" t="n">
         <v>67181</v>
       </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -808,6 +846,11 @@
       <c r="M11" t="n">
         <v>237843.4</v>
       </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>2018-09-28</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -851,6 +894,11 @@
       <c r="M12" t="n">
         <v>80679.25999999999</v>
       </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -894,6 +942,11 @@
       <c r="M13" t="n">
         <v>84870.92999999999</v>
       </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -937,6 +990,11 @@
       <c r="M14" t="n">
         <v>7492.65</v>
       </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>2018-12-05</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -980,6 +1038,11 @@
       <c r="M15" t="n">
         <v>0</v>
       </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>2024-05-28</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1022,6 +1085,11 @@
       </c>
       <c r="M16" t="n">
         <v>32742.4</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -1066,6 +1134,11 @@
       <c r="M17" t="n">
         <v>36067.65</v>
       </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1109,6 +1182,11 @@
       <c r="M18" t="n">
         <v>0</v>
       </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>2024-10-18</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1152,6 +1230,11 @@
       <c r="M19" t="n">
         <v>143052.28</v>
       </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>2023-12-19</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1195,6 +1278,11 @@
       <c r="M20" t="n">
         <v>76989.35000000001</v>
       </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>2020-04-28</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1238,6 +1326,11 @@
       <c r="M21" t="n">
         <v>0</v>
       </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>2023-03-14</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1281,6 +1374,11 @@
       <c r="M22" t="n">
         <v>0</v>
       </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>2024-06-28</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1324,6 +1422,11 @@
       <c r="M23" t="n">
         <v>3845.25</v>
       </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>2019-11-25</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1367,6 +1470,11 @@
       <c r="M24" t="n">
         <v>15958.78</v>
       </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>2024-02-22</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1410,6 +1518,11 @@
       <c r="M25" t="n">
         <v>0</v>
       </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>2020-11-24</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1453,6 +1566,11 @@
       <c r="M26" t="n">
         <v>45397.15</v>
       </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>2022-02-24</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1496,6 +1614,11 @@
       <c r="M27" t="n">
         <v>4273.44</v>
       </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>2025-07-25</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1539,6 +1662,11 @@
       <c r="M28" t="n">
         <v>60976.47</v>
       </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>2024-12-13</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1582,6 +1710,11 @@
       <c r="M29" t="n">
         <v>0</v>
       </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>2023-10-17</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1624,6 +1757,11 @@
       </c>
       <c r="M30" t="n">
         <v>51038.52</v>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>2022-12-21</t>
+        </is>
       </c>
     </row>
     <row r="31">
@@ -1668,6 +1806,11 @@
       <c r="M31" t="n">
         <v>20567.37</v>
       </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1711,6 +1854,11 @@
       <c r="M32" t="n">
         <v>13652.86</v>
       </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>2025-12-19</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1754,6 +1902,11 @@
       <c r="M33" t="n">
         <v>38958.2</v>
       </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1797,6 +1950,11 @@
       <c r="M34" t="n">
         <v>41354.29</v>
       </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1840,6 +1998,11 @@
       <c r="M35" t="n">
         <v>0</v>
       </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>2024-10-31</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1882,6 +2045,11 @@
       </c>
       <c r="M36" t="n">
         <v>3062.5</v>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>2023-07-10</t>
+        </is>
       </c>
     </row>
     <row r="37">
@@ -1926,6 +2094,11 @@
       <c r="M37" t="n">
         <v>27369.85</v>
       </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1969,6 +2142,11 @@
       <c r="M38" t="n">
         <v>16577.8</v>
       </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>2025-07-14</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2012,6 +2190,11 @@
       <c r="M39" t="n">
         <v>10804.65</v>
       </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>2025-03-20</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2055,6 +2238,11 @@
       <c r="M40" t="n">
         <v>3494.59</v>
       </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>2022-07-21</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2098,6 +2286,11 @@
       <c r="M41" t="n">
         <v>0</v>
       </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>2025-12-09</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2141,6 +2334,11 @@
       <c r="M42" t="n">
         <v>0</v>
       </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>2024-08-21</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2184,6 +2382,11 @@
       <c r="M43" t="n">
         <v>3487.19</v>
       </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>2025-11-25</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2227,6 +2430,11 @@
       <c r="M44" t="n">
         <v>1693.99</v>
       </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>2025-09-30</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2270,6 +2478,11 @@
       <c r="M45" t="n">
         <v>17425.73</v>
       </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>2025-09-04</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2312,6 +2525,11 @@
       </c>
       <c r="M46" t="n">
         <v>12811.03</v>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>2023-10-02</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-10-14 10:59)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -413,13 +413,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N43"/>
+  <dimension ref="A1:N45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>6 de octubre de 2026</t>
+          <t>12 de octubre de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -471,32 +471,32 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>110453</t>
+          <t>87538</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ANAIS LUA MORENO</t>
+          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>31095.36</v>
       </c>
       <c r="H4" t="n">
-        <v>15025.21</v>
+        <v>13502.83</v>
       </c>
       <c r="I4" t="n">
-        <v>15025.21</v>
+        <v>44598.19</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -505,46 +505,46 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>89494.05</v>
+        <v>150657.52</v>
       </c>
       <c r="M4" t="n">
-        <v>89494.05</v>
+        <v>150657.52</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2024-11-04</t>
+          <t>2019-09-23</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>104343</t>
+          <t>110453</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
+          <t>ANAIS LUA MORENO</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>3113.05</v>
       </c>
       <c r="H5" t="n">
-        <v>10358.06</v>
+        <v>17256.79</v>
       </c>
       <c r="I5" t="n">
-        <v>10358.06</v>
+        <v>20369.84</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -553,31 +553,31 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>2487.3</v>
+        <v>89494.05</v>
       </c>
       <c r="M5" t="n">
-        <v>2487.3</v>
+        <v>89494.05</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2023-10-02</t>
+          <t>2024-11-04</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>116883</t>
+          <t>104343</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>SOFIA CAMPILLO VASCONCELOS</t>
+          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -589,10 +589,10 @@
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>9690.030000000001</v>
+        <v>10358.06</v>
       </c>
       <c r="I6" t="n">
-        <v>9690.030000000001</v>
+        <v>10358.06</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -601,31 +601,31 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>90526.00999999999</v>
+        <v>2487.3</v>
       </c>
       <c r="M6" t="n">
-        <v>90526.00999999999</v>
+        <v>2487.3</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2023-10-02</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>88234</t>
+          <t>116883</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
+          <t>SOFIA CAMPILLO VASCONCELOS</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -637,10 +637,10 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>8514.83</v>
+        <v>9690.030000000001</v>
       </c>
       <c r="I7" t="n">
-        <v>8514.83</v>
+        <v>9690.030000000001</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -649,21 +649,21 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>1927.78</v>
+        <v>90526.00999999999</v>
       </c>
       <c r="M7" t="n">
-        <v>1927.78</v>
+        <v>90526.00999999999</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2019-11-25</t>
+          <t>2026-04-14</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>117440</t>
+          <t>88234</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -673,7 +673,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MONSERRAT VELASCO SANTOS</t>
+          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -685,33 +685,33 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>7572.06</v>
+        <v>8514.83</v>
       </c>
       <c r="I8" t="n">
-        <v>7572.06</v>
+        <v>8514.83</v>
       </c>
       <c r="J8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>8568.16</v>
+        <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>86380.78999999999</v>
+        <v>1927.78</v>
       </c>
       <c r="M8" t="n">
-        <v>94948.95</v>
+        <v>1927.78</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2019-11-25</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>104750</t>
+          <t>117440</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -721,7 +721,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
+          <t>MONSERRAT VELASCO SANTOS</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
@@ -733,33 +733,33 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>4904.69</v>
+        <v>7572.06</v>
       </c>
       <c r="I9" t="n">
-        <v>4904.69</v>
+        <v>7572.06</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>8568.16</v>
       </c>
       <c r="L9" t="n">
-        <v>0</v>
+        <v>86380.78999999999</v>
       </c>
       <c r="M9" t="n">
-        <v>0</v>
+        <v>94948.95</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2023-11-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>87538</t>
+          <t>80122</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -769,55 +769,55 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
+          <t>DESIREE DE LA PEÐA OROZCO</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>2423.1</v>
       </c>
       <c r="H10" t="n">
-        <v>3644.33</v>
+        <v>2719.05</v>
       </c>
       <c r="I10" t="n">
-        <v>3644.33</v>
+        <v>5142.15</v>
       </c>
       <c r="J10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K10" t="n">
-        <v>31095.36</v>
+        <v>8452.73</v>
       </c>
       <c r="L10" t="n">
-        <v>160516.04</v>
+        <v>148411.78</v>
       </c>
       <c r="M10" t="n">
-        <v>191611.4</v>
+        <v>156864.51</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2019-09-23</t>
+          <t>2018-09-28</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>104750</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -829,10 +829,10 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>3533.64</v>
+        <v>4904.69</v>
       </c>
       <c r="I11" t="n">
-        <v>3533.64</v>
+        <v>4904.69</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -841,21 +841,21 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>39399.35</v>
+        <v>0</v>
       </c>
       <c r="M11" t="n">
-        <v>39399.35</v>
+        <v>0</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2023-11-06</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>120051</t>
+          <t>115047</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -865,22 +865,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>GUILLERMO JOSE RAMIREZ RAMIREZ</t>
+          <t>VELIA PATRICIA BERNAL RAMOS</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>3489.2</v>
+        <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>4819.53</v>
       </c>
       <c r="I12" t="n">
-        <v>3489.2</v>
+        <v>4819.53</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -889,79 +889,79 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>65824.42</v>
+        <v>18583.84</v>
       </c>
       <c r="M12" t="n">
-        <v>65824.42</v>
+        <v>18583.84</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2025-10-14</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>119447</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>LUIS ANTONIO SALAZAR ESPINOSA</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>2881.5</v>
       </c>
       <c r="H13" t="n">
-        <v>2639.98</v>
+        <v>888</v>
       </c>
       <c r="I13" t="n">
-        <v>2639.98</v>
+        <v>3769.5</v>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>1803.3</v>
       </c>
       <c r="L13" t="n">
-        <v>18380.26</v>
+        <v>87197.37</v>
       </c>
       <c r="M13" t="n">
-        <v>18380.26</v>
+        <v>89000.67</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2018-12-05</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>65046</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -973,10 +973,10 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>1751.98</v>
+        <v>3533.64</v>
       </c>
       <c r="I14" t="n">
-        <v>1751.98</v>
+        <v>3533.64</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -985,46 +985,46 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>1751.98</v>
+        <v>39399.35</v>
       </c>
       <c r="M14" t="n">
-        <v>1751.98</v>
+        <v>39399.35</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2022-07-21</t>
+          <t>2026-03-30</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>105696</t>
+          <t>120051</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>GABRIELA CASTAÐEDA SALAZAR</t>
+          <t>GUILLERMO JOSE RAMIREZ RAMIREZ</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>3489.2</v>
       </c>
       <c r="H15" t="n">
-        <v>1742.08</v>
+        <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>1742.08</v>
+        <v>3489.2</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -1033,21 +1033,21 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>141996.97</v>
+        <v>65824.42</v>
       </c>
       <c r="M15" t="n">
-        <v>141996.97</v>
+        <v>65824.42</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2023-12-19</t>
+          <t>2026-08-25</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>104718</t>
+          <t>47116</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ROGELIO TORRES ORTIZ</t>
+          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1069,10 +1069,10 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>1741.91</v>
+        <v>3458.46</v>
       </c>
       <c r="I16" t="n">
-        <v>1741.91</v>
+        <v>3458.46</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1081,21 +1081,21 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>14626.63</v>
+        <v>40578.53</v>
       </c>
       <c r="M16" t="n">
-        <v>14626.63</v>
+        <v>40578.53</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2023-12-04</t>
+          <t>2022-02-24</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1105,7 +1105,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1117,10 +1117,10 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>1707.19</v>
+        <v>2639.98</v>
       </c>
       <c r="I17" t="n">
-        <v>1707.19</v>
+        <v>2639.98</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1129,21 +1129,21 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>8535.940000000001</v>
+        <v>18380.26</v>
       </c>
       <c r="M17" t="n">
-        <v>8535.940000000001</v>
+        <v>18380.26</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2025-09-04</t>
+          <t>2018-12-05</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>47116</t>
+          <t>118246</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1153,7 +1153,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
+          <t>JOSE ANTEMIO OLIVA SANTOS</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1165,33 +1165,33 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>1577.24</v>
+        <v>1973.01</v>
       </c>
       <c r="I18" t="n">
-        <v>1577.24</v>
+        <v>1973.01</v>
       </c>
       <c r="J18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>30213.13</v>
       </c>
       <c r="L18" t="n">
-        <v>42118.14</v>
+        <v>20622.49</v>
       </c>
       <c r="M18" t="n">
-        <v>42118.14</v>
+        <v>50835.62</v>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2022-02-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1201,7 +1201,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -1210,13 +1210,13 @@
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>0</v>
+        <v>-1206.47</v>
       </c>
       <c r="H19" t="n">
-        <v>1520.61</v>
+        <v>2972.23</v>
       </c>
       <c r="I19" t="n">
-        <v>1520.61</v>
+        <v>1765.76</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1225,31 +1225,31 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>0</v>
+        <v>36521.92</v>
       </c>
       <c r="M19" t="n">
-        <v>0</v>
+        <v>36521.92</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2024-08-21</t>
+          <t>2024-06-24</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>119447</t>
+          <t>65046</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>LUIS ANTONIO SALAZAR ESPINOSA</t>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1261,10 +1261,10 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>0</v>
+        <v>1751.98</v>
       </c>
       <c r="I20" t="n">
-        <v>0</v>
+        <v>1751.98</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1273,21 +1273,21 @@
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>67361.03</v>
+        <v>1751.98</v>
       </c>
       <c r="M20" t="n">
-        <v>67361.03</v>
+        <v>1751.98</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2022-07-21</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>119223</t>
+          <t>105696</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1297,7 +1297,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>OSCAR RAMIREZ RUIZ</t>
+          <t>GABRIELA CASTAÐEDA SALAZAR</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1309,10 +1309,10 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>0</v>
+        <v>1742.08</v>
       </c>
       <c r="I21" t="n">
-        <v>0</v>
+        <v>1742.08</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -1321,21 +1321,21 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>36164.3</v>
+        <v>141996.97</v>
       </c>
       <c r="M21" t="n">
-        <v>36164.3</v>
+        <v>141996.97</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2023-12-19</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>118915</t>
+          <t>104718</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
+          <t>ROGELIO TORRES ORTIZ</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -1357,10 +1357,10 @@
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>0</v>
+        <v>1741.91</v>
       </c>
       <c r="I22" t="n">
-        <v>0</v>
+        <v>1741.91</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1369,21 +1369,21 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>32830.14</v>
+        <v>14626.63</v>
       </c>
       <c r="M22" t="n">
-        <v>32830.14</v>
+        <v>14626.63</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2023-12-04</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>118246</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1393,7 +1393,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>JOSE ANTEMIO OLIVA SANTOS</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -1405,10 +1405,10 @@
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>0</v>
+        <v>1707.19</v>
       </c>
       <c r="I23" t="n">
-        <v>0</v>
+        <v>1707.19</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -1417,31 +1417,31 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>22595.5</v>
+        <v>8535.940000000001</v>
       </c>
       <c r="M23" t="n">
-        <v>22595.5</v>
+        <v>8535.940000000001</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2025-09-04</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>118069</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>MARIO IVAN ROMERO GONZALEZ</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>0</v>
+        <v>1698.53</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
+        <v>1698.53</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
@@ -1465,31 +1465,31 @@
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>39062.59</v>
+        <v>0</v>
       </c>
       <c r="M24" t="n">
-        <v>39062.59</v>
+        <v>0</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2025-09-30</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1501,10 +1501,10 @@
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>0</v>
+        <v>1520.61</v>
       </c>
       <c r="I25" t="n">
-        <v>0</v>
+        <v>1520.61</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -1513,31 +1513,31 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>13689.45</v>
+        <v>0</v>
       </c>
       <c r="M25" t="n">
-        <v>13689.45</v>
+        <v>0</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2024-08-21</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>115404</t>
+          <t>114100</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
+          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1549,10 +1549,10 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>0</v>
+        <v>436.32</v>
       </c>
       <c r="I26" t="n">
-        <v>0</v>
+        <v>436.32</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1561,31 +1561,31 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>1748.27</v>
+        <v>24812.1</v>
       </c>
       <c r="M26" t="n">
-        <v>1748.27</v>
+        <v>24812.1</v>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-07-25</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>115047</t>
+          <t>120596</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>VELIA PATRICIA BERNAL RAMOS</t>
+          <t>OLGA SOFIA GAXIOLA IBARRA</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1603,27 +1603,27 @@
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K27" t="n">
-        <v>0</v>
+        <v>42182.62</v>
       </c>
       <c r="L27" t="n">
-        <v>16174.08</v>
+        <v>0</v>
       </c>
       <c r="M27" t="n">
-        <v>16174.08</v>
+        <v>42182.62</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2025-10-14</t>
+          <t>2026-10-06</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>119223</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>OSCAR RAMIREZ RUIZ</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1657,31 +1657,31 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>1698.53</v>
+        <v>36164.3</v>
       </c>
       <c r="M28" t="n">
-        <v>1698.53</v>
+        <v>36164.3</v>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2025-09-30</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>114100</t>
+          <t>118915</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
+          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1705,31 +1705,31 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>24812.1</v>
+        <v>32830.14</v>
       </c>
       <c r="M29" t="n">
-        <v>24812.1</v>
+        <v>32830.14</v>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2025-07-25</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>113450</t>
+          <t>118069</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
+          <t>MARIO IVAN ROMERO GONZALEZ</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1753,31 +1753,31 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>16622.23</v>
+        <v>39062.59</v>
       </c>
       <c r="M30" t="n">
-        <v>16622.23</v>
+        <v>39062.59</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2025-07-14</t>
+          <t>2026-06-19</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1801,21 +1801,21 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>10833.6</v>
+        <v>13689.45</v>
       </c>
       <c r="M31" t="n">
-        <v>10833.6</v>
+        <v>13689.45</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2025-03-20</t>
+          <t>2025-12-19</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>111056</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1825,7 +1825,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>JORGE ANTONIO LUNA LARA</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -1849,21 +1849,21 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>61139.88</v>
+        <v>1748.27</v>
       </c>
       <c r="M32" t="n">
-        <v>61139.88</v>
+        <v>1748.27</v>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2024-12-13</t>
+          <t>2025-11-25</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>113450</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1873,7 +1873,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1897,21 +1897,21 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>3049.62</v>
+        <v>16622.23</v>
       </c>
       <c r="M33" t="n">
-        <v>3049.62</v>
+        <v>16622.23</v>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2024-06-28</t>
+          <t>2025-07-14</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1921,7 +1921,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1945,21 +1945,21 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>1535.6</v>
+        <v>10833.6</v>
       </c>
       <c r="M34" t="n">
-        <v>1535.6</v>
+        <v>10833.6</v>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2024-05-28</t>
+          <t>2025-03-20</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>106018</t>
+          <t>111056</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1969,7 +1969,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>MIREYA LIZETTE TORRES GARCIA</t>
+          <t>JORGE ANTONIO LUNA LARA</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1993,21 +1993,21 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>21390.54</v>
+        <v>61139.88</v>
       </c>
       <c r="M35" t="n">
-        <v>21390.54</v>
+        <v>61139.88</v>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2024-02-22</t>
+          <t>2024-12-13</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>103982</t>
+          <t>110575</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2017,7 +2017,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA RIOS BERNAL</t>
+          <t>JOSE RENE DE ALBA MORALES</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -2035,27 +2035,27 @@
         <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K36" t="n">
-        <v>0</v>
+        <v>166560.33</v>
       </c>
       <c r="L36" t="n">
-        <v>6077.11</v>
+        <v>0</v>
       </c>
       <c r="M36" t="n">
-        <v>6077.11</v>
+        <v>166560.33</v>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2023-10-17</t>
+          <t>2024-10-18</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>108405</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2065,7 +2065,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -2089,21 +2089,21 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>5590.95</v>
+        <v>3049.62</v>
       </c>
       <c r="M37" t="n">
-        <v>5590.95</v>
+        <v>3049.62</v>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2023-07-10</t>
+          <t>2024-06-28</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2113,7 +2113,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -2137,21 +2137,21 @@
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>5468.35</v>
+        <v>1535.6</v>
       </c>
       <c r="M38" t="n">
-        <v>5468.35</v>
+        <v>1535.6</v>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2023-03-14</t>
+          <t>2024-05-28</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>95148</t>
+          <t>106018</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2161,7 +2161,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
+          <t>MIREYA LIZETTE TORRES GARCIA</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -2185,21 +2185,21 @@
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>53502.58</v>
+        <v>21390.54</v>
       </c>
       <c r="M39" t="n">
-        <v>53502.58</v>
+        <v>21390.54</v>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2022-12-21</t>
+          <t>2024-02-22</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>94156</t>
+          <t>103982</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2209,7 +2209,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>MARIA TERESA ASENCIO LOZANO</t>
+          <t>MARIA FERNANDA RIOS BERNAL</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2233,21 +2233,21 @@
         <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>7507.58</v>
+        <v>6077.11</v>
       </c>
       <c r="M40" t="n">
-        <v>7507.58</v>
+        <v>6077.11</v>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2020-11-24</t>
+          <t>2023-10-17</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>90355</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2257,7 +2257,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>DARINKA UREÐA CASILLAS</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2281,21 +2281,21 @@
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>126626.83</v>
+        <v>2520.24</v>
       </c>
       <c r="M41" t="n">
-        <v>126626.83</v>
+        <v>2520.24</v>
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>2020-04-28</t>
+          <t>2023-07-10</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>80122</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2305,7 +2305,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>DESIREE DE LA PEÐA OROZCO</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2323,27 +2323,27 @@
         <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K42" t="n">
-        <v>8452.73</v>
+        <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>148411.78</v>
+        <v>5468.35</v>
       </c>
       <c r="M42" t="n">
-        <v>156864.51</v>
+        <v>5468.35</v>
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>2018-09-28</t>
+          <t>2023-03-14</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>95148</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2353,7 +2353,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -2362,13 +2362,13 @@
         <v>0</v>
       </c>
       <c r="G43" t="n">
-        <v>-1206.47</v>
+        <v>0</v>
       </c>
       <c r="H43" t="n">
-        <v>859.38</v>
+        <v>0</v>
       </c>
       <c r="I43" t="n">
-        <v>-347.09</v>
+        <v>0</v>
       </c>
       <c r="J43" t="n">
         <v>0</v>
@@ -2377,14 +2377,110 @@
         <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>31964.11</v>
+        <v>53502.58</v>
       </c>
       <c r="M43" t="n">
-        <v>31964.11</v>
+        <v>53502.58</v>
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>2024-06-24</t>
+          <t>2022-12-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>94156</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2043</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>MARIA TERESA ASENCIO LOZANO</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" t="n">
+        <v>0</v>
+      </c>
+      <c r="L44" t="n">
+        <v>7507.58</v>
+      </c>
+      <c r="M44" t="n">
+        <v>7507.58</v>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>2020-11-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>90355</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2043</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>DARINKA UREÐA CASILLAS</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" t="n">
+        <v>0</v>
+      </c>
+      <c r="L45" t="n">
+        <v>126626.83</v>
+      </c>
+      <c r="M45" t="n">
+        <v>126626.83</v>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>2020-04-28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: Actualización de reportes (2026-10-15)
MDRT, Legión Centurión, Camino a la Cumbre, El Poder de Elegirte y Comparativo
de Vida al 9 de octubre; Proactivos y Asesores sin Emisión al 13 de octubre.
Publicado al servidor, avisos verificados en /api/comunicados/history y
archivado mensual completo.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>12 de octubre de 2026</t>
+          <t>13 de octubre de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -519,17 +519,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>110453</t>
+          <t>118246</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ANAIS LUA MORENO</t>
+          <t>JOSE ANTEMIO OLIVA SANTOS</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -538,13 +538,13 @@
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>3113.05</v>
+        <v>30213.13</v>
       </c>
       <c r="H5" t="n">
-        <v>17256.79</v>
+        <v>1973.01</v>
       </c>
       <c r="I5" t="n">
-        <v>20369.84</v>
+        <v>32186.14</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -553,46 +553,46 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>89494.05</v>
+        <v>20622.49</v>
       </c>
       <c r="M5" t="n">
-        <v>89494.05</v>
+        <v>20622.49</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2024-11-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>104343</t>
+          <t>110453</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
+          <t>ANAIS LUA MORENO</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>3113.05</v>
       </c>
       <c r="H6" t="n">
-        <v>10358.06</v>
+        <v>23099.39</v>
       </c>
       <c r="I6" t="n">
-        <v>10358.06</v>
+        <v>26212.44</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -601,31 +601,31 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>2487.3</v>
+        <v>83651.44</v>
       </c>
       <c r="M6" t="n">
-        <v>2487.3</v>
+        <v>83651.44</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2023-10-02</t>
+          <t>2024-11-04</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>116883</t>
+          <t>47116</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>SOFIA CAMPILLO VASCONCELOS</t>
+          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -637,10 +637,10 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>9690.030000000001</v>
+        <v>19301.17</v>
       </c>
       <c r="I7" t="n">
-        <v>9690.030000000001</v>
+        <v>19301.17</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -649,21 +649,21 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>90526.00999999999</v>
+        <v>24735.82</v>
       </c>
       <c r="M7" t="n">
-        <v>90526.00999999999</v>
+        <v>24735.82</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2022-02-24</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>88234</t>
+          <t>117440</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -673,45 +673,45 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
+          <t>MONSERRAT VELASCO SANTOS</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>2007.19</v>
       </c>
       <c r="H8" t="n">
-        <v>8514.83</v>
+        <v>10069.55</v>
       </c>
       <c r="I8" t="n">
-        <v>8514.83</v>
+        <v>12076.74</v>
       </c>
       <c r="J8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>4063.85</v>
       </c>
       <c r="L8" t="n">
-        <v>1927.78</v>
+        <v>86380.78999999999</v>
       </c>
       <c r="M8" t="n">
-        <v>1927.78</v>
+        <v>90444.64</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2019-11-25</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>117440</t>
+          <t>80122</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -721,45 +721,45 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MONSERRAT VELASCO SANTOS</t>
+          <t>DESIREE DE LA PEÐA OROZCO</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>2423.1</v>
       </c>
       <c r="H9" t="n">
-        <v>7572.06</v>
+        <v>8273.129999999999</v>
       </c>
       <c r="I9" t="n">
-        <v>7572.06</v>
+        <v>10696.23</v>
       </c>
       <c r="J9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K9" t="n">
-        <v>8568.16</v>
+        <v>28534.83</v>
       </c>
       <c r="L9" t="n">
-        <v>86380.78999999999</v>
+        <v>148411.78</v>
       </c>
       <c r="M9" t="n">
-        <v>94948.95</v>
+        <v>176946.61</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2018-09-28</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>80122</t>
+          <t>104343</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -769,55 +769,55 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>DESIREE DE LA PEÐA OROZCO</t>
+          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>2423.1</v>
+        <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>2719.05</v>
+        <v>10358.06</v>
       </c>
       <c r="I10" t="n">
-        <v>5142.15</v>
+        <v>10358.06</v>
       </c>
       <c r="J10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K10" t="n">
-        <v>8452.73</v>
+        <v>20225.92</v>
       </c>
       <c r="L10" t="n">
-        <v>148411.78</v>
+        <v>2487.3</v>
       </c>
       <c r="M10" t="n">
-        <v>156864.51</v>
+        <v>22713.22</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2018-09-28</t>
+          <t>2023-10-02</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>104750</t>
+          <t>116883</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
+          <t>SOFIA CAMPILLO VASCONCELOS</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -829,10 +829,10 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>4904.69</v>
+        <v>9690.030000000001</v>
       </c>
       <c r="I11" t="n">
-        <v>4904.69</v>
+        <v>9690.030000000001</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -841,31 +841,31 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>0</v>
+        <v>90526.00999999999</v>
       </c>
       <c r="M11" t="n">
-        <v>0</v>
+        <v>90526.00999999999</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2023-11-06</t>
+          <t>2026-04-14</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>115047</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>VELIA PATRICIA BERNAL RAMOS</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -877,10 +877,10 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>4819.53</v>
+        <v>8860.68</v>
       </c>
       <c r="I12" t="n">
-        <v>4819.53</v>
+        <v>8860.68</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -889,79 +889,79 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>18583.84</v>
+        <v>0</v>
       </c>
       <c r="M12" t="n">
-        <v>18583.84</v>
+        <v>0</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2025-10-14</t>
+          <t>2023-03-14</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>119447</t>
+          <t>88234</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>LUIS ANTONIO SALAZAR ESPINOSA</t>
+          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>2881.5</v>
+        <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>888</v>
+        <v>8514.83</v>
       </c>
       <c r="I13" t="n">
-        <v>3769.5</v>
+        <v>8514.83</v>
       </c>
       <c r="J13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>1803.3</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>87197.37</v>
+        <v>1927.78</v>
       </c>
       <c r="M13" t="n">
-        <v>89000.67</v>
+        <v>1927.78</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2019-11-25</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>104750</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -973,33 +973,33 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>3533.64</v>
+        <v>4904.69</v>
       </c>
       <c r="I14" t="n">
-        <v>3533.64</v>
+        <v>4904.69</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>50443.83</v>
       </c>
       <c r="L14" t="n">
-        <v>39399.35</v>
+        <v>0</v>
       </c>
       <c r="M14" t="n">
-        <v>39399.35</v>
+        <v>50443.83</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2023-11-06</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>120051</t>
+          <t>115047</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1009,22 +1009,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>GUILLERMO JOSE RAMIREZ RAMIREZ</t>
+          <t>VELIA PATRICIA BERNAL RAMOS</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>3489.2</v>
+        <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>4819.53</v>
       </c>
       <c r="I15" t="n">
-        <v>3489.2</v>
+        <v>4819.53</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -1033,79 +1033,79 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>65824.42</v>
+        <v>18583.84</v>
       </c>
       <c r="M15" t="n">
-        <v>65824.42</v>
+        <v>18583.84</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2025-10-14</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>47116</t>
+          <t>119447</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
+          <t>LUIS ANTONIO SALAZAR ESPINOSA</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G16" t="n">
-        <v>0</v>
+        <v>2881.5</v>
       </c>
       <c r="H16" t="n">
-        <v>3458.46</v>
+        <v>888</v>
       </c>
       <c r="I16" t="n">
-        <v>3458.46</v>
+        <v>3769.5</v>
       </c>
       <c r="J16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>1803.3</v>
       </c>
       <c r="L16" t="n">
-        <v>40578.53</v>
+        <v>87197.37</v>
       </c>
       <c r="M16" t="n">
-        <v>40578.53</v>
+        <v>89000.67</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2022-02-24</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1117,10 +1117,10 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>2639.98</v>
+        <v>3533.64</v>
       </c>
       <c r="I17" t="n">
-        <v>2639.98</v>
+        <v>3533.64</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1129,69 +1129,69 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>18380.26</v>
+        <v>39399.35</v>
       </c>
       <c r="M17" t="n">
-        <v>18380.26</v>
+        <v>39399.35</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2018-12-05</t>
+          <t>2026-03-30</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>118246</t>
+          <t>120051</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>JOSE ANTEMIO OLIVA SANTOS</t>
+          <t>GUILLERMO JOSE RAMIREZ RAMIREZ</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G18" t="n">
-        <v>0</v>
+        <v>3489.2</v>
       </c>
       <c r="H18" t="n">
-        <v>1973.01</v>
+        <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>1973.01</v>
+        <v>3489.2</v>
       </c>
       <c r="J18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>30213.13</v>
+        <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>20622.49</v>
+        <v>65824.42</v>
       </c>
       <c r="M18" t="n">
-        <v>50835.62</v>
+        <v>65824.42</v>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-25</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>108405</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1201,7 +1201,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -1210,13 +1210,13 @@
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>-1206.47</v>
+        <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>2972.23</v>
+        <v>3049.62</v>
       </c>
       <c r="I19" t="n">
-        <v>1765.76</v>
+        <v>3049.62</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1225,21 +1225,21 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>36521.92</v>
+        <v>0</v>
       </c>
       <c r="M19" t="n">
-        <v>36521.92</v>
+        <v>0</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2024-06-24</t>
+          <t>2024-06-28</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>65046</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1249,7 +1249,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1261,10 +1261,10 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>1751.98</v>
+        <v>2639.98</v>
       </c>
       <c r="I20" t="n">
-        <v>1751.98</v>
+        <v>2639.98</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1273,21 +1273,21 @@
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>1751.98</v>
+        <v>18380.26</v>
       </c>
       <c r="M20" t="n">
-        <v>1751.98</v>
+        <v>18380.26</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2022-07-21</t>
+          <t>2018-12-05</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>105696</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1297,7 +1297,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>GABRIELA CASTAÐEDA SALAZAR</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1306,13 +1306,13 @@
         <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>0</v>
+        <v>-1206.47</v>
       </c>
       <c r="H21" t="n">
-        <v>1742.08</v>
+        <v>2972.23</v>
       </c>
       <c r="I21" t="n">
-        <v>1742.08</v>
+        <v>1765.76</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -1321,21 +1321,21 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>141996.97</v>
+        <v>36521.92</v>
       </c>
       <c r="M21" t="n">
-        <v>141996.97</v>
+        <v>36521.92</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2023-12-19</t>
+          <t>2024-06-24</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>104718</t>
+          <t>65046</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ROGELIO TORRES ORTIZ</t>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -1357,10 +1357,10 @@
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>1741.91</v>
+        <v>1751.98</v>
       </c>
       <c r="I22" t="n">
-        <v>1741.91</v>
+        <v>1751.98</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1369,21 +1369,21 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>14626.63</v>
+        <v>1751.98</v>
       </c>
       <c r="M22" t="n">
-        <v>14626.63</v>
+        <v>1751.98</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2023-12-04</t>
+          <t>2022-07-21</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>105696</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1393,7 +1393,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>GABRIELA CASTAÐEDA SALAZAR</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -1405,10 +1405,10 @@
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>1707.19</v>
+        <v>1742.08</v>
       </c>
       <c r="I23" t="n">
-        <v>1707.19</v>
+        <v>1742.08</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -1417,21 +1417,21 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>8535.940000000001</v>
+        <v>141996.97</v>
       </c>
       <c r="M23" t="n">
-        <v>8535.940000000001</v>
+        <v>141996.97</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2025-09-04</t>
+          <t>2023-12-19</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>104718</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>ROGELIO TORRES ORTIZ</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>1698.53</v>
+        <v>1741.91</v>
       </c>
       <c r="I24" t="n">
-        <v>1698.53</v>
+        <v>1741.91</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
@@ -1465,21 +1465,21 @@
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>0</v>
+        <v>14626.63</v>
       </c>
       <c r="M24" t="n">
-        <v>0</v>
+        <v>14626.63</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2025-09-30</t>
+          <t>2023-12-04</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1489,7 +1489,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1501,10 +1501,10 @@
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>1520.61</v>
+        <v>1707.19</v>
       </c>
       <c r="I25" t="n">
-        <v>1520.61</v>
+        <v>1707.19</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -1513,31 +1513,31 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>0</v>
+        <v>8535.940000000001</v>
       </c>
       <c r="M25" t="n">
-        <v>0</v>
+        <v>8535.940000000001</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2024-08-21</t>
+          <t>2025-09-04</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>114100</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1549,10 +1549,10 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>436.32</v>
+        <v>1698.53</v>
       </c>
       <c r="I26" t="n">
-        <v>436.32</v>
+        <v>1698.53</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1561,21 +1561,21 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>24812.1</v>
+        <v>0</v>
       </c>
       <c r="M26" t="n">
-        <v>24812.1</v>
+        <v>0</v>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2025-07-25</t>
+          <t>2025-09-30</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>120596</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1585,7 +1585,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>OLGA SOFIA GAXIOLA IBARRA</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1597,43 +1597,43 @@
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>0</v>
+        <v>1520.61</v>
       </c>
       <c r="I27" t="n">
-        <v>0</v>
+        <v>1520.61</v>
       </c>
       <c r="J27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K27" t="n">
-        <v>42182.62</v>
+        <v>0</v>
       </c>
       <c r="L27" t="n">
         <v>0</v>
       </c>
       <c r="M27" t="n">
-        <v>42182.62</v>
+        <v>0</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2024-08-21</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>119223</t>
+          <t>114100</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>OSCAR RAMIREZ RUIZ</t>
+          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1645,10 +1645,10 @@
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>0</v>
+        <v>436.32</v>
       </c>
       <c r="I28" t="n">
-        <v>0</v>
+        <v>436.32</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -1657,21 +1657,21 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>36164.3</v>
+        <v>24812.1</v>
       </c>
       <c r="M28" t="n">
-        <v>36164.3</v>
+        <v>24812.1</v>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2025-07-25</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>118915</t>
+          <t>120596</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1681,7 +1681,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
+          <t>OLGA SOFIA GAXIOLA IBARRA</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1699,37 +1699,37 @@
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K29" t="n">
-        <v>0</v>
+        <v>42182.62</v>
       </c>
       <c r="L29" t="n">
-        <v>32830.14</v>
+        <v>0</v>
       </c>
       <c r="M29" t="n">
-        <v>32830.14</v>
+        <v>42182.62</v>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-10-06</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>118069</t>
+          <t>119223</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>MARIO IVAN ROMERO GONZALEZ</t>
+          <t>OSCAR RAMIREZ RUIZ</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1753,31 +1753,31 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>39062.59</v>
+        <v>36164.3</v>
       </c>
       <c r="M30" t="n">
-        <v>39062.59</v>
+        <v>36164.3</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>118915</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1801,31 +1801,31 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>13689.45</v>
+        <v>32830.14</v>
       </c>
       <c r="M31" t="n">
-        <v>13689.45</v>
+        <v>32830.14</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>115404</t>
+          <t>118069</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
+          <t>MARIO IVAN ROMERO GONZALEZ</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -1849,31 +1849,31 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>1748.27</v>
+        <v>39062.59</v>
       </c>
       <c r="M32" t="n">
-        <v>1748.27</v>
+        <v>39062.59</v>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2026-06-19</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>113450</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1897,21 +1897,21 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>16622.23</v>
+        <v>13689.45</v>
       </c>
       <c r="M33" t="n">
-        <v>16622.23</v>
+        <v>13689.45</v>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2025-07-14</t>
+          <t>2025-12-19</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1921,7 +1921,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1945,21 +1945,21 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>10833.6</v>
+        <v>1748.27</v>
       </c>
       <c r="M34" t="n">
-        <v>10833.6</v>
+        <v>1748.27</v>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2025-03-20</t>
+          <t>2025-11-25</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>111056</t>
+          <t>113450</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1969,7 +1969,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>JORGE ANTONIO LUNA LARA</t>
+          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1993,21 +1993,21 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>61139.88</v>
+        <v>16622.23</v>
       </c>
       <c r="M35" t="n">
-        <v>61139.88</v>
+        <v>16622.23</v>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2024-12-13</t>
+          <t>2025-07-14</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>110575</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2017,7 +2017,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>JOSE RENE DE ALBA MORALES</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -2035,27 +2035,27 @@
         <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K36" t="n">
-        <v>166560.33</v>
+        <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>0</v>
+        <v>10833.6</v>
       </c>
       <c r="M36" t="n">
-        <v>166560.33</v>
+        <v>10833.6</v>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2024-10-18</t>
+          <t>2025-03-20</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>111056</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2065,7 +2065,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>JORGE ANTONIO LUNA LARA</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -2089,21 +2089,21 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>3049.62</v>
+        <v>61139.88</v>
       </c>
       <c r="M37" t="n">
-        <v>3049.62</v>
+        <v>61139.88</v>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2024-06-28</t>
+          <t>2024-12-13</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>110575</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2113,7 +2113,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>JOSE RENE DE ALBA MORALES</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -2131,27 +2131,27 @@
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K38" t="n">
-        <v>0</v>
+        <v>166560.33</v>
       </c>
       <c r="L38" t="n">
-        <v>1535.6</v>
+        <v>0</v>
       </c>
       <c r="M38" t="n">
-        <v>1535.6</v>
+        <v>166560.33</v>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2024-05-28</t>
+          <t>2024-10-18</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>106018</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2161,7 +2161,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>MIREYA LIZETTE TORRES GARCIA</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -2185,21 +2185,21 @@
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>21390.54</v>
+        <v>1535.6</v>
       </c>
       <c r="M39" t="n">
-        <v>21390.54</v>
+        <v>1535.6</v>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2024-02-22</t>
+          <t>2024-05-28</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>103982</t>
+          <t>106018</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2209,7 +2209,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA RIOS BERNAL</t>
+          <t>MIREYA LIZETTE TORRES GARCIA</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2233,21 +2233,21 @@
         <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>6077.11</v>
+        <v>21390.54</v>
       </c>
       <c r="M40" t="n">
-        <v>6077.11</v>
+        <v>21390.54</v>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2023-10-17</t>
+          <t>2024-02-22</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>103982</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2257,7 +2257,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>MARIA FERNANDA RIOS BERNAL</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2281,21 +2281,21 @@
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>2520.24</v>
+        <v>6077.11</v>
       </c>
       <c r="M41" t="n">
-        <v>2520.24</v>
+        <v>6077.11</v>
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>2023-07-10</t>
+          <t>2023-10-17</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2305,7 +2305,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2329,14 +2329,14 @@
         <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>5468.35</v>
+        <v>2520.24</v>
       </c>
       <c r="M42" t="n">
-        <v>5468.35</v>
+        <v>2520.24</v>
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>2023-03-14</t>
+          <t>2023-07-10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-10-19 14:18)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>13 de octubre de 2026</t>
+          <t>16 de octubre de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -471,7 +471,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>87538</t>
+          <t>80122</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -481,22 +481,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
+          <t>DESIREE DE LA PEÐA OROZCO</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G4" t="n">
-        <v>31095.36</v>
+        <v>62959.52</v>
       </c>
       <c r="H4" t="n">
-        <v>13502.83</v>
+        <v>83617.09</v>
       </c>
       <c r="I4" t="n">
-        <v>44598.19</v>
+        <v>146576.61</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -505,21 +505,21 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>150657.52</v>
+        <v>118909.56</v>
       </c>
       <c r="M4" t="n">
-        <v>150657.52</v>
+        <v>118909.56</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2019-09-23</t>
+          <t>2018-09-28</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>118246</t>
+          <t>104750</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -529,7 +529,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>JOSE ANTEMIO OLIVA SANTOS</t>
+          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -538,13 +538,13 @@
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>30213.13</v>
+        <v>1992.97</v>
       </c>
       <c r="H5" t="n">
-        <v>1973.01</v>
+        <v>53355.54</v>
       </c>
       <c r="I5" t="n">
-        <v>32186.14</v>
+        <v>55348.51</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -553,31 +553,31 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>20622.49</v>
+        <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>20622.49</v>
+        <v>0</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2023-11-06</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>110453</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ANAIS LUA MORENO</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -586,13 +586,13 @@
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>3113.05</v>
+        <v>2973.12</v>
       </c>
       <c r="H6" t="n">
-        <v>23099.39</v>
+        <v>51866.38</v>
       </c>
       <c r="I6" t="n">
-        <v>26212.44</v>
+        <v>54839.5</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -601,21 +601,21 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>83651.44</v>
+        <v>31964.11</v>
       </c>
       <c r="M6" t="n">
-        <v>83651.44</v>
+        <v>31964.11</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2024-11-04</t>
+          <t>2024-06-24</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>47116</t>
+          <t>87538</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -625,22 +625,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
+          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>31095.36</v>
       </c>
       <c r="H7" t="n">
-        <v>19301.17</v>
+        <v>20932.3</v>
       </c>
       <c r="I7" t="n">
-        <v>19301.17</v>
+        <v>52027.66</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -649,31 +649,31 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>24735.82</v>
+        <v>143228.04</v>
       </c>
       <c r="M7" t="n">
-        <v>24735.82</v>
+        <v>143228.04</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2022-02-24</t>
+          <t>2019-09-23</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>117440</t>
+          <t>110453</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MONSERRAT VELASCO SANTOS</t>
+          <t>ANAIS LUA MORENO</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -682,36 +682,36 @@
         <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>2007.19</v>
+        <v>3113.05</v>
       </c>
       <c r="H8" t="n">
-        <v>10069.55</v>
+        <v>43114.8</v>
       </c>
       <c r="I8" t="n">
-        <v>12076.74</v>
+        <v>46227.85</v>
       </c>
       <c r="J8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>4063.85</v>
+        <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>86380.78999999999</v>
+        <v>59438.51</v>
       </c>
       <c r="M8" t="n">
-        <v>90444.64</v>
+        <v>59438.51</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2024-11-04</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>80122</t>
+          <t>118246</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -721,45 +721,45 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>DESIREE DE LA PEÐA OROZCO</t>
+          <t>JOSE ANTEMIO OLIVA SANTOS</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>2423.1</v>
+        <v>30213.13</v>
       </c>
       <c r="H9" t="n">
-        <v>8273.129999999999</v>
+        <v>1973.01</v>
       </c>
       <c r="I9" t="n">
-        <v>10696.23</v>
+        <v>32186.14</v>
       </c>
       <c r="J9" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>28534.83</v>
+        <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>148411.78</v>
+        <v>20622.49</v>
       </c>
       <c r="M9" t="n">
-        <v>176946.61</v>
+        <v>20622.49</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2018-09-28</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>104343</t>
+          <t>47116</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -769,7 +769,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
+          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -781,33 +781,33 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>10358.06</v>
+        <v>21042.72</v>
       </c>
       <c r="I10" t="n">
-        <v>10358.06</v>
+        <v>21042.72</v>
       </c>
       <c r="J10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>20225.92</v>
+        <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>2487.3</v>
+        <v>22994.27</v>
       </c>
       <c r="M10" t="n">
-        <v>22713.22</v>
+        <v>22994.27</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2023-10-02</t>
+          <t>2022-02-24</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>116883</t>
+          <t>114100</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -817,7 +817,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>SOFIA CAMPILLO VASCONCELOS</t>
+          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -829,10 +829,10 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>9690.030000000001</v>
+        <v>20960.31</v>
       </c>
       <c r="I11" t="n">
-        <v>9690.030000000001</v>
+        <v>20960.31</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -841,21 +841,21 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>90526.00999999999</v>
+        <v>4284.89</v>
       </c>
       <c r="M11" t="n">
-        <v>90526.00999999999</v>
+        <v>4284.89</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2025-07-25</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>117440</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -865,55 +865,55 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>MONSERRAT VELASCO SANTOS</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>2007.19</v>
       </c>
       <c r="H12" t="n">
-        <v>8860.68</v>
+        <v>10069.55</v>
       </c>
       <c r="I12" t="n">
-        <v>8860.68</v>
+        <v>12076.74</v>
       </c>
       <c r="J12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>4063.85</v>
       </c>
       <c r="L12" t="n">
-        <v>0</v>
+        <v>86380.78999999999</v>
       </c>
       <c r="M12" t="n">
-        <v>0</v>
+        <v>90444.64</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2023-03-14</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>88234</t>
+          <t>116883</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
+          <t>SOFIA CAMPILLO VASCONCELOS</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -925,10 +925,10 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>8514.83</v>
+        <v>11461.71</v>
       </c>
       <c r="I13" t="n">
-        <v>8514.83</v>
+        <v>11461.71</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -937,21 +937,21 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>1927.78</v>
+        <v>88754.33</v>
       </c>
       <c r="M13" t="n">
-        <v>1927.78</v>
+        <v>88754.33</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2019-11-25</t>
+          <t>2026-04-14</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>104750</t>
+          <t>104343</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
+          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -973,43 +973,43 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>4904.69</v>
+        <v>10358.06</v>
       </c>
       <c r="I14" t="n">
-        <v>4904.69</v>
+        <v>10358.06</v>
       </c>
       <c r="J14" t="n">
         <v>1</v>
       </c>
       <c r="K14" t="n">
-        <v>50443.83</v>
+        <v>20225.92</v>
       </c>
       <c r="L14" t="n">
-        <v>0</v>
+        <v>2487.3</v>
       </c>
       <c r="M14" t="n">
-        <v>50443.83</v>
+        <v>22713.22</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2023-11-06</t>
+          <t>2023-10-02</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>115047</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>VELIA PATRICIA BERNAL RAMOS</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -1021,10 +1021,10 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>4819.53</v>
+        <v>9879.52</v>
       </c>
       <c r="I15" t="n">
-        <v>4819.53</v>
+        <v>9879.52</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -1033,79 +1033,79 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>18583.84</v>
+        <v>0</v>
       </c>
       <c r="M15" t="n">
-        <v>18583.84</v>
+        <v>0</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2025-10-14</t>
+          <t>2023-03-14</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>119447</t>
+          <t>88234</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>LUIS ANTONIO SALAZAR ESPINOSA</t>
+          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>2881.5</v>
+        <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>888</v>
+        <v>8514.83</v>
       </c>
       <c r="I16" t="n">
-        <v>3769.5</v>
+        <v>8514.83</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>1803.3</v>
+        <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>87197.37</v>
+        <v>1927.78</v>
       </c>
       <c r="M16" t="n">
-        <v>89000.67</v>
+        <v>1927.78</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2019-11-25</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>103982</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>MARIA FERNANDA RIOS BERNAL</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1117,10 +1117,10 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>3533.64</v>
+        <v>6077.15</v>
       </c>
       <c r="I17" t="n">
-        <v>3533.64</v>
+        <v>6077.15</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1129,21 +1129,21 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>39399.35</v>
+        <v>0</v>
       </c>
       <c r="M17" t="n">
-        <v>39399.35</v>
+        <v>0</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2023-10-17</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>120051</t>
+          <t>115047</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1153,22 +1153,22 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>GUILLERMO JOSE RAMIREZ RAMIREZ</t>
+          <t>VELIA PATRICIA BERNAL RAMOS</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>3489.2</v>
+        <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>0</v>
+        <v>4819.53</v>
       </c>
       <c r="I18" t="n">
-        <v>3489.2</v>
+        <v>4819.53</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1177,21 +1177,21 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>65824.42</v>
+        <v>18583.84</v>
       </c>
       <c r="M18" t="n">
-        <v>65824.42</v>
+        <v>18583.84</v>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2025-10-14</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>95148</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1201,7 +1201,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -1213,10 +1213,10 @@
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>3049.62</v>
+        <v>3909.17</v>
       </c>
       <c r="I19" t="n">
-        <v>3049.62</v>
+        <v>3909.17</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1225,79 +1225,79 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>0</v>
+        <v>49593.45</v>
       </c>
       <c r="M19" t="n">
-        <v>0</v>
+        <v>49593.45</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2024-06-28</t>
+          <t>2022-12-21</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>119447</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>LUIS ANTONIO SALAZAR ESPINOSA</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G20" t="n">
-        <v>0</v>
+        <v>2881.5</v>
       </c>
       <c r="H20" t="n">
-        <v>2639.98</v>
+        <v>888</v>
       </c>
       <c r="I20" t="n">
-        <v>2639.98</v>
+        <v>3769.5</v>
       </c>
       <c r="J20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K20" t="n">
-        <v>0</v>
+        <v>1803.3</v>
       </c>
       <c r="L20" t="n">
-        <v>18380.26</v>
+        <v>87197.37</v>
       </c>
       <c r="M20" t="n">
-        <v>18380.26</v>
+        <v>89000.67</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2018-12-05</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1306,13 +1306,13 @@
         <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>-1206.47</v>
+        <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>2972.23</v>
+        <v>3533.64</v>
       </c>
       <c r="I21" t="n">
-        <v>1765.76</v>
+        <v>3533.64</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -1321,46 +1321,46 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>36521.92</v>
+        <v>39399.35</v>
       </c>
       <c r="M21" t="n">
-        <v>36521.92</v>
+        <v>39399.35</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2024-06-24</t>
+          <t>2026-03-30</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>65046</t>
+          <t>120051</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+          <t>GUILLERMO JOSE RAMIREZ RAMIREZ</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G22" t="n">
-        <v>0</v>
+        <v>3489.2</v>
       </c>
       <c r="H22" t="n">
-        <v>1751.98</v>
+        <v>0</v>
       </c>
       <c r="I22" t="n">
-        <v>1751.98</v>
+        <v>3489.2</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1369,31 +1369,31 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>1751.98</v>
+        <v>65824.42</v>
       </c>
       <c r="M22" t="n">
-        <v>1751.98</v>
+        <v>65824.42</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2022-07-21</t>
+          <t>2026-08-25</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>105696</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>GABRIELA CASTAÐEDA SALAZAR</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -1405,10 +1405,10 @@
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>1742.08</v>
+        <v>3206.78</v>
       </c>
       <c r="I23" t="n">
-        <v>1742.08</v>
+        <v>3206.78</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -1417,21 +1417,21 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>141996.97</v>
+        <v>10484.68</v>
       </c>
       <c r="M23" t="n">
-        <v>141996.97</v>
+        <v>10484.68</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2023-12-19</t>
+          <t>2025-12-19</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>104718</t>
+          <t>118915</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1441,22 +1441,22 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ROGELIO TORRES ORTIZ</t>
+          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G24" t="n">
-        <v>0</v>
+        <v>3120.29</v>
       </c>
       <c r="H24" t="n">
-        <v>1741.91</v>
+        <v>0</v>
       </c>
       <c r="I24" t="n">
-        <v>1741.91</v>
+        <v>3120.29</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
@@ -1465,21 +1465,21 @@
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>14626.63</v>
+        <v>67153.33</v>
       </c>
       <c r="M24" t="n">
-        <v>14626.63</v>
+        <v>67153.33</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2023-12-04</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>108405</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1489,7 +1489,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1501,10 +1501,10 @@
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>1707.19</v>
+        <v>3049.62</v>
       </c>
       <c r="I25" t="n">
-        <v>1707.19</v>
+        <v>3049.62</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -1513,21 +1513,21 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>8535.940000000001</v>
+        <v>0</v>
       </c>
       <c r="M25" t="n">
-        <v>8535.940000000001</v>
+        <v>0</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2025-09-04</t>
+          <t>2024-06-28</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1537,7 +1537,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1549,10 +1549,10 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>1698.53</v>
+        <v>2639.98</v>
       </c>
       <c r="I26" t="n">
-        <v>1698.53</v>
+        <v>2639.98</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1561,21 +1561,21 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>0</v>
+        <v>18380.26</v>
       </c>
       <c r="M26" t="n">
-        <v>0</v>
+        <v>18380.26</v>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2025-09-30</t>
+          <t>2018-12-05</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1585,7 +1585,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1597,10 +1597,10 @@
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>1520.61</v>
+        <v>1805.6</v>
       </c>
       <c r="I27" t="n">
-        <v>1520.61</v>
+        <v>1805.6</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
@@ -1609,31 +1609,31 @@
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>0</v>
+        <v>9028</v>
       </c>
       <c r="M27" t="n">
-        <v>0</v>
+        <v>9028</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2024-08-21</t>
+          <t>2025-03-20</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>114100</t>
+          <t>65046</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1645,10 +1645,10 @@
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>436.32</v>
+        <v>1751.98</v>
       </c>
       <c r="I28" t="n">
-        <v>436.32</v>
+        <v>1751.98</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -1657,21 +1657,21 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>24812.1</v>
+        <v>1751.98</v>
       </c>
       <c r="M28" t="n">
-        <v>24812.1</v>
+        <v>1751.98</v>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2025-07-25</t>
+          <t>2022-07-21</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>120596</t>
+          <t>105696</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1681,7 +1681,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>OLGA SOFIA GAXIOLA IBARRA</t>
+          <t>GABRIELA CASTAÐEDA SALAZAR</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1693,33 +1693,33 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>0</v>
+        <v>1742.08</v>
       </c>
       <c r="I29" t="n">
-        <v>0</v>
+        <v>1742.08</v>
       </c>
       <c r="J29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K29" t="n">
-        <v>42182.62</v>
+        <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>0</v>
+        <v>128661.02</v>
       </c>
       <c r="M29" t="n">
-        <v>42182.62</v>
+        <v>128661.02</v>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2023-12-19</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>119223</t>
+          <t>104718</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1729,7 +1729,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>OSCAR RAMIREZ RUIZ</t>
+          <t>ROGELIO TORRES ORTIZ</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1741,10 +1741,10 @@
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>0</v>
+        <v>1741.91</v>
       </c>
       <c r="I30" t="n">
-        <v>0</v>
+        <v>1741.91</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1753,21 +1753,21 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>36164.3</v>
+        <v>14626.63</v>
       </c>
       <c r="M30" t="n">
-        <v>36164.3</v>
+        <v>14626.63</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2023-12-04</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>118915</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1777,7 +1777,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1789,10 +1789,10 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>0</v>
+        <v>1707.19</v>
       </c>
       <c r="I31" t="n">
-        <v>0</v>
+        <v>1707.19</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1801,31 +1801,31 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>32830.14</v>
+        <v>8535.940000000001</v>
       </c>
       <c r="M31" t="n">
-        <v>32830.14</v>
+        <v>8535.940000000001</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2025-09-04</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>118069</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>MARIO IVAN ROMERO GONZALEZ</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -1837,10 +1837,10 @@
         <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>0</v>
+        <v>1698.53</v>
       </c>
       <c r="I32" t="n">
-        <v>0</v>
+        <v>1698.53</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1849,21 +1849,21 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>39062.59</v>
+        <v>0</v>
       </c>
       <c r="M32" t="n">
-        <v>39062.59</v>
+        <v>0</v>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2025-09-30</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>118069</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1873,7 +1873,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>MARIO IVAN ROMERO GONZALEZ</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1885,10 +1885,10 @@
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>0</v>
+        <v>1666.99</v>
       </c>
       <c r="I33" t="n">
-        <v>0</v>
+        <v>1666.99</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -1897,21 +1897,21 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>13689.45</v>
+        <v>37395.6</v>
       </c>
       <c r="M33" t="n">
-        <v>13689.45</v>
+        <v>37395.6</v>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2026-06-19</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>115404</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1921,7 +1921,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1933,10 +1933,10 @@
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>0</v>
+        <v>1520.61</v>
       </c>
       <c r="I34" t="n">
-        <v>0</v>
+        <v>1520.61</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
@@ -1945,21 +1945,21 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>1748.27</v>
+        <v>0</v>
       </c>
       <c r="M34" t="n">
-        <v>1748.27</v>
+        <v>0</v>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2024-08-21</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>113450</t>
+          <t>120596</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1969,7 +1969,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
+          <t>OLGA SOFIA GAXIOLA IBARRA</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1987,27 +1987,27 @@
         <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K35" t="n">
-        <v>0</v>
+        <v>74804.00999999999</v>
       </c>
       <c r="L35" t="n">
-        <v>16622.23</v>
+        <v>0</v>
       </c>
       <c r="M35" t="n">
-        <v>16622.23</v>
+        <v>74804.00999999999</v>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2025-07-14</t>
+          <t>2026-10-06</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>119223</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2017,7 +2017,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>OSCAR RAMIREZ RUIZ</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -2035,27 +2035,27 @@
         <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K36" t="n">
-        <v>0</v>
+        <v>76268.8</v>
       </c>
       <c r="L36" t="n">
-        <v>10833.6</v>
+        <v>36164.3</v>
       </c>
       <c r="M36" t="n">
-        <v>10833.6</v>
+        <v>112433.1</v>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2025-03-20</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>111056</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2065,7 +2065,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>JORGE ANTONIO LUNA LARA</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -2089,21 +2089,21 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>61139.88</v>
+        <v>1748.27</v>
       </c>
       <c r="M37" t="n">
-        <v>61139.88</v>
+        <v>1748.27</v>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2024-12-13</t>
+          <t>2025-11-25</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>110575</t>
+          <t>113450</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2113,7 +2113,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>JOSE RENE DE ALBA MORALES</t>
+          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -2131,27 +2131,27 @@
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K38" t="n">
-        <v>166560.33</v>
+        <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>0</v>
+        <v>16622.23</v>
       </c>
       <c r="M38" t="n">
-        <v>166560.33</v>
+        <v>16622.23</v>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2024-10-18</t>
+          <t>2025-07-14</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>111056</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2161,7 +2161,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>JORGE ANTONIO LUNA LARA</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -2185,21 +2185,21 @@
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>1535.6</v>
+        <v>61139.88</v>
       </c>
       <c r="M39" t="n">
-        <v>1535.6</v>
+        <v>61139.88</v>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2024-05-28</t>
+          <t>2024-12-13</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>106018</t>
+          <t>110575</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2209,7 +2209,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>MIREYA LIZETTE TORRES GARCIA</t>
+          <t>JOSE RENE DE ALBA MORALES</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2227,27 +2227,27 @@
         <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K40" t="n">
-        <v>0</v>
+        <v>166560.33</v>
       </c>
       <c r="L40" t="n">
-        <v>21390.54</v>
+        <v>0</v>
       </c>
       <c r="M40" t="n">
-        <v>21390.54</v>
+        <v>166560.33</v>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2024-02-22</t>
+          <t>2024-10-18</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>103982</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2257,7 +2257,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA RIOS BERNAL</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2281,21 +2281,21 @@
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>6077.11</v>
+        <v>1535.6</v>
       </c>
       <c r="M41" t="n">
-        <v>6077.11</v>
+        <v>1535.6</v>
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>2023-10-17</t>
+          <t>2024-05-28</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>106018</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2305,7 +2305,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>MIREYA LIZETTE TORRES GARCIA</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2329,21 +2329,21 @@
         <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>2520.24</v>
+        <v>21390.54</v>
       </c>
       <c r="M42" t="n">
-        <v>2520.24</v>
+        <v>21390.54</v>
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>2023-07-10</t>
+          <t>2024-02-22</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>95148</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2353,7 +2353,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -2377,14 +2377,14 @@
         <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>53502.58</v>
+        <v>2520.24</v>
       </c>
       <c r="M43" t="n">
-        <v>53502.58</v>
+        <v>2520.24</v>
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>2022-12-21</t>
+          <t>2023-07-10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-10-21 10:35)
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -413,13 +413,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N45"/>
+  <dimension ref="A1:N46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>16 de octubre de 2026</t>
+          <t>19 de octubre de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -759,17 +759,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>47116</t>
+          <t>114100</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
+          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -781,10 +781,10 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>21042.72</v>
+        <v>23102.75</v>
       </c>
       <c r="I10" t="n">
-        <v>21042.72</v>
+        <v>23102.75</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -793,31 +793,31 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>22994.27</v>
+        <v>2142.44</v>
       </c>
       <c r="M10" t="n">
-        <v>22994.27</v>
+        <v>2142.44</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2022-02-24</t>
+          <t>2025-07-25</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>114100</t>
+          <t>47116</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
+          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -829,10 +829,10 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>20960.31</v>
+        <v>21042.72</v>
       </c>
       <c r="I11" t="n">
-        <v>20960.31</v>
+        <v>21042.72</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -841,14 +841,14 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>4284.89</v>
+        <v>22994.27</v>
       </c>
       <c r="M11" t="n">
-        <v>4284.89</v>
+        <v>22994.27</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2025-07-25</t>
+          <t>2022-02-24</t>
         </is>
       </c>
     </row>
@@ -877,10 +877,10 @@
         <v>2007.19</v>
       </c>
       <c r="H12" t="n">
-        <v>10069.55</v>
+        <v>15277.78</v>
       </c>
       <c r="I12" t="n">
-        <v>12076.74</v>
+        <v>17284.97</v>
       </c>
       <c r="J12" t="n">
         <v>1</v>
@@ -889,10 +889,10 @@
         <v>4063.85</v>
       </c>
       <c r="L12" t="n">
-        <v>86380.78999999999</v>
+        <v>81172.53</v>
       </c>
       <c r="M12" t="n">
-        <v>90444.64</v>
+        <v>85236.38</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
@@ -903,17 +903,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>116883</t>
+          <t>105696</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>SOFIA CAMPILLO VASCONCELOS</t>
+          <t>GABRIELA CASTAÐEDA SALAZAR</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -925,10 +925,10 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>11461.71</v>
+        <v>15549.5</v>
       </c>
       <c r="I13" t="n">
-        <v>11461.71</v>
+        <v>15549.5</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -937,31 +937,31 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>88754.33</v>
+        <v>115314.53</v>
       </c>
       <c r="M13" t="n">
-        <v>88754.33</v>
+        <v>115314.53</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2023-12-19</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>104343</t>
+          <t>116883</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
+          <t>SOFIA CAMPILLO VASCONCELOS</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -973,33 +973,33 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>10358.06</v>
+        <v>11461.71</v>
       </c>
       <c r="I14" t="n">
-        <v>10358.06</v>
+        <v>11461.71</v>
       </c>
       <c r="J14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>20225.92</v>
+        <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>2487.3</v>
+        <v>88754.33</v>
       </c>
       <c r="M14" t="n">
-        <v>22713.22</v>
+        <v>88754.33</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2023-10-02</t>
+          <t>2026-04-14</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>104343</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1009,7 +1009,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>JORGE ALBERTO PRECIADO GONZALEZ</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -1021,33 +1021,33 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>9879.52</v>
+        <v>10358.06</v>
       </c>
       <c r="I15" t="n">
-        <v>9879.52</v>
+        <v>10358.06</v>
       </c>
       <c r="J15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>20225.92</v>
       </c>
       <c r="L15" t="n">
-        <v>0</v>
+        <v>2487.3</v>
       </c>
       <c r="M15" t="n">
-        <v>0</v>
+        <v>22713.22</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2023-03-14</t>
+          <t>2023-10-02</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>88234</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1069,10 +1069,10 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>8514.83</v>
+        <v>9879.52</v>
       </c>
       <c r="I16" t="n">
-        <v>8514.83</v>
+        <v>9879.52</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1081,21 +1081,21 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>1927.78</v>
+        <v>0</v>
       </c>
       <c r="M16" t="n">
-        <v>1927.78</v>
+        <v>0</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2019-11-25</t>
+          <t>2023-03-14</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>103982</t>
+          <t>88234</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1105,7 +1105,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA RIOS BERNAL</t>
+          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1117,10 +1117,10 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>6077.15</v>
+        <v>8514.83</v>
       </c>
       <c r="I17" t="n">
-        <v>6077.15</v>
+        <v>8514.83</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1129,31 +1129,31 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>0</v>
+        <v>1927.78</v>
       </c>
       <c r="M17" t="n">
-        <v>0</v>
+        <v>1927.78</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2023-10-17</t>
+          <t>2019-11-25</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>115047</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>VELIA PATRICIA BERNAL RAMOS</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1165,10 +1165,10 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>4819.53</v>
+        <v>7624.18</v>
       </c>
       <c r="I18" t="n">
-        <v>4819.53</v>
+        <v>7624.18</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1177,127 +1177,127 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>18583.84</v>
+        <v>18380.26</v>
       </c>
       <c r="M18" t="n">
-        <v>18583.84</v>
+        <v>18380.26</v>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2025-10-14</t>
+          <t>2018-12-05</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>95148</t>
+          <t>119447</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
+          <t>LUIS ANTONIO SALAZAR ESPINOSA</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G19" t="n">
-        <v>0</v>
+        <v>2881.5</v>
       </c>
       <c r="H19" t="n">
-        <v>3909.17</v>
+        <v>3954.23</v>
       </c>
       <c r="I19" t="n">
-        <v>3909.17</v>
+        <v>6835.73</v>
       </c>
       <c r="J19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K19" t="n">
-        <v>0</v>
+        <v>1803.3</v>
       </c>
       <c r="L19" t="n">
-        <v>49593.45</v>
+        <v>84131.14</v>
       </c>
       <c r="M19" t="n">
-        <v>49593.45</v>
+        <v>85934.44</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2022-12-21</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>119447</t>
+          <t>111056</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>LUIS ANTONIO SALAZAR ESPINOSA</t>
+          <t>JORGE ANTONIO LUNA LARA</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>2881.5</v>
+        <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>888</v>
+        <v>6113.99</v>
       </c>
       <c r="I20" t="n">
-        <v>3769.5</v>
+        <v>6113.99</v>
       </c>
       <c r="J20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K20" t="n">
-        <v>1803.3</v>
+        <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>87197.37</v>
+        <v>55025.89</v>
       </c>
       <c r="M20" t="n">
-        <v>89000.67</v>
+        <v>55025.89</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2024-12-13</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>103982</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>MARIA FERNANDA RIOS BERNAL</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1309,10 +1309,10 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>3533.64</v>
+        <v>6077.15</v>
       </c>
       <c r="I21" t="n">
-        <v>3533.64</v>
+        <v>6077.15</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -1321,21 +1321,21 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>39399.35</v>
+        <v>0</v>
       </c>
       <c r="M21" t="n">
-        <v>39399.35</v>
+        <v>0</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2023-10-17</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>120051</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1345,22 +1345,22 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>GUILLERMO JOSE RAMIREZ RAMIREZ</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>3489.2</v>
+        <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>0</v>
+        <v>4992.59</v>
       </c>
       <c r="I22" t="n">
-        <v>3489.2</v>
+        <v>4992.59</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1369,21 +1369,21 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>65824.42</v>
+        <v>8698.870000000001</v>
       </c>
       <c r="M22" t="n">
-        <v>65824.42</v>
+        <v>8698.870000000001</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2025-12-19</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>115047</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1393,7 +1393,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>VELIA PATRICIA BERNAL RAMOS</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -1405,10 +1405,10 @@
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>3206.78</v>
+        <v>4819.53</v>
       </c>
       <c r="I23" t="n">
-        <v>3206.78</v>
+        <v>4819.53</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -1417,21 +1417,21 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>10484.68</v>
+        <v>18583.84</v>
       </c>
       <c r="M23" t="n">
-        <v>10484.68</v>
+        <v>18583.84</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2025-10-14</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>118915</t>
+          <t>104718</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1441,22 +1441,22 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
+          <t>ROGELIO TORRES ORTIZ</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>3120.29</v>
+        <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>0</v>
+        <v>4624.39</v>
       </c>
       <c r="I24" t="n">
-        <v>3120.29</v>
+        <v>4624.39</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
@@ -1465,21 +1465,21 @@
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>67153.33</v>
+        <v>11744.14</v>
       </c>
       <c r="M24" t="n">
-        <v>67153.33</v>
+        <v>11744.14</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2023-12-04</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>95148</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1489,7 +1489,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1501,10 +1501,10 @@
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>3049.62</v>
+        <v>3909.17</v>
       </c>
       <c r="I25" t="n">
-        <v>3049.62</v>
+        <v>3909.17</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -1513,31 +1513,31 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>0</v>
+        <v>49593.45</v>
       </c>
       <c r="M25" t="n">
-        <v>0</v>
+        <v>49593.45</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2024-06-28</t>
+          <t>2022-12-21</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1549,10 +1549,10 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>2639.98</v>
+        <v>3533.64</v>
       </c>
       <c r="I26" t="n">
-        <v>2639.98</v>
+        <v>3533.64</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1561,46 +1561,46 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>18380.26</v>
+        <v>39399.35</v>
       </c>
       <c r="M26" t="n">
-        <v>18380.26</v>
+        <v>39399.35</v>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2018-12-05</t>
+          <t>2026-03-30</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>120051</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>GUILLERMO JOSE RAMIREZ RAMIREZ</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G27" t="n">
-        <v>0</v>
+        <v>3489.2</v>
       </c>
       <c r="H27" t="n">
-        <v>1805.6</v>
+        <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>1805.6</v>
+        <v>3489.2</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
@@ -1609,21 +1609,21 @@
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>9028</v>
+        <v>65824.42</v>
       </c>
       <c r="M27" t="n">
-        <v>9028</v>
+        <v>65824.42</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2025-03-20</t>
+          <t>2026-08-25</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>65046</t>
+          <t>118915</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1633,22 +1633,22 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G28" t="n">
-        <v>0</v>
+        <v>3120.29</v>
       </c>
       <c r="H28" t="n">
-        <v>1751.98</v>
+        <v>0</v>
       </c>
       <c r="I28" t="n">
-        <v>1751.98</v>
+        <v>3120.29</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -1657,21 +1657,21 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>1751.98</v>
+        <v>67153.33</v>
       </c>
       <c r="M28" t="n">
-        <v>1751.98</v>
+        <v>67153.33</v>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2022-07-21</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>105696</t>
+          <t>108405</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1681,7 +1681,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>GABRIELA CASTAÐEDA SALAZAR</t>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1693,10 +1693,10 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>1742.08</v>
+        <v>3049.62</v>
       </c>
       <c r="I29" t="n">
-        <v>1742.08</v>
+        <v>3049.62</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -1705,21 +1705,21 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>128661.02</v>
+        <v>0</v>
       </c>
       <c r="M29" t="n">
-        <v>128661.02</v>
+        <v>0</v>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2023-12-19</t>
+          <t>2024-06-28</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>104718</t>
+          <t>90355</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1729,7 +1729,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ROGELIO TORRES ORTIZ</t>
+          <t>DARINKA UREÐA CASILLAS</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1741,10 +1741,10 @@
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>1741.91</v>
+        <v>2369.22</v>
       </c>
       <c r="I30" t="n">
-        <v>1741.91</v>
+        <v>2369.22</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1753,21 +1753,21 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>14626.63</v>
+        <v>124257.58</v>
       </c>
       <c r="M30" t="n">
-        <v>14626.63</v>
+        <v>124257.58</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2023-12-04</t>
+          <t>2020-04-28</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1777,7 +1777,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1789,10 +1789,10 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>1707.19</v>
+        <v>1805.6</v>
       </c>
       <c r="I31" t="n">
-        <v>1707.19</v>
+        <v>1805.6</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1801,21 +1801,21 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>8535.940000000001</v>
+        <v>9028</v>
       </c>
       <c r="M31" t="n">
-        <v>8535.940000000001</v>
+        <v>9028</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2025-09-04</t>
+          <t>2025-03-20</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>65046</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1825,7 +1825,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -1837,10 +1837,10 @@
         <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>1698.53</v>
+        <v>1751.98</v>
       </c>
       <c r="I32" t="n">
-        <v>1698.53</v>
+        <v>1751.98</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1849,31 +1849,31 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>0</v>
+        <v>1751.98</v>
       </c>
       <c r="M32" t="n">
-        <v>0</v>
+        <v>1751.98</v>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2025-09-30</t>
+          <t>2022-07-21</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>118069</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>MARIO IVAN ROMERO GONZALEZ</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1885,10 +1885,10 @@
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>1666.99</v>
+        <v>1707.19</v>
       </c>
       <c r="I33" t="n">
-        <v>1666.99</v>
+        <v>1707.19</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -1897,21 +1897,21 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>37395.6</v>
+        <v>8535.940000000001</v>
       </c>
       <c r="M33" t="n">
-        <v>37395.6</v>
+        <v>8535.940000000001</v>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2025-09-04</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1921,7 +1921,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1933,10 +1933,10 @@
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>1520.61</v>
+        <v>1698.53</v>
       </c>
       <c r="I34" t="n">
-        <v>1520.61</v>
+        <v>1698.53</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
@@ -1952,24 +1952,24 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2024-08-21</t>
+          <t>2025-09-30</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>120596</t>
+          <t>118069</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>OLGA SOFIA GAXIOLA IBARRA</t>
+          <t>MARIO IVAN ROMERO GONZALEZ</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1981,33 +1981,33 @@
         <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>0</v>
+        <v>1666.99</v>
       </c>
       <c r="I35" t="n">
-        <v>0</v>
+        <v>1666.99</v>
       </c>
       <c r="J35" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K35" t="n">
-        <v>74804.00999999999</v>
+        <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>0</v>
+        <v>37395.6</v>
       </c>
       <c r="M35" t="n">
-        <v>74804.00999999999</v>
+        <v>37395.6</v>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-06-19</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>119223</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2017,7 +2017,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>OSCAR RAMIREZ RUIZ</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -2029,33 +2029,33 @@
         <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>0</v>
+        <v>1520.61</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>1520.61</v>
       </c>
       <c r="J36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K36" t="n">
-        <v>76268.8</v>
+        <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>36164.3</v>
+        <v>0</v>
       </c>
       <c r="M36" t="n">
-        <v>112433.1</v>
+        <v>0</v>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2024-08-21</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>115404</t>
+          <t>106018</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2065,7 +2065,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
+          <t>MIREYA LIZETTE TORRES GARCIA</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -2077,10 +2077,10 @@
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>0</v>
+        <v>220.85</v>
       </c>
       <c r="I37" t="n">
-        <v>0</v>
+        <v>220.85</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -2089,21 +2089,21 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>1748.27</v>
+        <v>18881.74</v>
       </c>
       <c r="M37" t="n">
-        <v>1748.27</v>
+        <v>18881.74</v>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2024-02-22</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>113450</t>
+          <t>120704</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2113,7 +2113,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
+          <t>BRUNO PADILLA SALDATE</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -2131,27 +2131,27 @@
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K38" t="n">
-        <v>0</v>
+        <v>43536.36</v>
       </c>
       <c r="L38" t="n">
-        <v>16622.23</v>
+        <v>43536.36</v>
       </c>
       <c r="M38" t="n">
-        <v>16622.23</v>
+        <v>87072.72</v>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2025-07-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>111056</t>
+          <t>120596</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2161,7 +2161,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>JORGE ANTONIO LUNA LARA</t>
+          <t>OLGA SOFIA GAXIOLA IBARRA</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -2179,27 +2179,27 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K39" t="n">
-        <v>0</v>
+        <v>74804.00999999999</v>
       </c>
       <c r="L39" t="n">
-        <v>61139.88</v>
+        <v>0</v>
       </c>
       <c r="M39" t="n">
-        <v>61139.88</v>
+        <v>74804.00999999999</v>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2024-12-13</t>
+          <t>2026-10-06</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>110575</t>
+          <t>119223</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2209,7 +2209,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>JOSE RENE DE ALBA MORALES</t>
+          <t>OSCAR RAMIREZ RUIZ</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2230,24 +2230,24 @@
         <v>1</v>
       </c>
       <c r="K40" t="n">
-        <v>166560.33</v>
+        <v>76268.8</v>
       </c>
       <c r="L40" t="n">
-        <v>0</v>
+        <v>36164.3</v>
       </c>
       <c r="M40" t="n">
-        <v>166560.33</v>
+        <v>112433.1</v>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2024-10-18</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2257,7 +2257,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2281,21 +2281,21 @@
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>1535.6</v>
+        <v>1748.27</v>
       </c>
       <c r="M41" t="n">
-        <v>1535.6</v>
+        <v>1748.27</v>
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>2024-05-28</t>
+          <t>2025-11-25</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>106018</t>
+          <t>113450</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2305,7 +2305,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>MIREYA LIZETTE TORRES GARCIA</t>
+          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2329,21 +2329,21 @@
         <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>21390.54</v>
+        <v>16622.23</v>
       </c>
       <c r="M42" t="n">
-        <v>21390.54</v>
+        <v>16622.23</v>
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>2024-02-22</t>
+          <t>2025-07-14</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>110575</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2353,7 +2353,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>JOSE RENE DE ALBA MORALES</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -2371,27 +2371,27 @@
         <v>0</v>
       </c>
       <c r="J43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K43" t="n">
-        <v>0</v>
+        <v>166560.33</v>
       </c>
       <c r="L43" t="n">
-        <v>2520.24</v>
+        <v>0</v>
       </c>
       <c r="M43" t="n">
-        <v>2520.24</v>
+        <v>166560.33</v>
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>2023-07-10</t>
+          <t>2024-10-18</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>94156</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2401,7 +2401,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>MARIA TERESA ASENCIO LOZANO</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -2425,21 +2425,21 @@
         <v>0</v>
       </c>
       <c r="L44" t="n">
-        <v>7507.58</v>
+        <v>1535.6</v>
       </c>
       <c r="M44" t="n">
-        <v>7507.58</v>
+        <v>1535.6</v>
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>2020-11-24</t>
+          <t>2024-05-28</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>90355</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2449,7 +2449,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>DARINKA UREÐA CASILLAS</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -2473,14 +2473,62 @@
         <v>0</v>
       </c>
       <c r="L45" t="n">
-        <v>126626.83</v>
+        <v>2520.24</v>
       </c>
       <c r="M45" t="n">
-        <v>126626.83</v>
+        <v>2520.24</v>
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>2020-04-28</t>
+          <t>2023-07-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>94156</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2043</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>MARIA TERESA ASENCIO LOZANO</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" t="n">
+        <v>0</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" t="n">
+        <v>0</v>
+      </c>
+      <c r="L46" t="n">
+        <v>7507.58</v>
+      </c>
+      <c r="M46" t="n">
+        <v>7507.58</v>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>2020-11-24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: Pagado y Emitido al 21-oct, Altamar en la consulta de campañas, fix fecha Convenciones Promotores, premios al 16-oct
- Pagado/Pendiente y Reclutas actualizados al corte del 21 de octubre (aviso enviado y verificado)
- descargar_campanas.js: regla Altamar (fecha desde la hoja Asesores) y Convenciones Promotores lee la fecha de B16 y no la de IGC/LIMRA (B17)
- archivar_historial_mensual.js: Altamar no se archiva por mes
- datos de premios y snapshot actualizados

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido.xlsx
@@ -413,13 +413,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N46"/>
+  <dimension ref="A1:N48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>19 de octubre de 2026</t>
+          <t>21 de octubre de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -493,10 +493,10 @@
         <v>62959.52</v>
       </c>
       <c r="H4" t="n">
-        <v>83617.09</v>
+        <v>83637.05</v>
       </c>
       <c r="I4" t="n">
-        <v>146576.61</v>
+        <v>146596.57</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -519,7 +519,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>104750</t>
+          <t>119223</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -529,7 +529,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
+          <t>OSCAR RAMIREZ RUIZ</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -538,36 +538,36 @@
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>1992.97</v>
+        <v>76268.8</v>
       </c>
       <c r="H5" t="n">
-        <v>53355.54</v>
+        <v>2407.73</v>
       </c>
       <c r="I5" t="n">
-        <v>55348.51</v>
+        <v>78676.53</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>1926.72</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>54950.44</v>
       </c>
       <c r="M5" t="n">
-        <v>0</v>
+        <v>56877.16</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2023-11-06</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>108404</t>
+          <t>104750</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
+          <t>PAULINA LIZBETH SOTO MUÐIZ</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -586,13 +586,13 @@
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>2973.12</v>
+        <v>1992.97</v>
       </c>
       <c r="H6" t="n">
-        <v>51866.38</v>
+        <v>53355.54</v>
       </c>
       <c r="I6" t="n">
-        <v>54839.5</v>
+        <v>55348.51</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -601,21 +601,21 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>31964.11</v>
+        <v>0</v>
       </c>
       <c r="M6" t="n">
-        <v>31964.11</v>
+        <v>0</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2024-06-24</t>
+          <t>2023-11-06</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>87538</t>
+          <t>108404</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
+          <t>LILIANA IVETTE CASTILLO SANCHEZ</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -634,13 +634,13 @@
         <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>31095.36</v>
+        <v>2973.12</v>
       </c>
       <c r="H7" t="n">
-        <v>20932.3</v>
+        <v>51866.38</v>
       </c>
       <c r="I7" t="n">
-        <v>52027.66</v>
+        <v>54839.5</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -649,31 +649,31 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>143228.04</v>
+        <v>31964.11</v>
       </c>
       <c r="M7" t="n">
-        <v>143228.04</v>
+        <v>31964.11</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2019-09-23</t>
+          <t>2024-06-24</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>110453</t>
+          <t>87538</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ANAIS LUA MORENO</t>
+          <t>MONICA ANDREA AMBRIZ GOMEZ</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -682,13 +682,13 @@
         <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>3113.05</v>
+        <v>31095.36</v>
       </c>
       <c r="H8" t="n">
-        <v>43114.8</v>
+        <v>20932.3</v>
       </c>
       <c r="I8" t="n">
-        <v>46227.85</v>
+        <v>52027.66</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -697,31 +697,31 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>59438.51</v>
+        <v>143228.04</v>
       </c>
       <c r="M8" t="n">
-        <v>59438.51</v>
+        <v>143228.04</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2024-11-04</t>
+          <t>2019-09-23</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>118246</t>
+          <t>110453</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>JOSE ANTEMIO OLIVA SANTOS</t>
+          <t>ANAIS LUA MORENO</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
@@ -730,13 +730,13 @@
         <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>30213.13</v>
+        <v>3113.05</v>
       </c>
       <c r="H9" t="n">
-        <v>1973.01</v>
+        <v>43114.8</v>
       </c>
       <c r="I9" t="n">
-        <v>32186.14</v>
+        <v>46227.85</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -745,46 +745,46 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>20622.49</v>
+        <v>59438.51</v>
       </c>
       <c r="M9" t="n">
-        <v>20622.49</v>
+        <v>59438.51</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2024-11-04</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>114100</t>
+          <t>118246</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
+          <t>JOSE ANTEMIO OLIVA SANTOS</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>30213.13</v>
       </c>
       <c r="H10" t="n">
-        <v>23102.75</v>
+        <v>1973.01</v>
       </c>
       <c r="I10" t="n">
-        <v>23102.75</v>
+        <v>32186.14</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -793,21 +793,21 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>2142.44</v>
+        <v>20622.49</v>
       </c>
       <c r="M10" t="n">
-        <v>2142.44</v>
+        <v>20622.49</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2025-07-25</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>47116</t>
+          <t>117440</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -817,22 +817,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
+          <t>MONSERRAT VELASCO SANTOS</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>3924.98</v>
       </c>
       <c r="H11" t="n">
-        <v>21042.72</v>
+        <v>19482.19</v>
       </c>
       <c r="I11" t="n">
-        <v>21042.72</v>
+        <v>23407.17</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -841,69 +841,69 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>22994.27</v>
+        <v>81172.53</v>
       </c>
       <c r="M11" t="n">
-        <v>22994.27</v>
+        <v>81172.53</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2022-02-24</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>117440</t>
+          <t>114100</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MONSERRAT VELASCO SANTOS</t>
+          <t>ADRIANA ALEJANDRA JOYA MARTINEZ</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>2007.19</v>
+        <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>15277.78</v>
+        <v>23102.75</v>
       </c>
       <c r="I12" t="n">
-        <v>17284.97</v>
+        <v>23102.75</v>
       </c>
       <c r="J12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>4063.85</v>
+        <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>81172.53</v>
+        <v>2142.44</v>
       </c>
       <c r="M12" t="n">
-        <v>85236.38</v>
+        <v>2142.44</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2025-07-25</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>105696</t>
+          <t>47116</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -913,7 +913,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>GABRIELA CASTAÐEDA SALAZAR</t>
+          <t>RAFAEL ALBERTO SUAREZ BAQUEDANO</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -925,10 +925,10 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>15549.5</v>
+        <v>21042.72</v>
       </c>
       <c r="I13" t="n">
-        <v>15549.5</v>
+        <v>21042.72</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -937,31 +937,31 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>115314.53</v>
+        <v>22994.27</v>
       </c>
       <c r="M13" t="n">
-        <v>115314.53</v>
+        <v>22994.27</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2023-12-19</t>
+          <t>2022-02-24</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>116883</t>
+          <t>105696</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>SOFIA CAMPILLO VASCONCELOS</t>
+          <t>GABRIELA CASTAÐEDA SALAZAR</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -973,10 +973,10 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>11461.71</v>
+        <v>18431.98</v>
       </c>
       <c r="I14" t="n">
-        <v>11461.71</v>
+        <v>18431.98</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -985,14 +985,14 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>88754.33</v>
+        <v>112432.04</v>
       </c>
       <c r="M14" t="n">
-        <v>88754.33</v>
+        <v>112432.04</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2023-12-19</t>
         </is>
       </c>
     </row>
@@ -1021,10 +1021,10 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>10358.06</v>
+        <v>12845.39</v>
       </c>
       <c r="I15" t="n">
-        <v>10358.06</v>
+        <v>12845.39</v>
       </c>
       <c r="J15" t="n">
         <v>1</v>
@@ -1033,10 +1033,10 @@
         <v>20225.92</v>
       </c>
       <c r="L15" t="n">
-        <v>2487.3</v>
+        <v>0</v>
       </c>
       <c r="M15" t="n">
-        <v>22713.22</v>
+        <v>20225.92</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
@@ -1047,17 +1047,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>100677</t>
+          <t>116883</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>JULIANA RIASCOS VALENCIA</t>
+          <t>SOFIA CAMPILLO VASCONCELOS</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -1069,10 +1069,10 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>9879.52</v>
+        <v>11461.71</v>
       </c>
       <c r="I16" t="n">
-        <v>9879.52</v>
+        <v>11461.71</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1081,21 +1081,21 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>0</v>
+        <v>88754.33</v>
       </c>
       <c r="M16" t="n">
-        <v>0</v>
+        <v>88754.33</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2023-03-14</t>
+          <t>2026-04-14</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>88234</t>
+          <t>100677</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1105,7 +1105,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
+          <t>JULIANA RIASCOS VALENCIA</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1117,10 +1117,10 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>8514.83</v>
+        <v>9879.52</v>
       </c>
       <c r="I17" t="n">
-        <v>8514.83</v>
+        <v>9879.52</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1129,117 +1129,117 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>1927.78</v>
+        <v>0</v>
       </c>
       <c r="M17" t="n">
-        <v>1927.78</v>
+        <v>0</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2019-11-25</t>
+          <t>2023-03-14</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>80925</t>
+          <t>119447</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MARICELA ARREOLA LOPEZ</t>
+          <t>LUIS ANTONIO SALAZAR ESPINOSA</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G18" t="n">
-        <v>0</v>
+        <v>2881.5</v>
       </c>
       <c r="H18" t="n">
-        <v>7624.18</v>
+        <v>5701.79</v>
       </c>
       <c r="I18" t="n">
-        <v>7624.18</v>
+        <v>8583.290000000001</v>
       </c>
       <c r="J18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>1803.3</v>
       </c>
       <c r="L18" t="n">
-        <v>18380.26</v>
+        <v>82383.58</v>
       </c>
       <c r="M18" t="n">
-        <v>18380.26</v>
+        <v>84186.88</v>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2018-12-05</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>119447</t>
+          <t>88234</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>LUIS ANTONIO SALAZAR ESPINOSA</t>
+          <t>ANDREA CELESTE IBAÐEZ RINCON</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>2881.5</v>
+        <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>3954.23</v>
+        <v>8514.83</v>
       </c>
       <c r="I19" t="n">
-        <v>6835.73</v>
+        <v>8514.83</v>
       </c>
       <c r="J19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K19" t="n">
-        <v>1803.3</v>
+        <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>84131.14</v>
+        <v>1927.78</v>
       </c>
       <c r="M19" t="n">
-        <v>85934.44</v>
+        <v>1927.78</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2019-11-25</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>111056</t>
+          <t>80925</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1249,7 +1249,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>JORGE ANTONIO LUNA LARA</t>
+          <t>MARICELA ARREOLA LOPEZ</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1261,10 +1261,10 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>6113.99</v>
+        <v>7624.18</v>
       </c>
       <c r="I20" t="n">
-        <v>6113.99</v>
+        <v>7624.18</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1273,21 +1273,21 @@
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>55025.89</v>
+        <v>18380.26</v>
       </c>
       <c r="M20" t="n">
-        <v>55025.89</v>
+        <v>18380.26</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2024-12-13</t>
+          <t>2018-12-05</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>103982</t>
+          <t>106018</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1297,7 +1297,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA RIOS BERNAL</t>
+          <t>MIREYA LIZETTE TORRES GARCIA</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1309,10 +1309,10 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>6077.15</v>
+        <v>6198.8</v>
       </c>
       <c r="I21" t="n">
-        <v>6077.15</v>
+        <v>6198.8</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -1321,31 +1321,31 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>0</v>
+        <v>16001.55</v>
       </c>
       <c r="M21" t="n">
-        <v>0</v>
+        <v>16001.55</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2023-10-17</t>
+          <t>2024-02-22</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>116060</t>
+          <t>111056</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
+          <t>JORGE ANTONIO LUNA LARA</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -1357,10 +1357,10 @@
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>4992.59</v>
+        <v>6113.99</v>
       </c>
       <c r="I22" t="n">
-        <v>4992.59</v>
+        <v>6113.99</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1369,31 +1369,31 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>8698.870000000001</v>
+        <v>55025.89</v>
       </c>
       <c r="M22" t="n">
-        <v>8698.870000000001</v>
+        <v>55025.89</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2025-12-19</t>
+          <t>2024-12-13</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>115047</t>
+          <t>103982</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>VELIA PATRICIA BERNAL RAMOS</t>
+          <t>MARIA FERNANDA RIOS BERNAL</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -1405,10 +1405,10 @@
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>4819.53</v>
+        <v>6077.15</v>
       </c>
       <c r="I23" t="n">
-        <v>4819.53</v>
+        <v>6077.15</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -1417,21 +1417,21 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>18583.84</v>
+        <v>0</v>
       </c>
       <c r="M23" t="n">
-        <v>18583.84</v>
+        <v>0</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2025-10-14</t>
+          <t>2023-10-17</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>104718</t>
+          <t>107488</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ROGELIO TORRES ORTIZ</t>
+          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>4624.39</v>
+        <v>5018.74</v>
       </c>
       <c r="I24" t="n">
-        <v>4624.39</v>
+        <v>5018.74</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
@@ -1465,31 +1465,31 @@
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>11744.14</v>
+        <v>0</v>
       </c>
       <c r="M24" t="n">
-        <v>11744.14</v>
+        <v>0</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2023-12-04</t>
+          <t>2024-05-28</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>95148</t>
+          <t>116060</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
+          <t>LUVIA PATRICIA FIGUEROA CASTRO</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -1501,10 +1501,10 @@
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>3909.17</v>
+        <v>4992.59</v>
       </c>
       <c r="I25" t="n">
-        <v>3909.17</v>
+        <v>4992.59</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -1513,21 +1513,21 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>49593.45</v>
+        <v>8698.870000000001</v>
       </c>
       <c r="M25" t="n">
-        <v>49593.45</v>
+        <v>8698.870000000001</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2022-12-21</t>
+          <t>2025-12-19</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>116876</t>
+          <t>115047</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1537,7 +1537,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>PAULA ANGELICA LOMELI CAZARES</t>
+          <t>VELIA PATRICIA BERNAL RAMOS</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1549,10 +1549,10 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>3533.64</v>
+        <v>4819.53</v>
       </c>
       <c r="I26" t="n">
-        <v>3533.64</v>
+        <v>4819.53</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1561,46 +1561,46 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>39399.35</v>
+        <v>18583.84</v>
       </c>
       <c r="M26" t="n">
-        <v>39399.35</v>
+        <v>18583.84</v>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2025-10-14</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>120051</t>
+          <t>104718</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>GUILLERMO JOSE RAMIREZ RAMIREZ</t>
+          <t>ROGELIO TORRES ORTIZ</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>3489.2</v>
+        <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>0</v>
+        <v>4624.39</v>
       </c>
       <c r="I27" t="n">
-        <v>3489.2</v>
+        <v>4624.39</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
@@ -1609,21 +1609,21 @@
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>65824.42</v>
+        <v>11744.14</v>
       </c>
       <c r="M27" t="n">
-        <v>65824.42</v>
+        <v>11744.14</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2023-12-04</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>118915</t>
+          <t>95148</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1633,22 +1633,22 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
+          <t>ENRIQUE ADRIAN GUTIERREZ JIMENEZ</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>3120.29</v>
+        <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>0</v>
+        <v>3909.17</v>
       </c>
       <c r="I28" t="n">
-        <v>3120.29</v>
+        <v>3909.17</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -1657,31 +1657,31 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>67153.33</v>
+        <v>49593.45</v>
       </c>
       <c r="M28" t="n">
-        <v>67153.33</v>
+        <v>49593.45</v>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2022-12-21</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>108405</t>
+          <t>116876</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
+          <t>PAULA ANGELICA LOMELI CAZARES</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1693,10 +1693,10 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>3049.62</v>
+        <v>3533.64</v>
       </c>
       <c r="I29" t="n">
-        <v>3049.62</v>
+        <v>3533.64</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -1705,46 +1705,46 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>0</v>
+        <v>39399.35</v>
       </c>
       <c r="M29" t="n">
-        <v>0</v>
+        <v>39399.35</v>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2024-06-28</t>
+          <t>2026-03-30</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>90355</t>
+          <t>120051</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>DARINKA UREÐA CASILLAS</t>
+          <t>GUILLERMO JOSE RAMIREZ RAMIREZ</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G30" t="n">
-        <v>0</v>
+        <v>3489.2</v>
       </c>
       <c r="H30" t="n">
-        <v>2369.22</v>
+        <v>0</v>
       </c>
       <c r="I30" t="n">
-        <v>2369.22</v>
+        <v>3489.2</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1753,21 +1753,21 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>124257.58</v>
+        <v>65824.42</v>
       </c>
       <c r="M30" t="n">
-        <v>124257.58</v>
+        <v>65824.42</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2020-04-28</t>
+          <t>2026-08-25</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>112083</t>
+          <t>114157</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1777,7 +1777,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
+          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1789,10 +1789,10 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>1805.6</v>
+        <v>3414.38</v>
       </c>
       <c r="I31" t="n">
-        <v>1805.6</v>
+        <v>3414.38</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1801,21 +1801,21 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>9028</v>
+        <v>6828.75</v>
       </c>
       <c r="M31" t="n">
-        <v>9028</v>
+        <v>6828.75</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2025-03-20</t>
+          <t>2025-09-04</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>65046</t>
+          <t>118915</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1825,22 +1825,22 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>PAULINA RODRIGUEZ DE LA MORA</t>
+          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G32" t="n">
-        <v>0</v>
+        <v>3120.29</v>
       </c>
       <c r="H32" t="n">
-        <v>1751.98</v>
+        <v>0</v>
       </c>
       <c r="I32" t="n">
-        <v>1751.98</v>
+        <v>3120.29</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1849,21 +1849,21 @@
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>1751.98</v>
+        <v>67153.33</v>
       </c>
       <c r="M32" t="n">
-        <v>1751.98</v>
+        <v>67153.33</v>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2022-07-21</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>114157</t>
+          <t>108405</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1873,7 +1873,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>HANA SOFIA LOPEZ QUIÐONEZ</t>
+          <t>MARIA ELIZABETH LLAMAS LOPEZ</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1885,10 +1885,10 @@
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>1707.19</v>
+        <v>3049.62</v>
       </c>
       <c r="I33" t="n">
-        <v>1707.19</v>
+        <v>3049.62</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -1897,21 +1897,21 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>8535.940000000001</v>
+        <v>0</v>
       </c>
       <c r="M33" t="n">
-        <v>8535.940000000001</v>
+        <v>0</v>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2025-09-04</t>
+          <t>2024-06-28</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>114431</t>
+          <t>102825</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1921,7 +1921,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>MARIA JOSE GUZMAN ZAMORA</t>
+          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1933,10 +1933,10 @@
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>1698.53</v>
+        <v>2520.28</v>
       </c>
       <c r="I34" t="n">
-        <v>1698.53</v>
+        <v>2520.28</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
@@ -1952,62 +1952,62 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2025-09-30</t>
+          <t>2023-07-10</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>118069</t>
+          <t>120596</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2856</t>
+          <t>2043</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>MARIO IVAN ROMERO GONZALEZ</t>
+          <t>OLGA SOFIA GAXIOLA IBARRA</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G35" t="n">
-        <v>0</v>
+        <v>2423.81</v>
       </c>
       <c r="H35" t="n">
-        <v>1666.99</v>
+        <v>0</v>
       </c>
       <c r="I35" t="n">
-        <v>1666.99</v>
+        <v>2423.81</v>
       </c>
       <c r="J35" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K35" t="n">
-        <v>0</v>
+        <v>120890.51</v>
       </c>
       <c r="L35" t="n">
-        <v>37395.6</v>
+        <v>26661.91</v>
       </c>
       <c r="M35" t="n">
-        <v>37395.6</v>
+        <v>147552.42</v>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-10-06</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>109007</t>
+          <t>90355</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2017,7 +2017,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
+          <t>DARINKA UREÐA CASILLAS</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -2029,10 +2029,10 @@
         <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>1520.61</v>
+        <v>2369.22</v>
       </c>
       <c r="I36" t="n">
-        <v>1520.61</v>
+        <v>2369.22</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
@@ -2041,21 +2041,21 @@
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>0</v>
+        <v>124257.58</v>
       </c>
       <c r="M36" t="n">
-        <v>0</v>
+        <v>124257.58</v>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2024-08-21</t>
+          <t>2020-04-28</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>106018</t>
+          <t>94156</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2065,7 +2065,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>MIREYA LIZETTE TORRES GARCIA</t>
+          <t>MARIA TERESA ASENCIO LOZANO</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -2077,10 +2077,10 @@
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>220.85</v>
+        <v>2315.59</v>
       </c>
       <c r="I37" t="n">
-        <v>220.85</v>
+        <v>2315.59</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -2089,21 +2089,21 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>18881.74</v>
+        <v>5192.03</v>
       </c>
       <c r="M37" t="n">
-        <v>18881.74</v>
+        <v>5192.03</v>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2024-02-22</t>
+          <t>2020-11-24</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>120704</t>
+          <t>113450</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2113,7 +2113,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>BRUNO PADILLA SALDATE</t>
+          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -2125,33 +2125,33 @@
         <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>0</v>
+        <v>2077.78</v>
       </c>
       <c r="I38" t="n">
-        <v>0</v>
+        <v>2077.78</v>
       </c>
       <c r="J38" t="n">
         <v>1</v>
       </c>
       <c r="K38" t="n">
-        <v>43536.36</v>
+        <v>1902.95</v>
       </c>
       <c r="L38" t="n">
-        <v>43536.36</v>
+        <v>35476.92</v>
       </c>
       <c r="M38" t="n">
-        <v>87072.72</v>
+        <v>37379.87</v>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2025-07-14</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>120596</t>
+          <t>112083</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2161,7 +2161,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>OLGA SOFIA GAXIOLA IBARRA</t>
+          <t>LUIS GUILLERMO OLGUIN FERNANDEZ</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -2173,33 +2173,33 @@
         <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>0</v>
+        <v>1805.6</v>
       </c>
       <c r="I39" t="n">
-        <v>0</v>
+        <v>1805.6</v>
       </c>
       <c r="J39" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K39" t="n">
-        <v>74804.00999999999</v>
+        <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>0</v>
+        <v>9028</v>
       </c>
       <c r="M39" t="n">
-        <v>74804.00999999999</v>
+        <v>9028</v>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2025-03-20</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>119223</t>
+          <t>65046</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2209,7 +2209,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>OSCAR RAMIREZ RUIZ</t>
+          <t>PAULINA RODRIGUEZ DE LA MORA</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2221,33 +2221,33 @@
         <v>0</v>
       </c>
       <c r="H40" t="n">
-        <v>0</v>
+        <v>1751.98</v>
       </c>
       <c r="I40" t="n">
-        <v>0</v>
+        <v>1751.98</v>
       </c>
       <c r="J40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K40" t="n">
-        <v>76268.8</v>
+        <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>36164.3</v>
+        <v>1751.98</v>
       </c>
       <c r="M40" t="n">
-        <v>112433.1</v>
+        <v>1751.98</v>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2022-07-21</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>115404</t>
+          <t>114431</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2257,7 +2257,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ANA VERONICA GONZALEZ GAYTAN</t>
+          <t>MARIA JOSE GUZMAN ZAMORA</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2269,10 +2269,10 @@
         <v>0</v>
       </c>
       <c r="H41" t="n">
-        <v>0</v>
+        <v>1698.53</v>
       </c>
       <c r="I41" t="n">
-        <v>0</v>
+        <v>1698.53</v>
       </c>
       <c r="J41" t="n">
         <v>0</v>
@@ -2281,31 +2281,31 @@
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>1748.27</v>
+        <v>0</v>
       </c>
       <c r="M41" t="n">
-        <v>1748.27</v>
+        <v>0</v>
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-09-30</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>113450</t>
+          <t>118069</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2043</t>
+          <t>2856</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ANA LAURA CONTRERAS IÐIGUEZ</t>
+          <t>MARIO IVAN ROMERO GONZALEZ</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2317,10 +2317,10 @@
         <v>0</v>
       </c>
       <c r="H42" t="n">
-        <v>0</v>
+        <v>1666.99</v>
       </c>
       <c r="I42" t="n">
-        <v>0</v>
+        <v>1666.99</v>
       </c>
       <c r="J42" t="n">
         <v>0</v>
@@ -2329,21 +2329,21 @@
         <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>16622.23</v>
+        <v>37395.6</v>
       </c>
       <c r="M42" t="n">
-        <v>16622.23</v>
+        <v>37395.6</v>
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>2025-07-14</t>
+          <t>2026-06-19</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>110575</t>
+          <t>116795</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2353,7 +2353,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>JOSE RENE DE ALBA MORALES</t>
+          <t>GERARDO DANIEL BARAJAS TORRES</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -2365,33 +2365,33 @@
         <v>0</v>
       </c>
       <c r="H43" t="n">
-        <v>0</v>
+        <v>1603.03</v>
       </c>
       <c r="I43" t="n">
-        <v>0</v>
+        <v>1603.03</v>
       </c>
       <c r="J43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K43" t="n">
-        <v>166560.33</v>
+        <v>0</v>
       </c>
       <c r="L43" t="n">
         <v>0</v>
       </c>
       <c r="M43" t="n">
-        <v>166560.33</v>
+        <v>0</v>
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>2024-10-18</t>
+          <t>2025-12-09</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>107488</t>
+          <t>109007</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2401,7 +2401,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>ORLANDA JIMENA CERVANTES NUÐEZ</t>
+          <t>ISAI ANTONIO ROJAS MARTINEZ</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -2413,10 +2413,10 @@
         <v>0</v>
       </c>
       <c r="H44" t="n">
-        <v>0</v>
+        <v>1520.61</v>
       </c>
       <c r="I44" t="n">
-        <v>0</v>
+        <v>1520.61</v>
       </c>
       <c r="J44" t="n">
         <v>0</v>
@@ -2425,21 +2425,21 @@
         <v>0</v>
       </c>
       <c r="L44" t="n">
-        <v>1535.6</v>
+        <v>0</v>
       </c>
       <c r="M44" t="n">
-        <v>1535.6</v>
+        <v>0</v>
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>2024-05-28</t>
+          <t>2024-08-21</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>102825</t>
+          <t>120704</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2449,7 +2449,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>JOSE EDUARDO EZQUERRO BARQUERA</t>
+          <t>BRUNO PADILLA SALDATE</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -2467,27 +2467,27 @@
         <v>0</v>
       </c>
       <c r="J45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K45" t="n">
-        <v>0</v>
+        <v>43536.36</v>
       </c>
       <c r="L45" t="n">
-        <v>2520.24</v>
+        <v>43536.36</v>
       </c>
       <c r="M45" t="n">
-        <v>2520.24</v>
+        <v>87072.72</v>
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>2023-07-10</t>
+          <t>2026-10-13</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>94156</t>
+          <t>115404</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2497,7 +2497,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>MARIA TERESA ASENCIO LOZANO</t>
+          <t>ANA VERONICA GONZALEZ GAYTAN</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -2521,14 +2521,110 @@
         <v>0</v>
       </c>
       <c r="L46" t="n">
-        <v>7507.58</v>
+        <v>1748.27</v>
       </c>
       <c r="M46" t="n">
-        <v>7507.58</v>
+        <v>1748.27</v>
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>2020-11-24</t>
+          <t>2025-11-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>110575</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2043</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>JOSE RENE DE ALBA MORALES</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" t="n">
+        <v>0</v>
+      </c>
+      <c r="J47" t="n">
+        <v>1</v>
+      </c>
+      <c r="K47" t="n">
+        <v>166560.33</v>
+      </c>
+      <c r="L47" t="n">
+        <v>0</v>
+      </c>
+      <c r="M47" t="n">
+        <v>166560.33</v>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>2024-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>21615</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2043</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>SELINA JANET LEMUS MIRAMONTES</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" t="n">
+        <v>0</v>
+      </c>
+      <c r="J48" t="n">
+        <v>1</v>
+      </c>
+      <c r="K48" t="n">
+        <v>30137.95</v>
+      </c>
+      <c r="L48" t="n">
+        <v>0</v>
+      </c>
+      <c r="M48" t="n">
+        <v>30137.95</v>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>2021-07-30</t>
         </is>
       </c>
     </row>

</xml_diff>